<commit_message>
Fix IDF formulas in K26:K28 missing leading equals
Those cells were stored as text (IF...) instead of formulas (=IF...),
which made LibreOffice show formula fragments and broke L26:L28.

Co-authored-by: acon560-prog <acon560-prog@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/engineering/drainage-design/Dimensionnement_reseau_pluvial_ADAPTE_methode_simple OLIVIER TECH. MODIF.xlsx
+++ b/engineering/drainage-design/Dimensionnement_reseau_pluvial_ADAPTE_methode_simple OLIVIER TECH. MODIF.xlsx
@@ -3853,10 +3853,9 @@
         <f>IF(H26=0,0,I26/H26)</f>
         <v/>
       </c>
-      <c r="K26" s="249" t="inlineStr">
-        <is>
-          <t>IF($S$2=0.5,$R$5/((D26+$S$5)^$T$5),IF($S$2=0.2,$R$6/((D26+$S$6)^$T$6),IF($S$2=0.1,$R$7/((D26+$S$7)^$T$7),IF($S$2=0.04,$R$8/((D26+$S$8)^$T$8),IF($S$2=0.02,$R$9/((D26+$S$9)^$T$9),$R$10/((D26+$S$10)^$T$10))))))</t>
-        </is>
+      <c r="K26" s="249">
+        <f>IF($S$2=0.5,$R$5/((D26+$S$5)^$T$5),IF($S$2=0.2,$R$6/((D26+$S$6)^$T$6),IF($S$2=0.1,$R$7/((D26+$S$7)^$T$7),IF($S$2=0.04,$R$8/((D26+$S$8)^$T$8),IF($S$2=0.02,$R$9/((D26+$S$9)^$T$9),$R$10/((D26+$S$10)^$T$10))))))</f>
+        <v/>
       </c>
       <c r="L26" s="253">
         <f>0.00275*H26*J26*K26</f>
@@ -3868,24 +3867,24 @@
       <c r="N26" s="113" t="n">
         <v>300</v>
       </c>
-      <c r="O26" s="108">
+      <c r="O26" s="249">
         <f>IF(OR(N26&lt;=0,M26&lt;=0),0,((N26/4000)^(2/3)*SQRT(M26))/$S$11)</f>
         <v/>
       </c>
       <c r="P26" s="248" t="n">
         <v>14.3</v>
       </c>
-      <c r="Q26" s="108">
+      <c r="Q26" s="249">
         <f>IF(O26=0,0,P26/(O26*60))</f>
         <v/>
       </c>
-      <c r="R26" s="112">
+      <c r="R26" s="253">
         <f>O26*(PI()*(N26/1000)^2/4)</f>
         <v/>
       </c>
       <c r="S26" s="114" t="n"/>
       <c r="T26" s="114" t="n"/>
-      <c r="U26" s="231">
+      <c r="U26" s="253">
         <f>V26+(M26*P26)</f>
         <v/>
       </c>
@@ -3895,13 +3894,13 @@
       </c>
       <c r="W26" s="112" t="n"/>
       <c r="X26" s="112" t="n"/>
-      <c r="Y26" s="112">
+      <c r="Y26" s="253">
         <f>P26*PI()*(N26/1000)^2/4</f>
         <v/>
       </c>
       <c r="Z26" s="95" t="n"/>
       <c r="AA26" s="115" t="n"/>
-      <c r="AB26" s="116">
+      <c r="AB26" s="256">
         <f>IF(R26&gt;L26,"OK","AUGMENTER D")</f>
         <v/>
       </c>
@@ -3953,10 +3952,9 @@
         <f>IF(H27=0,0,I27/H27)</f>
         <v/>
       </c>
-      <c r="K27" s="249" t="inlineStr">
-        <is>
-          <t>IF($S$2=0.5,$R$5/((D27+$S$5)^$T$5),IF($S$2=0.2,$R$6/((D27+$S$6)^$T$6),IF($S$2=0.1,$R$7/((D27+$S$7)^$T$7),IF($S$2=0.04,$R$8/((D27+$S$8)^$T$8),IF($S$2=0.02,$R$9/((D27+$S$9)^$T$9),$R$10/((D27+$S$10)^$T$10))))))</t>
-        </is>
+      <c r="K27" s="249">
+        <f>IF($S$2=0.5,$R$5/((D27+$S$5)^$T$5),IF($S$2=0.2,$R$6/((D27+$S$6)^$T$6),IF($S$2=0.1,$R$7/((D27+$S$7)^$T$7),IF($S$2=0.04,$R$8/((D27+$S$8)^$T$8),IF($S$2=0.02,$R$9/((D27+$S$9)^$T$9),$R$10/((D27+$S$10)^$T$10))))))</f>
+        <v/>
       </c>
       <c r="L27" s="253">
         <f>0.00275*H27*J27*K27</f>
@@ -4053,10 +4051,9 @@
         <f>IF(H28=0,0,I28/H28)</f>
         <v/>
       </c>
-      <c r="K28" s="249" t="inlineStr">
-        <is>
-          <t>IF($S$2=0.5,$R$5/((D28+$S$5)^$T$5),IF($S$2=0.2,$R$6/((D28+$S$6)^$T$6),IF($S$2=0.1,$R$7/((D28+$S$7)^$T$7),IF($S$2=0.04,$R$8/((D28+$S$8)^$T$8),IF($S$2=0.02,$R$9/((D28+$S$9)^$T$9),$R$10/((D28+$S$10)^$T$10))))))</t>
-        </is>
+      <c r="K28" s="249">
+        <f>IF($S$2=0.5,$R$5/((D28+$S$5)^$T$5),IF($S$2=0.2,$R$6/((D28+$S$6)^$T$6),IF($S$2=0.1,$R$7/((D28+$S$7)^$T$7),IF($S$2=0.04,$R$8/((D28+$S$8)^$T$8),IF($S$2=0.02,$R$9/((D28+$S$9)^$T$9),$R$10/((D28+$S$10)^$T$10))))))</f>
+        <v/>
       </c>
       <c r="L28" s="253">
         <f>0.00275*H28*J28*K28</f>

</xml_diff>

<commit_message>
Add network invert elevations with MIN rule at junctions
Compute radiers from PUB=15.305 upstream using max(s,1%) and 0.02 m
drops; at confluences keep the lowest invert. Add roof node T1→P11
(zone N) and document results on a Radiers sheet.

Co-authored-by: acon560-prog <acon560-prog@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/engineering/drainage-design/Dimensionnement_reseau_pluvial_ADAPTE_methode_simple OLIVIER TECH. MODIF.xlsx
+++ b/engineering/drainage-design/Dimensionnement_reseau_pluvial_ADAPTE_methode_simple OLIVIER TECH. MODIF.xlsx
@@ -7,12 +7,13 @@
   </bookViews>
   <sheets>
     <sheet name="Guide_adaptation" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Calcul_reseau" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Temps de concentration" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Radiers" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Calcul_reseau" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Temps de concentration" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Titles" localSheetId="1">'Calcul_reseau'!$1:$15</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'Calcul_reseau'!$A$1:$AA$35</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="2">'Calcul_reseau'!$1:$15</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="2">'Calcul_reseau'!$A$1:$AA$35</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
@@ -28,7 +29,7 @@
     <numFmt numFmtId="168" formatCode="0.0000"/>
     <numFmt numFmtId="169" formatCode="0.00000"/>
   </numFmts>
-  <fonts count="19">
+  <fonts count="24">
     <font>
       <name val="Times New Roman"/>
       <charset val="1"/>
@@ -155,8 +156,35 @@
       <b val="1"/>
       <sz val="12"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001F4E79"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="00C00000"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="16">
+  <fills count="19">
     <fill>
       <patternFill/>
     </fill>
@@ -245,8 +273,23 @@
         <fgColor rgb="00FFFF99"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F4E79"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCE4D6"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="65">
+  <borders count="66">
     <border>
       <left/>
       <right/>
@@ -1048,12 +1091,26 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00B0B0B0"/>
+      </left>
+      <right style="thin">
+        <color rgb="00B0B0B0"/>
+      </right>
+      <top style="thin">
+        <color rgb="00B0B0B0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00B0B0B0"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="272">
+  <cellXfs count="298">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
@@ -1752,6 +1809,58 @@
     </xf>
     <xf numFmtId="165" fontId="2" fillId="0" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="65" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="21" fillId="17" borderId="65" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="65" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="0" fillId="14" borderId="65" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="65" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="0" fillId="16" borderId="65" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="65" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="0" fillId="14" borderId="65" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="5" fillId="16" borderId="47" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="5" fillId="16" borderId="47" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="16" borderId="47" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="16" borderId="47" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="5" fillId="16" borderId="47" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="2" fillId="16" borderId="41" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="14" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="16" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="16" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="16" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="2" fillId="16" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="65" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="0" fillId="18" borderId="65" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="48" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -2020,7 +2129,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A23"/>
+  <dimension ref="A1:A28"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.5" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="110" customWidth="1" style="227" min="1" max="1"/>
@@ -2163,6 +2272,34 @@
       <c r="A23" s="4" t="inlineStr">
         <is>
           <t>H/I: à J01, P02→J01 ne cumule pas le réseau amont; J01→RP03 = H(P01→J01)+H(P02→J01)+DA.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>MAJ radiers + T1:</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>- Onglet Radiers: inverts depuis PUB=15.305, chute 0.02, pente min 1%, MIN aux confluences P06/J01/P11</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>- Nouveau T1 (toit zone N) → P11; DA 903 m² retirée de P10→P11</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>- Calcul_reseau U/V = radiers calculés (vert)</t>
         </is>
       </c>
     </row>
@@ -2176,9 +2313,1012 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J42"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" style="227" min="1" max="1"/>
+    <col width="10" customWidth="1" style="227" min="2" max="2"/>
+    <col width="10" customWidth="1" style="227" min="3" max="3"/>
+    <col width="10" customWidth="1" style="227" min="4" max="4"/>
+    <col width="12" customWidth="1" style="227" min="5" max="5"/>
+    <col width="16" customWidth="1" style="227" min="6" max="6"/>
+    <col width="14" customWidth="1" style="227" min="7" max="7"/>
+    <col width="12" customWidth="1" style="227" min="8" max="8"/>
+    <col width="12" customWidth="1" style="227" min="9" max="9"/>
+    <col width="16" customWidth="1" style="227" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="272" t="inlineStr">
+        <is>
+          <t>RADIERS (invert elevations) — règle MIN aux confluences</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Exutoire PUB fixe = 15.305 m. Remontée: Inv_amont = Inv_aval + max(s,1%)*L + chute 0.02 m.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Si plusieurs branches proposent un radier au même noeud → on garde le PLUS BAS.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="294" t="inlineStr">
+        <is>
+          <t>Règle confluences (P06, J01, P11): toutes les branches amont se calent sur le radier du noeud fixé depuis l’aval; si plusieurs contraintes, retenir le PLUS BAS.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="273" t="inlineStr">
+        <is>
+          <t>Paramètres</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Invert PUB (m)</t>
+        </is>
+      </c>
+      <c r="B6" s="274" t="n">
+        <v>15.305</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Chute regard (m)</t>
+        </is>
+      </c>
+      <c r="B7" s="274" t="n">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Pente min radier</t>
+        </is>
+      </c>
+      <c r="B8" s="274" t="n">
+        <v>0.01</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="275" t="inlineStr">
+        <is>
+          <t>Noeud</t>
+        </is>
+      </c>
+      <c r="B10" s="275" t="inlineStr">
+        <is>
+          <t>Invert (m)</t>
+        </is>
+      </c>
+      <c r="C10" s="275" t="inlineStr">
+        <is>
+          <t>Sol (m)</t>
+        </is>
+      </c>
+      <c r="D10" s="275" t="inlineStr">
+        <is>
+          <t>Couverture approx (m)</t>
+        </is>
+      </c>
+      <c r="E10" s="275" t="inlineStr">
+        <is>
+          <t>Nb propositions</t>
+        </is>
+      </c>
+      <c r="F10" s="275" t="inlineStr">
+        <is>
+          <t>Propositions (m)</t>
+        </is>
+      </c>
+      <c r="G10" s="275" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="276" t="inlineStr">
+        <is>
+          <t>P09</t>
+        </is>
+      </c>
+      <c r="B11" s="277" t="n">
+        <v>16.976</v>
+      </c>
+      <c r="C11" s="278" t="n">
+        <v>17.62</v>
+      </c>
+      <c r="D11" s="277" t="n">
+        <v>0.644</v>
+      </c>
+      <c r="E11" s="276" t="n">
+        <v>1</v>
+      </c>
+      <c r="F11" s="276" t="inlineStr">
+        <is>
+          <t>16.976</t>
+        </is>
+      </c>
+      <c r="G11" s="276" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="276" t="inlineStr">
+        <is>
+          <t>P07</t>
+        </is>
+      </c>
+      <c r="B12" s="277" t="n">
+        <v>16.567</v>
+      </c>
+      <c r="C12" s="278" t="n">
+        <v>17.09</v>
+      </c>
+      <c r="D12" s="277" t="n">
+        <v>0.523</v>
+      </c>
+      <c r="E12" s="276" t="n">
+        <v>1</v>
+      </c>
+      <c r="F12" s="276" t="inlineStr">
+        <is>
+          <t>16.567</t>
+        </is>
+      </c>
+      <c r="G12" s="276" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="295" t="inlineStr">
+        <is>
+          <t>P06</t>
+        </is>
+      </c>
+      <c r="B13" s="296" t="n">
+        <v>16.422</v>
+      </c>
+      <c r="C13" s="296" t="n">
+        <v>17.14</v>
+      </c>
+      <c r="D13" s="296" t="n">
+        <v>0.718</v>
+      </c>
+      <c r="E13" s="295" t="n">
+        <v>1</v>
+      </c>
+      <c r="F13" s="295" t="inlineStr">
+        <is>
+          <t>16.422</t>
+        </is>
+      </c>
+      <c r="G13" s="295" t="inlineStr">
+        <is>
+          <t>CONFLUENCE — radier unique (plus bas / calé aval); branches amont: P06</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="276" t="inlineStr">
+        <is>
+          <t>P04</t>
+        </is>
+      </c>
+      <c r="B14" s="277" t="n">
+        <v>16.306</v>
+      </c>
+      <c r="C14" s="278" t="n">
+        <v>17.28</v>
+      </c>
+      <c r="D14" s="277" t="n">
+        <v>0.974</v>
+      </c>
+      <c r="E14" s="276" t="n">
+        <v>1</v>
+      </c>
+      <c r="F14" s="276" t="inlineStr">
+        <is>
+          <t>16.306</t>
+        </is>
+      </c>
+      <c r="G14" s="276" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="276" t="inlineStr">
+        <is>
+          <t>P01</t>
+        </is>
+      </c>
+      <c r="B15" s="277" t="n">
+        <v>16.153</v>
+      </c>
+      <c r="C15" s="278" t="n">
+        <v>17.23</v>
+      </c>
+      <c r="D15" s="277" t="n">
+        <v>1.077</v>
+      </c>
+      <c r="E15" s="276" t="n">
+        <v>1</v>
+      </c>
+      <c r="F15" s="276" t="inlineStr">
+        <is>
+          <t>16.153</t>
+        </is>
+      </c>
+      <c r="G15" s="276" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="276" t="inlineStr">
+        <is>
+          <t>P02</t>
+        </is>
+      </c>
+      <c r="B16" s="277" t="n">
+        <v>16.025</v>
+      </c>
+      <c r="C16" s="278" t="n">
+        <v>17.131</v>
+      </c>
+      <c r="D16" s="277" t="n">
+        <v>1.106</v>
+      </c>
+      <c r="E16" s="276" t="n">
+        <v>1</v>
+      </c>
+      <c r="F16" s="276" t="inlineStr">
+        <is>
+          <t>16.025</t>
+        </is>
+      </c>
+      <c r="G16" s="276" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="295" t="inlineStr">
+        <is>
+          <t>J01</t>
+        </is>
+      </c>
+      <c r="B17" s="296" t="n">
+        <v>15.989</v>
+      </c>
+      <c r="C17" s="296" t="n">
+        <v>17.12</v>
+      </c>
+      <c r="D17" s="296" t="n">
+        <v>1.131</v>
+      </c>
+      <c r="E17" s="295" t="n">
+        <v>1</v>
+      </c>
+      <c r="F17" s="295" t="inlineStr">
+        <is>
+          <t>15.989</t>
+        </is>
+      </c>
+      <c r="G17" s="295" t="inlineStr">
+        <is>
+          <t>CONFLUENCE — radier unique (plus bas / calé aval); branches amont: J01</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="276" t="inlineStr">
+        <is>
+          <t>RP03</t>
+        </is>
+      </c>
+      <c r="B18" s="277" t="n">
+        <v>15.857</v>
+      </c>
+      <c r="C18" s="278" t="n">
+        <v>17.01</v>
+      </c>
+      <c r="D18" s="277" t="n">
+        <v>1.153</v>
+      </c>
+      <c r="E18" s="276" t="n">
+        <v>1</v>
+      </c>
+      <c r="F18" s="276" t="inlineStr">
+        <is>
+          <t>15.857</t>
+        </is>
+      </c>
+      <c r="G18" s="276" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="276" t="inlineStr">
+        <is>
+          <t>P10</t>
+        </is>
+      </c>
+      <c r="B19" s="277" t="n">
+        <v>15.766</v>
+      </c>
+      <c r="C19" s="278" t="n">
+        <v>16.965</v>
+      </c>
+      <c r="D19" s="277" t="n">
+        <v>1.199</v>
+      </c>
+      <c r="E19" s="276" t="n">
+        <v>1</v>
+      </c>
+      <c r="F19" s="276" t="inlineStr">
+        <is>
+          <t>15.766</t>
+        </is>
+      </c>
+      <c r="G19" s="276" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="276" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="B20" s="277" t="n">
+        <v>15.743</v>
+      </c>
+      <c r="C20" s="278" t="n">
+        <v>17.01</v>
+      </c>
+      <c r="D20" s="277" t="n">
+        <v>1.267</v>
+      </c>
+      <c r="E20" s="276" t="n">
+        <v>1</v>
+      </c>
+      <c r="F20" s="276" t="inlineStr">
+        <is>
+          <t>15.743</t>
+        </is>
+      </c>
+      <c r="G20" s="276" t="inlineStr">
+        <is>
+          <t>Toiture (zone N)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="295" t="inlineStr">
+        <is>
+          <t>P11</t>
+        </is>
+      </c>
+      <c r="B21" s="296" t="n">
+        <v>15.603</v>
+      </c>
+      <c r="C21" s="296" t="n">
+        <v>16.874</v>
+      </c>
+      <c r="D21" s="296" t="n">
+        <v>1.271</v>
+      </c>
+      <c r="E21" s="295" t="n">
+        <v>1</v>
+      </c>
+      <c r="F21" s="295" t="inlineStr">
+        <is>
+          <t>15.603</t>
+        </is>
+      </c>
+      <c r="G21" s="295" t="inlineStr">
+        <is>
+          <t>CONFLUENCE — radier unique (plus bas / calé aval); branches amont: P11</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="276" t="inlineStr">
+        <is>
+          <t>P12</t>
+        </is>
+      </c>
+      <c r="B22" s="277" t="n">
+        <v>15.449</v>
+      </c>
+      <c r="C22" s="278" t="n">
+        <v>16.73</v>
+      </c>
+      <c r="D22" s="277" t="n">
+        <v>1.281</v>
+      </c>
+      <c r="E22" s="276" t="n">
+        <v>1</v>
+      </c>
+      <c r="F22" s="276" t="inlineStr">
+        <is>
+          <t>15.449</t>
+        </is>
+      </c>
+      <c r="G22" s="276" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="276" t="inlineStr">
+        <is>
+          <t>PUB</t>
+        </is>
+      </c>
+      <c r="B23" s="277" t="n">
+        <v>15.305</v>
+      </c>
+      <c r="C23" s="278" t="n">
+        <v>16.73</v>
+      </c>
+      <c r="D23" s="277" t="n">
+        <v>1.425</v>
+      </c>
+      <c r="E23" s="276" t="n">
+        <v>1</v>
+      </c>
+      <c r="F23" s="276" t="inlineStr">
+        <is>
+          <t>15.305</t>
+        </is>
+      </c>
+      <c r="G23" s="276" t="inlineStr">
+        <is>
+          <t>Exutoire fixe</t>
+        </is>
+      </c>
+    </row>
+    <row r="24"/>
+    <row r="25">
+      <c r="A25" s="273" t="inlineStr">
+        <is>
+          <t>Profil par conduite (U amont / V aval)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="275" t="inlineStr">
+        <is>
+          <t>Pipe_ID</t>
+        </is>
+      </c>
+      <c r="B26" s="275" t="inlineStr">
+        <is>
+          <t>De</t>
+        </is>
+      </c>
+      <c r="C26" s="275" t="inlineStr">
+        <is>
+          <t>Vers</t>
+        </is>
+      </c>
+      <c r="D26" s="275" t="inlineStr">
+        <is>
+          <t>L (m)</t>
+        </is>
+      </c>
+      <c r="E26" s="275" t="inlineStr">
+        <is>
+          <t>s design</t>
+        </is>
+      </c>
+      <c r="F26" s="275" t="inlineStr">
+        <is>
+          <t>s radier utilisée</t>
+        </is>
+      </c>
+      <c r="G26" s="275" t="inlineStr">
+        <is>
+          <t>U amont (m)</t>
+        </is>
+      </c>
+      <c r="H26" s="275" t="inlineStr">
+        <is>
+          <t>V aval (m)</t>
+        </is>
+      </c>
+      <c r="I26" s="275" t="inlineStr">
+        <is>
+          <t>ΔU-V (m)</t>
+        </is>
+      </c>
+      <c r="J26" s="275" t="inlineStr">
+        <is>
+          <t>s réelle (U-V)/L</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="276" t="inlineStr">
+        <is>
+          <t>L06_P09_P06</t>
+        </is>
+      </c>
+      <c r="B27" s="276" t="inlineStr">
+        <is>
+          <t>P09</t>
+        </is>
+      </c>
+      <c r="C27" s="276" t="inlineStr">
+        <is>
+          <t>P06</t>
+        </is>
+      </c>
+      <c r="D27" s="279" t="n">
+        <v>17.458</v>
+      </c>
+      <c r="E27" s="280" t="n">
+        <v>0.0306</v>
+      </c>
+      <c r="F27" s="281" t="n">
+        <v>0.0306</v>
+      </c>
+      <c r="G27" s="277" t="n">
+        <v>16.976</v>
+      </c>
+      <c r="H27" s="277" t="n">
+        <v>16.422</v>
+      </c>
+      <c r="I27" s="277" t="n">
+        <v>0.554</v>
+      </c>
+      <c r="J27" s="281" t="n">
+        <v>0.0317</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="276" t="inlineStr">
+        <is>
+          <t>L07_P07_P06</t>
+        </is>
+      </c>
+      <c r="B28" s="276" t="inlineStr">
+        <is>
+          <t>P07</t>
+        </is>
+      </c>
+      <c r="C28" s="276" t="inlineStr">
+        <is>
+          <t>P06</t>
+        </is>
+      </c>
+      <c r="D28" s="279" t="n">
+        <v>12.477</v>
+      </c>
+      <c r="E28" s="280" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="F28" s="281" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="G28" s="277" t="n">
+        <v>16.567</v>
+      </c>
+      <c r="H28" s="277" t="n">
+        <v>16.422</v>
+      </c>
+      <c r="I28" s="277" t="n">
+        <v>0.145</v>
+      </c>
+      <c r="J28" s="281" t="n">
+        <v>0.0116</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="276" t="inlineStr">
+        <is>
+          <t>L08_P06_P04</t>
+        </is>
+      </c>
+      <c r="B29" s="276" t="inlineStr">
+        <is>
+          <t>P06</t>
+        </is>
+      </c>
+      <c r="C29" s="276" t="inlineStr">
+        <is>
+          <t>P04</t>
+        </is>
+      </c>
+      <c r="D29" s="279" t="n">
+        <v>9.579000000000001</v>
+      </c>
+      <c r="E29" s="280" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="F29" s="281" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="G29" s="277" t="n">
+        <v>16.422</v>
+      </c>
+      <c r="H29" s="277" t="n">
+        <v>16.306</v>
+      </c>
+      <c r="I29" s="277" t="n">
+        <v>0.116</v>
+      </c>
+      <c r="J29" s="281" t="n">
+        <v>0.0121</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="276" t="inlineStr">
+        <is>
+          <t>L09_P04_P01</t>
+        </is>
+      </c>
+      <c r="B30" s="276" t="inlineStr">
+        <is>
+          <t>P04</t>
+        </is>
+      </c>
+      <c r="C30" s="276" t="inlineStr">
+        <is>
+          <t>P01</t>
+        </is>
+      </c>
+      <c r="D30" s="279" t="n">
+        <v>13.317</v>
+      </c>
+      <c r="E30" s="280" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="F30" s="281" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="G30" s="277" t="n">
+        <v>16.306</v>
+      </c>
+      <c r="H30" s="277" t="n">
+        <v>16.153</v>
+      </c>
+      <c r="I30" s="277" t="n">
+        <v>0.153</v>
+      </c>
+      <c r="J30" s="281" t="n">
+        <v>0.0115</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="276" t="inlineStr">
+        <is>
+          <t>L01_P01_J01</t>
+        </is>
+      </c>
+      <c r="B31" s="276" t="inlineStr">
+        <is>
+          <t>P01</t>
+        </is>
+      </c>
+      <c r="C31" s="276" t="inlineStr">
+        <is>
+          <t>J01</t>
+        </is>
+      </c>
+      <c r="D31" s="279" t="n">
+        <v>14.401</v>
+      </c>
+      <c r="E31" s="280" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="F31" s="281" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="G31" s="277" t="n">
+        <v>16.153</v>
+      </c>
+      <c r="H31" s="277" t="n">
+        <v>15.989</v>
+      </c>
+      <c r="I31" s="277" t="n">
+        <v>0.164</v>
+      </c>
+      <c r="J31" s="281" t="n">
+        <v>0.0114</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="276" t="inlineStr">
+        <is>
+          <t>L12_P02_J01</t>
+        </is>
+      </c>
+      <c r="B32" s="276" t="inlineStr">
+        <is>
+          <t>P02</t>
+        </is>
+      </c>
+      <c r="C32" s="276" t="inlineStr">
+        <is>
+          <t>J01</t>
+        </is>
+      </c>
+      <c r="D32" s="279" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="E32" s="280" t="n">
+        <v>0.0114</v>
+      </c>
+      <c r="F32" s="281" t="n">
+        <v>0.0114</v>
+      </c>
+      <c r="G32" s="277" t="n">
+        <v>16.025</v>
+      </c>
+      <c r="H32" s="277" t="n">
+        <v>15.989</v>
+      </c>
+      <c r="I32" s="277" t="n">
+        <v>0.036</v>
+      </c>
+      <c r="J32" s="281" t="n">
+        <v>0.0257</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="276" t="inlineStr">
+        <is>
+          <t>L02_J01_RP03</t>
+        </is>
+      </c>
+      <c r="B33" s="276" t="inlineStr">
+        <is>
+          <t>J01</t>
+        </is>
+      </c>
+      <c r="C33" s="276" t="inlineStr">
+        <is>
+          <t>RP03</t>
+        </is>
+      </c>
+      <c r="D33" s="279" t="n">
+        <v>11.2</v>
+      </c>
+      <c r="E33" s="280" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="F33" s="281" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="G33" s="277" t="n">
+        <v>15.989</v>
+      </c>
+      <c r="H33" s="277" t="n">
+        <v>15.857</v>
+      </c>
+      <c r="I33" s="277" t="n">
+        <v>0.132</v>
+      </c>
+      <c r="J33" s="281" t="n">
+        <v>0.0118</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="276" t="inlineStr">
+        <is>
+          <t>L03_RP03_P10</t>
+        </is>
+      </c>
+      <c r="B34" s="276" t="inlineStr">
+        <is>
+          <t>RP03</t>
+        </is>
+      </c>
+      <c r="C34" s="276" t="inlineStr">
+        <is>
+          <t>P10</t>
+        </is>
+      </c>
+      <c r="D34" s="279" t="n">
+        <v>7.1</v>
+      </c>
+      <c r="E34" s="280" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="F34" s="281" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="G34" s="277" t="n">
+        <v>15.857</v>
+      </c>
+      <c r="H34" s="277" t="n">
+        <v>15.766</v>
+      </c>
+      <c r="I34" s="277" t="n">
+        <v>0.091</v>
+      </c>
+      <c r="J34" s="281" t="n">
+        <v>0.0128</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="276" t="inlineStr">
+        <is>
+          <t>L10_P10_P11</t>
+        </is>
+      </c>
+      <c r="B35" s="276" t="inlineStr">
+        <is>
+          <t>P10</t>
+        </is>
+      </c>
+      <c r="C35" s="276" t="inlineStr">
+        <is>
+          <t>P11</t>
+        </is>
+      </c>
+      <c r="D35" s="279" t="n">
+        <v>14.3</v>
+      </c>
+      <c r="E35" s="280" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="F35" s="281" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="G35" s="277" t="n">
+        <v>15.766</v>
+      </c>
+      <c r="H35" s="277" t="n">
+        <v>15.603</v>
+      </c>
+      <c r="I35" s="277" t="n">
+        <v>0.163</v>
+      </c>
+      <c r="J35" s="281" t="n">
+        <v>0.0114</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="276" t="inlineStr">
+        <is>
+          <t>LT1_T1_P11</t>
+        </is>
+      </c>
+      <c r="B36" s="276" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="C36" s="276" t="inlineStr">
+        <is>
+          <t>P11</t>
+        </is>
+      </c>
+      <c r="D36" s="279" t="n">
+        <v>12</v>
+      </c>
+      <c r="E36" s="280" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="F36" s="281" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="G36" s="277" t="n">
+        <v>15.743</v>
+      </c>
+      <c r="H36" s="277" t="n">
+        <v>15.603</v>
+      </c>
+      <c r="I36" s="277" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="J36" s="281" t="n">
+        <v>0.0117</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="276" t="inlineStr">
+        <is>
+          <t>L11_P11_P12</t>
+        </is>
+      </c>
+      <c r="B37" s="276" t="inlineStr">
+        <is>
+          <t>P11</t>
+        </is>
+      </c>
+      <c r="C37" s="276" t="inlineStr">
+        <is>
+          <t>P12</t>
+        </is>
+      </c>
+      <c r="D37" s="279" t="n">
+        <v>10.9</v>
+      </c>
+      <c r="E37" s="280" t="n">
+        <v>0.0123</v>
+      </c>
+      <c r="F37" s="281" t="n">
+        <v>0.0123</v>
+      </c>
+      <c r="G37" s="277" t="n">
+        <v>15.603</v>
+      </c>
+      <c r="H37" s="277" t="n">
+        <v>15.449</v>
+      </c>
+      <c r="I37" s="277" t="n">
+        <v>0.154</v>
+      </c>
+      <c r="J37" s="281" t="n">
+        <v>0.0141</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="276" t="inlineStr">
+        <is>
+          <t>L12_P12_PUB</t>
+        </is>
+      </c>
+      <c r="B38" s="276" t="inlineStr">
+        <is>
+          <t>P12</t>
+        </is>
+      </c>
+      <c r="C38" s="276" t="inlineStr">
+        <is>
+          <t>PUB</t>
+        </is>
+      </c>
+      <c r="D38" s="279" t="n">
+        <v>12.4</v>
+      </c>
+      <c r="E38" s="280" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="F38" s="281" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="G38" s="277" t="n">
+        <v>15.449</v>
+      </c>
+      <c r="H38" s="277" t="n">
+        <v>15.305</v>
+      </c>
+      <c r="I38" s="277" t="n">
+        <v>0.144</v>
+      </c>
+      <c r="J38" s="281" t="n">
+        <v>0.0116</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="282" t="inlineStr">
+        <is>
+          <t>Lecture: aux confluences, la cellule Invert orange = MIN des propositions des branches.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Les U/V de Calcul_reseau sont alignés sur cette table. Si vous changez une longueur (ex. T1), il faut recalculer les radiers.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AC173"/>
+  <dimension ref="A1:AC174"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="12" customWidth="1" style="206" min="1" max="1"/>
@@ -2240,7 +3380,7 @@
       <c r="G2" s="234" t="n"/>
       <c r="H2" s="10" t="inlineStr">
         <is>
-          <t>Réseau pluvial – projet (fichier Olivier TECH. MODIF)</t>
+          <t>Réseau pluvial – Olivier TECH. MODIF + radiers + T1</t>
         </is>
       </c>
       <c r="I2" s="10" t="n"/>
@@ -2323,7 +3463,7 @@
       <c r="L4" s="23" t="n"/>
       <c r="M4" s="215" t="inlineStr">
         <is>
-          <t>Réseau local → exutoire P12 / PUB</t>
+          <t>Réseau local → T1/P11 → P12 / PUB</t>
         </is>
       </c>
       <c r="P4" s="236" t="n"/>
@@ -2989,7 +4129,7 @@
     <row r="17" ht="22.5" customHeight="1" s="227">
       <c r="A17" s="104" t="inlineStr">
         <is>
-          <t>Tronçons (amont → aval) — modif Olivier: P01→J01, P02→J01 (1.4 m), J01→RP03</t>
+          <t>Tronçons (amont → aval) — J01 + T1(toit)→P11; radiers: plus bas aux confluences</t>
         </is>
       </c>
       <c r="B17" s="92" t="n"/>
@@ -3035,80 +4175,88 @@
           <t>P06</t>
         </is>
       </c>
-      <c r="D18" s="108">
+      <c r="D18" s="249">
         <f>'Temps de concentration'!B7</f>
         <v/>
       </c>
-      <c r="E18" s="109" t="n">
+      <c r="E18" s="283" t="n">
         <v>0.0447</v>
       </c>
-      <c r="F18" s="110" t="n">
+      <c r="F18" s="284" t="n">
         <v>0.425</v>
       </c>
-      <c r="G18" s="111">
+      <c r="G18" s="250">
         <f>E18*F18</f>
         <v/>
       </c>
-      <c r="H18" s="111">
+      <c r="H18" s="250">
         <f>E18</f>
         <v/>
       </c>
-      <c r="I18" s="111">
+      <c r="I18" s="250">
         <f>G18</f>
         <v/>
       </c>
-      <c r="J18" s="112">
+      <c r="J18" s="253">
         <f>IF(H18=0,0,I18/H18)</f>
         <v/>
       </c>
-      <c r="K18" s="108">
+      <c r="K18" s="249">
         <f>IF($S$2=0.5,$R$5/((D18+$S$5)^$T$5),IF($S$2=0.2,$R$6/((D18+$S$6)^$T$6),IF($S$2=0.1,$R$7/((D18+$S$7)^$T$7),IF($S$2=0.04,$R$8/((D18+$S$8)^$T$8),IF($S$2=0.02,$R$9/((D18+$S$9)^$T$9),$R$10/((D18+$S$10)^$T$10))))))</f>
         <v/>
       </c>
-      <c r="L18" s="112">
+      <c r="L18" s="253">
         <f>0.00275*H18*J18*K18</f>
         <v/>
       </c>
-      <c r="M18" s="109" t="n">
+      <c r="M18" s="283" t="n">
         <v>0.0306</v>
       </c>
-      <c r="N18" s="113" t="n">
+      <c r="N18" s="285" t="n">
         <v>200</v>
       </c>
-      <c r="O18" s="108">
+      <c r="O18" s="249">
         <f>IF(OR(N18&lt;=0,M18&lt;=0),0,((N18/4000)^(2/3)*SQRT(M18))/$S$11)</f>
         <v/>
       </c>
-      <c r="P18" s="248" t="n">
+      <c r="P18" s="286" t="n">
         <v>17.458</v>
       </c>
-      <c r="Q18" s="108">
+      <c r="Q18" s="249">
         <f>IF(O18=0,0,P18/(O18*60))</f>
         <v/>
       </c>
-      <c r="R18" s="112">
+      <c r="R18" s="253">
         <f>O18*(PI()*(N18/1000)^2/4)</f>
         <v/>
       </c>
-      <c r="S18" s="114" t="n"/>
-      <c r="T18" s="114" t="n"/>
-      <c r="U18" s="231">
-        <f>V18+(M18*P18)</f>
-        <v/>
-      </c>
-      <c r="V18" s="231">
-        <f>U19</f>
-        <v/>
-      </c>
-      <c r="W18" s="112" t="n"/>
-      <c r="X18" s="112" t="n"/>
-      <c r="Y18" s="112">
+      <c r="S18" s="287" t="n">
+        <v>17.62</v>
+      </c>
+      <c r="T18" s="287" t="n">
+        <v>17.14</v>
+      </c>
+      <c r="U18" s="253" t="n">
+        <v>16.976</v>
+      </c>
+      <c r="V18" s="253" t="n">
+        <v>16.422</v>
+      </c>
+      <c r="W18" s="253">
+        <f>IF(OR(S18="",U18=""),"",S18-U18-N18/1000)</f>
+        <v/>
+      </c>
+      <c r="X18" s="253">
+        <f>IF(OR(T18="",V18=""),"",T18-V18-N18/1000)</f>
+        <v/>
+      </c>
+      <c r="Y18" s="253">
         <f>P18*PI()*(N18/1000)^2/4</f>
         <v/>
       </c>
       <c r="Z18" s="95" t="n"/>
       <c r="AA18" s="115" t="n"/>
-      <c r="AB18" s="116">
+      <c r="AB18" s="256">
         <f>IF(R18&gt;L18,"OK","AUGMENTER D")</f>
         <v/>
       </c>
@@ -3134,80 +4282,88 @@
           <t>P06</t>
         </is>
       </c>
-      <c r="D19" s="108">
+      <c r="D19" s="249">
         <f>MAX('Temps de concentration'!C7, D18+Q18)</f>
         <v/>
       </c>
-      <c r="E19" s="109" t="n">
+      <c r="E19" s="283" t="n">
         <v>0.0442</v>
       </c>
-      <c r="F19" s="110" t="n">
+      <c r="F19" s="284" t="n">
         <v>0.765</v>
       </c>
-      <c r="G19" s="111">
+      <c r="G19" s="250">
         <f>E19*F19</f>
         <v/>
       </c>
-      <c r="H19" s="111">
-        <f>H18+E19</f>
-        <v/>
-      </c>
-      <c r="I19" s="111">
-        <f>I18+G19</f>
-        <v/>
-      </c>
-      <c r="J19" s="112">
+      <c r="H19" s="250">
+        <f>E19</f>
+        <v/>
+      </c>
+      <c r="I19" s="250">
+        <f>G19</f>
+        <v/>
+      </c>
+      <c r="J19" s="253">
         <f>IF(H19=0,0,I19/H19)</f>
         <v/>
       </c>
-      <c r="K19" s="108">
+      <c r="K19" s="249">
         <f>IF($S$2=0.5,$R$5/((D19+$S$5)^$T$5),IF($S$2=0.2,$R$6/((D19+$S$6)^$T$6),IF($S$2=0.1,$R$7/((D19+$S$7)^$T$7),IF($S$2=0.04,$R$8/((D19+$S$8)^$T$8),IF($S$2=0.02,$R$9/((D19+$S$9)^$T$9),$R$10/((D19+$S$10)^$T$10))))))</f>
         <v/>
       </c>
-      <c r="L19" s="112">
+      <c r="L19" s="253">
         <f>0.00275*H19*J19*K19</f>
         <v/>
       </c>
-      <c r="M19" s="109" t="n">
+      <c r="M19" s="283" t="n">
         <v>0.01</v>
       </c>
-      <c r="N19" s="113" t="n">
+      <c r="N19" s="285" t="n">
         <v>200</v>
       </c>
-      <c r="O19" s="108">
+      <c r="O19" s="249">
         <f>IF(OR(N19&lt;=0,M19&lt;=0),0,((N19/4000)^(2/3)*SQRT(M19))/$S$11)</f>
         <v/>
       </c>
-      <c r="P19" s="248" t="n">
+      <c r="P19" s="286" t="n">
         <v>12.477</v>
       </c>
-      <c r="Q19" s="108">
+      <c r="Q19" s="249">
         <f>IF(O19=0,0,P19/(O19*60))</f>
         <v/>
       </c>
-      <c r="R19" s="112">
+      <c r="R19" s="253">
         <f>O19*(PI()*(N19/1000)^2/4)</f>
         <v/>
       </c>
-      <c r="S19" s="114" t="n"/>
-      <c r="T19" s="114" t="n"/>
-      <c r="U19" s="231">
-        <f>V19+(M19*P19)</f>
-        <v/>
-      </c>
-      <c r="V19" s="231">
-        <f>U20</f>
-        <v/>
-      </c>
-      <c r="W19" s="112" t="n"/>
-      <c r="X19" s="112" t="n"/>
-      <c r="Y19" s="112">
+      <c r="S19" s="287" t="n">
+        <v>17.09</v>
+      </c>
+      <c r="T19" s="287" t="n">
+        <v>17.14</v>
+      </c>
+      <c r="U19" s="253" t="n">
+        <v>16.567</v>
+      </c>
+      <c r="V19" s="253" t="n">
+        <v>16.422</v>
+      </c>
+      <c r="W19" s="253">
+        <f>IF(OR(S19="",U19=""),"",S19-U19-N19/1000)</f>
+        <v/>
+      </c>
+      <c r="X19" s="253">
+        <f>IF(OR(T19="",V19=""),"",T19-V19-N19/1000)</f>
+        <v/>
+      </c>
+      <c r="Y19" s="253">
         <f>P19*PI()*(N19/1000)^2/4</f>
         <v/>
       </c>
       <c r="Z19" s="95" t="n"/>
       <c r="AA19" s="115" t="n"/>
-      <c r="AB19" s="116">
+      <c r="AB19" s="256">
         <f>IF(R19&gt;L19,"OK","AUGMENTER D")</f>
         <v/>
       </c>
@@ -3233,80 +4389,88 @@
           <t>P04</t>
         </is>
       </c>
-      <c r="D20" s="108">
-        <f>MAX('Temps de concentration'!D7, D19+Q19)</f>
-        <v/>
-      </c>
-      <c r="E20" s="109" t="n">
+      <c r="D20" s="249">
+        <f>MAX('Temps de concentration'!D7, MAX(D18+Q18,D19+Q19))</f>
+        <v/>
+      </c>
+      <c r="E20" s="283" t="n">
         <v>0.0148</v>
       </c>
-      <c r="F20" s="110" t="n">
+      <c r="F20" s="284" t="n">
         <v>0.6840000000000001</v>
       </c>
-      <c r="G20" s="111">
+      <c r="G20" s="250">
         <f>E20*F20</f>
         <v/>
       </c>
-      <c r="H20" s="111">
-        <f>H19+E20</f>
-        <v/>
-      </c>
-      <c r="I20" s="111">
-        <f>I19+G20</f>
-        <v/>
-      </c>
-      <c r="J20" s="112">
+      <c r="H20" s="250">
+        <f>H18+H19+E20</f>
+        <v/>
+      </c>
+      <c r="I20" s="250">
+        <f>I18+I19+G20</f>
+        <v/>
+      </c>
+      <c r="J20" s="253">
         <f>IF(H20=0,0,I20/H20)</f>
         <v/>
       </c>
-      <c r="K20" s="108">
+      <c r="K20" s="249">
         <f>IF($S$2=0.5,$R$5/((D20+$S$5)^$T$5),IF($S$2=0.2,$R$6/((D20+$S$6)^$T$6),IF($S$2=0.1,$R$7/((D20+$S$7)^$T$7),IF($S$2=0.04,$R$8/((D20+$S$8)^$T$8),IF($S$2=0.02,$R$9/((D20+$S$9)^$T$9),$R$10/((D20+$S$10)^$T$10))))))</f>
         <v/>
       </c>
-      <c r="L20" s="112">
+      <c r="L20" s="253">
         <f>0.00275*H20*J20*K20</f>
         <v/>
       </c>
-      <c r="M20" s="109" t="n">
+      <c r="M20" s="283" t="n">
         <v>0.01</v>
       </c>
-      <c r="N20" s="113" t="n">
+      <c r="N20" s="285" t="n">
         <v>200</v>
       </c>
-      <c r="O20" s="108">
+      <c r="O20" s="249">
         <f>IF(OR(N20&lt;=0,M20&lt;=0),0,((N20/4000)^(2/3)*SQRT(M20))/$S$11)</f>
         <v/>
       </c>
-      <c r="P20" s="248" t="n">
+      <c r="P20" s="286" t="n">
         <v>9.579000000000001</v>
       </c>
-      <c r="Q20" s="108">
+      <c r="Q20" s="249">
         <f>IF(O20=0,0,P20/(O20*60))</f>
         <v/>
       </c>
-      <c r="R20" s="112">
+      <c r="R20" s="253">
         <f>O20*(PI()*(N20/1000)^2/4)</f>
         <v/>
       </c>
-      <c r="S20" s="114" t="n"/>
-      <c r="T20" s="114" t="n"/>
-      <c r="U20" s="231">
-        <f>V20+(M20*P20)</f>
-        <v/>
-      </c>
-      <c r="V20" s="231">
-        <f>U21</f>
-        <v/>
-      </c>
-      <c r="W20" s="112" t="n"/>
-      <c r="X20" s="112" t="n"/>
-      <c r="Y20" s="112">
+      <c r="S20" s="287" t="n">
+        <v>17.14</v>
+      </c>
+      <c r="T20" s="287" t="n">
+        <v>17.28</v>
+      </c>
+      <c r="U20" s="253" t="n">
+        <v>16.422</v>
+      </c>
+      <c r="V20" s="253" t="n">
+        <v>16.306</v>
+      </c>
+      <c r="W20" s="253">
+        <f>IF(OR(S20="",U20=""),"",S20-U20-N20/1000)</f>
+        <v/>
+      </c>
+      <c r="X20" s="253">
+        <f>IF(OR(T20="",V20=""),"",T20-V20-N20/1000)</f>
+        <v/>
+      </c>
+      <c r="Y20" s="253">
         <f>P20*PI()*(N20/1000)^2/4</f>
         <v/>
       </c>
       <c r="Z20" s="95" t="n"/>
       <c r="AA20" s="115" t="n"/>
-      <c r="AB20" s="116">
+      <c r="AB20" s="256">
         <f>IF(R20&gt;L20,"OK","AUGMENTER D")</f>
         <v/>
       </c>
@@ -3332,80 +4496,88 @@
           <t>P01</t>
         </is>
       </c>
-      <c r="D21" s="108">
+      <c r="D21" s="249">
         <f>MAX('Temps de concentration'!E7, D20+Q20)</f>
         <v/>
       </c>
-      <c r="E21" s="109" t="n">
+      <c r="E21" s="283" t="n">
         <v>0.0095</v>
       </c>
-      <c r="F21" s="110" t="n">
+      <c r="F21" s="284" t="n">
         <v>0.547</v>
       </c>
-      <c r="G21" s="111">
+      <c r="G21" s="250">
         <f>E21*F21</f>
         <v/>
       </c>
-      <c r="H21" s="111">
+      <c r="H21" s="250">
         <f>H20+E21</f>
         <v/>
       </c>
-      <c r="I21" s="111">
+      <c r="I21" s="250">
         <f>I20+G21</f>
         <v/>
       </c>
-      <c r="J21" s="112">
+      <c r="J21" s="253">
         <f>IF(H21=0,0,I21/H21)</f>
         <v/>
       </c>
-      <c r="K21" s="108">
+      <c r="K21" s="249">
         <f>IF($S$2=0.5,$R$5/((D21+$S$5)^$T$5),IF($S$2=0.2,$R$6/((D21+$S$6)^$T$6),IF($S$2=0.1,$R$7/((D21+$S$7)^$T$7),IF($S$2=0.04,$R$8/((D21+$S$8)^$T$8),IF($S$2=0.02,$R$9/((D21+$S$9)^$T$9),$R$10/((D21+$S$10)^$T$10))))))</f>
         <v/>
       </c>
-      <c r="L21" s="112">
+      <c r="L21" s="253">
         <f>0.00275*H21*J21*K21</f>
         <v/>
       </c>
-      <c r="M21" s="109" t="n">
+      <c r="M21" s="283" t="n">
         <v>0.01</v>
       </c>
-      <c r="N21" s="113" t="n">
+      <c r="N21" s="285" t="n">
         <v>250</v>
       </c>
-      <c r="O21" s="108">
+      <c r="O21" s="249">
         <f>IF(OR(N21&lt;=0,M21&lt;=0),0,((N21/4000)^(2/3)*SQRT(M21))/$S$11)</f>
         <v/>
       </c>
-      <c r="P21" s="248" t="n">
+      <c r="P21" s="286" t="n">
         <v>13.317</v>
       </c>
-      <c r="Q21" s="108">
+      <c r="Q21" s="249">
         <f>IF(O21=0,0,P21/(O21*60))</f>
         <v/>
       </c>
-      <c r="R21" s="112">
+      <c r="R21" s="253">
         <f>O21*(PI()*(N21/1000)^2/4)</f>
         <v/>
       </c>
-      <c r="S21" s="114" t="n"/>
-      <c r="T21" s="114" t="n"/>
-      <c r="U21" s="231">
-        <f>V21+(M21*P21)</f>
-        <v/>
-      </c>
-      <c r="V21" s="231">
-        <f>U22</f>
-        <v/>
-      </c>
-      <c r="W21" s="112" t="n"/>
-      <c r="X21" s="112" t="n"/>
-      <c r="Y21" s="112">
+      <c r="S21" s="287" t="n">
+        <v>17.28</v>
+      </c>
+      <c r="T21" s="287" t="n">
+        <v>17.23</v>
+      </c>
+      <c r="U21" s="253" t="n">
+        <v>16.306</v>
+      </c>
+      <c r="V21" s="253" t="n">
+        <v>16.153</v>
+      </c>
+      <c r="W21" s="253">
+        <f>IF(OR(S21="",U21=""),"",S21-U21-N21/1000)</f>
+        <v/>
+      </c>
+      <c r="X21" s="253">
+        <f>IF(OR(T21="",V21=""),"",T21-V21-N21/1000)</f>
+        <v/>
+      </c>
+      <c r="Y21" s="253">
         <f>P21*PI()*(N21/1000)^2/4</f>
         <v/>
       </c>
       <c r="Z21" s="95" t="n"/>
       <c r="AA21" s="115" t="n"/>
-      <c r="AB21" s="116">
+      <c r="AB21" s="256">
         <f>IF(R21&gt;L21,"OK","AUGMENTER D")</f>
         <v/>
       </c>
@@ -3431,80 +4603,88 @@
           <t>J01</t>
         </is>
       </c>
-      <c r="D22" s="108">
+      <c r="D22" s="249">
         <f>MAX('Temps de concentration'!F7, D21+Q21)</f>
         <v/>
       </c>
-      <c r="E22" s="109" t="n">
+      <c r="E22" s="283" t="n">
         <v>0.0257</v>
       </c>
-      <c r="F22" s="110" t="n">
+      <c r="F22" s="284" t="n">
         <v>0.633</v>
       </c>
-      <c r="G22" s="111">
+      <c r="G22" s="250">
         <f>E22*F22</f>
         <v/>
       </c>
-      <c r="H22" s="111">
+      <c r="H22" s="250">
         <f>H21+E22</f>
         <v/>
       </c>
-      <c r="I22" s="111">
+      <c r="I22" s="250">
         <f>I21+G22</f>
         <v/>
       </c>
-      <c r="J22" s="112">
+      <c r="J22" s="253">
         <f>IF(H22=0,0,I22/H22)</f>
         <v/>
       </c>
-      <c r="K22" s="108">
+      <c r="K22" s="249">
         <f>IF($S$2=0.5,$R$5/((D22+$S$5)^$T$5),IF($S$2=0.2,$R$6/((D22+$S$6)^$T$6),IF($S$2=0.1,$R$7/((D22+$S$7)^$T$7),IF($S$2=0.04,$R$8/((D22+$S$8)^$T$8),IF($S$2=0.02,$R$9/((D22+$S$9)^$T$9),$R$10/((D22+$S$10)^$T$10))))))</f>
         <v/>
       </c>
-      <c r="L22" s="112">
+      <c r="L22" s="253">
         <f>0.00275*H22*J22*K22</f>
         <v/>
       </c>
-      <c r="M22" s="109" t="n">
+      <c r="M22" s="283" t="n">
         <v>0.01</v>
       </c>
-      <c r="N22" s="113" t="n">
+      <c r="N22" s="285" t="n">
         <v>250</v>
       </c>
-      <c r="O22" s="108">
+      <c r="O22" s="249">
         <f>IF(OR(N22&lt;=0,M22&lt;=0),0,((N22/4000)^(2/3)*SQRT(M22))/$S$11)</f>
         <v/>
       </c>
-      <c r="P22" s="248" t="n">
+      <c r="P22" s="286" t="n">
         <v>14.401</v>
       </c>
-      <c r="Q22" s="108">
+      <c r="Q22" s="249">
         <f>IF(O22=0,0,P22/(O22*60))</f>
         <v/>
       </c>
-      <c r="R22" s="112">
+      <c r="R22" s="253">
         <f>O22*(PI()*(N22/1000)^2/4)</f>
         <v/>
       </c>
-      <c r="S22" s="114" t="n"/>
-      <c r="T22" s="114" t="n"/>
-      <c r="U22" s="231">
-        <f>V22+(M22*P22)</f>
-        <v/>
-      </c>
-      <c r="V22" s="231">
-        <f>U23</f>
-        <v/>
-      </c>
-      <c r="W22" s="112" t="n"/>
-      <c r="X22" s="112" t="n"/>
-      <c r="Y22" s="112">
+      <c r="S22" s="287" t="n">
+        <v>17.23</v>
+      </c>
+      <c r="T22" s="287" t="n">
+        <v>17.12</v>
+      </c>
+      <c r="U22" s="253" t="n">
+        <v>16.153</v>
+      </c>
+      <c r="V22" s="253" t="n">
+        <v>15.989</v>
+      </c>
+      <c r="W22" s="253">
+        <f>IF(OR(S22="",U22=""),"",S22-U22-N22/1000)</f>
+        <v/>
+      </c>
+      <c r="X22" s="253">
+        <f>IF(OR(T22="",V22=""),"",T22-V22-N22/1000)</f>
+        <v/>
+      </c>
+      <c r="Y22" s="253">
         <f>P22*PI()*(N22/1000)^2/4</f>
         <v/>
       </c>
       <c r="Z22" s="95" t="n"/>
       <c r="AA22" s="115" t="n"/>
-      <c r="AB22" s="116">
+      <c r="AB22" s="256">
         <f>IF(R22&gt;L22,"OK","AUGMENTER D")</f>
         <v/>
       </c>
@@ -3534,13 +4714,13 @@
         <f>'Temps de concentration'!G7</f>
         <v/>
       </c>
-      <c r="E23" s="109" t="n">
+      <c r="E23" s="283" t="n">
         <v>0.0468</v>
       </c>
-      <c r="F23" s="110" t="n">
+      <c r="F23" s="284" t="n">
         <v>0.642</v>
       </c>
-      <c r="G23" s="111">
+      <c r="G23" s="250">
         <f>E23*F23</f>
         <v/>
       </c>
@@ -3552,58 +4732,66 @@
         <f>G23</f>
         <v/>
       </c>
-      <c r="J23" s="112">
+      <c r="J23" s="253">
         <f>IF(H23=0,0,I23/H23)</f>
         <v/>
       </c>
-      <c r="K23" s="108">
+      <c r="K23" s="249">
         <f>IF($S$2=0.5,$R$5/((D23+$S$5)^$T$5),IF($S$2=0.2,$R$6/((D23+$S$6)^$T$6),IF($S$2=0.1,$R$7/((D23+$S$7)^$T$7),IF($S$2=0.04,$R$8/((D23+$S$8)^$T$8),IF($S$2=0.02,$R$9/((D23+$S$9)^$T$9),$R$10/((D23+$S$10)^$T$10))))))</f>
         <v/>
       </c>
-      <c r="L23" s="112">
+      <c r="L23" s="253">
         <f>0.00275*H23*J23*K23</f>
         <v/>
       </c>
-      <c r="M23" s="109" t="n">
+      <c r="M23" s="283" t="n">
         <v>0.0114</v>
       </c>
-      <c r="N23" s="113" t="n">
+      <c r="N23" s="285" t="n">
         <v>250</v>
       </c>
-      <c r="O23" s="108">
+      <c r="O23" s="249">
         <f>IF(OR(N23&lt;=0,M23&lt;=0),0,((N23/4000)^(2/3)*SQRT(M23))/$S$11)</f>
         <v/>
       </c>
-      <c r="P23" s="248" t="n">
+      <c r="P23" s="286" t="n">
         <v>1.4</v>
       </c>
-      <c r="Q23" s="108">
+      <c r="Q23" s="249">
         <f>IF(O23=0,0,P23/(O23*60))</f>
         <v/>
       </c>
-      <c r="R23" s="112">
+      <c r="R23" s="253">
         <f>O23*(PI()*(N23/1000)^2/4)</f>
         <v/>
       </c>
-      <c r="S23" s="114" t="n"/>
-      <c r="T23" s="114" t="n"/>
-      <c r="U23" s="231">
-        <f>V23+(M23*P23)</f>
-        <v/>
-      </c>
-      <c r="V23" s="231">
-        <f>U24</f>
-        <v/>
-      </c>
-      <c r="W23" s="112" t="n"/>
-      <c r="X23" s="112" t="n"/>
-      <c r="Y23" s="112">
+      <c r="S23" s="287" t="n">
+        <v>17.131</v>
+      </c>
+      <c r="T23" s="287" t="n">
+        <v>17.12</v>
+      </c>
+      <c r="U23" s="253" t="n">
+        <v>16.025</v>
+      </c>
+      <c r="V23" s="253" t="n">
+        <v>15.989</v>
+      </c>
+      <c r="W23" s="253">
+        <f>IF(OR(S23="",U23=""),"",S23-U23-N23/1000)</f>
+        <v/>
+      </c>
+      <c r="X23" s="253">
+        <f>IF(OR(T23="",V23=""),"",T23-V23-N23/1000)</f>
+        <v/>
+      </c>
+      <c r="Y23" s="253">
         <f>P23*PI()*(N23/1000)^2/4</f>
         <v/>
       </c>
       <c r="Z23" s="95" t="n"/>
       <c r="AA23" s="115" t="n"/>
-      <c r="AB23" s="116">
+      <c r="AB23" s="256">
         <f>IF(R23&gt;L23,"OK","AUGMENTER D")</f>
         <v/>
       </c>
@@ -3633,13 +4821,13 @@
         <f>MAX(D22+Q22, D23+Q23)</f>
         <v/>
       </c>
-      <c r="E24" s="109" t="n">
+      <c r="E24" s="283" t="n">
         <v>0</v>
       </c>
-      <c r="F24" s="110" t="n">
+      <c r="F24" s="284" t="n">
         <v>0.9</v>
       </c>
-      <c r="G24" s="111">
+      <c r="G24" s="250">
         <f>E24*F24</f>
         <v/>
       </c>
@@ -3651,58 +4839,66 @@
         <f>I22+I23+G24</f>
         <v/>
       </c>
-      <c r="J24" s="112">
+      <c r="J24" s="253">
         <f>IF(H24=0,0,I24/H24)</f>
         <v/>
       </c>
-      <c r="K24" s="108">
+      <c r="K24" s="249">
         <f>IF($S$2=0.5,$R$5/((D24+$S$5)^$T$5),IF($S$2=0.2,$R$6/((D24+$S$6)^$T$6),IF($S$2=0.1,$R$7/((D24+$S$7)^$T$7),IF($S$2=0.04,$R$8/((D24+$S$8)^$T$8),IF($S$2=0.02,$R$9/((D24+$S$9)^$T$9),$R$10/((D24+$S$10)^$T$10))))))</f>
         <v/>
       </c>
-      <c r="L24" s="112">
+      <c r="L24" s="253">
         <f>0.00275*H24*J24*K24</f>
         <v/>
       </c>
-      <c r="M24" s="109" t="n">
+      <c r="M24" s="283" t="n">
         <v>0.01</v>
       </c>
-      <c r="N24" s="113" t="n">
+      <c r="N24" s="285" t="n">
         <v>250</v>
       </c>
-      <c r="O24" s="108">
+      <c r="O24" s="249">
         <f>IF(OR(N24&lt;=0,M24&lt;=0),0,((N24/4000)^(2/3)*SQRT(M24))/$S$11)</f>
         <v/>
       </c>
-      <c r="P24" s="248" t="n">
+      <c r="P24" s="286" t="n">
         <v>11.2</v>
       </c>
-      <c r="Q24" s="108">
+      <c r="Q24" s="249">
         <f>IF(O24=0,0,P24/(O24*60))</f>
         <v/>
       </c>
-      <c r="R24" s="112">
+      <c r="R24" s="253">
         <f>O24*(PI()*(N24/1000)^2/4)</f>
         <v/>
       </c>
-      <c r="S24" s="114" t="n"/>
-      <c r="T24" s="114" t="n"/>
-      <c r="U24" s="231">
-        <f>V24+(M24*P24)</f>
-        <v/>
-      </c>
-      <c r="V24" s="231">
-        <f>U25</f>
-        <v/>
-      </c>
-      <c r="W24" s="112" t="n"/>
-      <c r="X24" s="112" t="n"/>
-      <c r="Y24" s="112">
+      <c r="S24" s="287" t="n">
+        <v>17.12</v>
+      </c>
+      <c r="T24" s="287" t="n">
+        <v>17.01</v>
+      </c>
+      <c r="U24" s="253" t="n">
+        <v>15.989</v>
+      </c>
+      <c r="V24" s="253" t="n">
+        <v>15.857</v>
+      </c>
+      <c r="W24" s="253">
+        <f>IF(OR(S24="",U24=""),"",S24-U24-N24/1000)</f>
+        <v/>
+      </c>
+      <c r="X24" s="253">
+        <f>IF(OR(T24="",V24=""),"",T24-V24-N24/1000)</f>
+        <v/>
+      </c>
+      <c r="Y24" s="253">
         <f>P24*PI()*(N24/1000)^2/4</f>
         <v/>
       </c>
       <c r="Z24" s="95" t="n"/>
       <c r="AA24" s="115" t="n"/>
-      <c r="AB24" s="116">
+      <c r="AB24" s="256">
         <f>IF(R24&gt;L24,"OK","AUGMENTER D")</f>
         <v/>
       </c>
@@ -3732,13 +4928,13 @@
         <f>D24+Q24</f>
         <v/>
       </c>
-      <c r="E25" s="251" t="n">
+      <c r="E25" s="283" t="n">
         <v>0</v>
       </c>
-      <c r="F25" s="252" t="n">
+      <c r="F25" s="284" t="n">
         <v>0.9</v>
       </c>
-      <c r="G25" s="111">
+      <c r="G25" s="250">
         <f>E25*F25</f>
         <v/>
       </c>
@@ -3750,58 +4946,66 @@
         <f>I24+G25</f>
         <v/>
       </c>
-      <c r="J25" s="112">
+      <c r="J25" s="253">
         <f>IF(H25=0,0,I25/H25)</f>
         <v/>
       </c>
-      <c r="K25" s="108">
+      <c r="K25" s="249">
         <f>IF($S$2=0.5,$R$5/((D25+$S$5)^$T$5),IF($S$2=0.2,$R$6/((D25+$S$6)^$T$6),IF($S$2=0.1,$R$7/((D25+$S$7)^$T$7),IF($S$2=0.04,$R$8/((D25+$S$8)^$T$8),IF($S$2=0.02,$R$9/((D25+$S$9)^$T$9),$R$10/((D25+$S$10)^$T$10))))))</f>
         <v/>
       </c>
-      <c r="L25" s="112">
+      <c r="L25" s="253">
         <f>0.00275*H25*J25*K25</f>
         <v/>
       </c>
-      <c r="M25" s="109" t="n">
+      <c r="M25" s="283" t="n">
         <v>0.01</v>
       </c>
-      <c r="N25" s="113" t="n">
+      <c r="N25" s="285" t="n">
         <v>300</v>
       </c>
-      <c r="O25" s="108">
+      <c r="O25" s="249">
         <f>IF(OR(N25&lt;=0,M25&lt;=0),0,((N25/4000)^(2/3)*SQRT(M25))/$S$11)</f>
         <v/>
       </c>
-      <c r="P25" s="248" t="n">
+      <c r="P25" s="286" t="n">
         <v>7.1</v>
       </c>
-      <c r="Q25" s="108">
+      <c r="Q25" s="249">
         <f>IF(O25=0,0,P25/(O25*60))</f>
         <v/>
       </c>
-      <c r="R25" s="112">
+      <c r="R25" s="253">
         <f>O25*(PI()*(N25/1000)^2/4)</f>
         <v/>
       </c>
-      <c r="S25" s="114" t="n"/>
-      <c r="T25" s="114" t="n"/>
-      <c r="U25" s="231">
-        <f>V25+(M25*P25)</f>
-        <v/>
-      </c>
-      <c r="V25" s="231">
-        <f>U26</f>
-        <v/>
-      </c>
-      <c r="W25" s="112" t="n"/>
-      <c r="X25" s="112" t="n"/>
-      <c r="Y25" s="112">
+      <c r="S25" s="287" t="n">
+        <v>17.01</v>
+      </c>
+      <c r="T25" s="287" t="n">
+        <v>16.965</v>
+      </c>
+      <c r="U25" s="253" t="n">
+        <v>15.857</v>
+      </c>
+      <c r="V25" s="253" t="n">
+        <v>15.766</v>
+      </c>
+      <c r="W25" s="253">
+        <f>IF(OR(S25="",U25=""),"",S25-U25-N25/1000)</f>
+        <v/>
+      </c>
+      <c r="X25" s="253">
+        <f>IF(OR(T25="",V25=""),"",T25-V25-N25/1000)</f>
+        <v/>
+      </c>
+      <c r="Y25" s="253">
         <f>P25*PI()*(N25/1000)^2/4</f>
         <v/>
       </c>
       <c r="Z25" s="95" t="n"/>
       <c r="AA25" s="115" t="n"/>
-      <c r="AB25" s="116">
+      <c r="AB25" s="256">
         <f>IF(R25&gt;L25,"OK","AUGMENTER D")</f>
         <v/>
       </c>
@@ -3831,11 +5035,11 @@
         <f>MAX('Temps de concentration'!H7, D25+Q25)</f>
         <v/>
       </c>
-      <c r="E26" s="251" t="n">
-        <v>0.09030000000000001</v>
-      </c>
-      <c r="F26" s="252" t="n">
-        <v>0.95</v>
+      <c r="E26" s="283" t="n">
+        <v>0</v>
+      </c>
+      <c r="F26" s="284" t="n">
+        <v>0.9</v>
       </c>
       <c r="G26" s="250">
         <f>E26*F26</f>
@@ -3861,17 +5065,17 @@
         <f>0.00275*H26*J26*K26</f>
         <v/>
       </c>
-      <c r="M26" s="109" t="n">
-        <v>0.0123</v>
-      </c>
-      <c r="N26" s="113" t="n">
+      <c r="M26" s="283" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="N26" s="285" t="n">
         <v>300</v>
       </c>
       <c r="O26" s="249">
         <f>IF(OR(N26&lt;=0,M26&lt;=0),0,((N26/4000)^(2/3)*SQRT(M26))/$S$11)</f>
         <v/>
       </c>
-      <c r="P26" s="248" t="n">
+      <c r="P26" s="286" t="n">
         <v>14.3</v>
       </c>
       <c r="Q26" s="249">
@@ -3882,18 +5086,26 @@
         <f>O26*(PI()*(N26/1000)^2/4)</f>
         <v/>
       </c>
-      <c r="S26" s="114" t="n"/>
-      <c r="T26" s="114" t="n"/>
-      <c r="U26" s="253">
-        <f>V26+(M26*P26)</f>
-        <v/>
-      </c>
-      <c r="V26" s="231">
-        <f>U27</f>
-        <v/>
-      </c>
-      <c r="W26" s="112" t="n"/>
-      <c r="X26" s="112" t="n"/>
+      <c r="S26" s="287" t="n">
+        <v>16.965</v>
+      </c>
+      <c r="T26" s="287" t="n">
+        <v>16.874</v>
+      </c>
+      <c r="U26" s="253" t="n">
+        <v>15.766</v>
+      </c>
+      <c r="V26" s="253" t="n">
+        <v>15.603</v>
+      </c>
+      <c r="W26" s="253">
+        <f>IF(OR(S26="",U26=""),"",S26-U26-N26/1000)</f>
+        <v/>
+      </c>
+      <c r="X26" s="253">
+        <f>IF(OR(T26="",V26=""),"",T26-V26-N26/1000)</f>
+        <v/>
+      </c>
       <c r="Y26" s="253">
         <f>P26*PI()*(N26/1000)^2/4</f>
         <v/>
@@ -3913,39 +5125,39 @@
     <row r="27" ht="22.5" customHeight="1" s="227">
       <c r="A27" s="107" t="inlineStr">
         <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="B27" s="107" t="inlineStr">
+        <is>
+          <t>@</t>
+        </is>
+      </c>
+      <c r="C27" s="107" t="inlineStr">
+        <is>
           <t>P11</t>
         </is>
       </c>
-      <c r="B27" s="107" t="inlineStr">
-        <is>
-          <t>@</t>
-        </is>
-      </c>
-      <c r="C27" s="107" t="inlineStr">
-        <is>
-          <t>P12</t>
-        </is>
-      </c>
       <c r="D27" s="249">
-        <f>MAX('Temps de concentration'!I7, D26+Q26)</f>
-        <v/>
-      </c>
-      <c r="E27" s="251" t="n">
-        <v>0.0498</v>
-      </c>
-      <c r="F27" s="252" t="n">
-        <v>0.335</v>
+        <f>'Temps de concentration'!K7</f>
+        <v/>
+      </c>
+      <c r="E27" s="283" t="n">
+        <v>0.09030000000000001</v>
+      </c>
+      <c r="F27" s="284" t="n">
+        <v>0.95</v>
       </c>
       <c r="G27" s="250">
         <f>E27*F27</f>
         <v/>
       </c>
       <c r="H27" s="250">
-        <f>H26+E27</f>
+        <f>E27</f>
         <v/>
       </c>
       <c r="I27" s="250">
-        <f>I26+G27</f>
+        <f>G27</f>
         <v/>
       </c>
       <c r="J27" s="253">
@@ -3960,18 +5172,18 @@
         <f>0.00275*H27*J27*K27</f>
         <v/>
       </c>
-      <c r="M27" s="251" t="n">
-        <v>0.0123</v>
-      </c>
-      <c r="N27" s="254" t="n">
+      <c r="M27" s="283" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="N27" s="285" t="n">
         <v>250</v>
       </c>
       <c r="O27" s="249">
         <f>IF(OR(N27&lt;=0,M27&lt;=0),0,((N27/4000)^(2/3)*SQRT(M27))/$S$11)</f>
         <v/>
       </c>
-      <c r="P27" s="255" t="n">
-        <v>10.9</v>
+      <c r="P27" s="286" t="n">
+        <v>12</v>
       </c>
       <c r="Q27" s="249">
         <f>IF(O27=0,0,P27/(O27*60))</f>
@@ -3981,18 +5193,26 @@
         <f>O27*(PI()*(N27/1000)^2/4)</f>
         <v/>
       </c>
-      <c r="S27" s="114" t="n"/>
-      <c r="T27" s="114" t="n"/>
-      <c r="U27" s="253">
-        <f>V27+(M27*P27)</f>
-        <v/>
-      </c>
-      <c r="V27" s="231">
-        <f>U28</f>
-        <v/>
-      </c>
-      <c r="W27" s="112" t="n"/>
-      <c r="X27" s="112" t="n"/>
+      <c r="S27" s="287" t="n">
+        <v>17.01</v>
+      </c>
+      <c r="T27" s="287" t="n">
+        <v>16.874</v>
+      </c>
+      <c r="U27" s="253" t="n">
+        <v>15.743</v>
+      </c>
+      <c r="V27" s="253" t="n">
+        <v>15.603</v>
+      </c>
+      <c r="W27" s="253">
+        <f>IF(OR(S27="",U27=""),"",S27-U27-N27/1000)</f>
+        <v/>
+      </c>
+      <c r="X27" s="253">
+        <f>IF(OR(T27="",V27=""),"",T27-V27-N27/1000)</f>
+        <v/>
+      </c>
       <c r="Y27" s="253">
         <f>P27*PI()*(N27/1000)^2/4</f>
         <v/>
@@ -4005,46 +5225,46 @@
       </c>
       <c r="AC27" s="117" t="inlineStr">
         <is>
-          <t>L11_P11_P12</t>
+          <t>LT1_T1_P11</t>
         </is>
       </c>
     </row>
     <row r="28" ht="22.5" customHeight="1" s="227">
       <c r="A28" s="107" t="inlineStr">
         <is>
+          <t>P11</t>
+        </is>
+      </c>
+      <c r="B28" s="107" t="inlineStr">
+        <is>
+          <t>@</t>
+        </is>
+      </c>
+      <c r="C28" s="107" t="inlineStr">
+        <is>
           <t>P12</t>
         </is>
       </c>
-      <c r="B28" s="107" t="inlineStr">
-        <is>
-          <t>@</t>
-        </is>
-      </c>
-      <c r="C28" s="107" t="inlineStr">
-        <is>
-          <t>PUB</t>
-        </is>
-      </c>
       <c r="D28" s="249">
-        <f>D27+Q27</f>
-        <v/>
-      </c>
-      <c r="E28" s="251" t="n">
-        <v>0</v>
-      </c>
-      <c r="F28" s="252" t="n">
-        <v>0.9</v>
+        <f>MAX('Temps de concentration'!I7, MAX(D26+Q26, D27+Q27))</f>
+        <v/>
+      </c>
+      <c r="E28" s="283" t="n">
+        <v>0.0498</v>
+      </c>
+      <c r="F28" s="284" t="n">
+        <v>0.335</v>
       </c>
       <c r="G28" s="250">
         <f>E28*F28</f>
         <v/>
       </c>
       <c r="H28" s="250">
-        <f>H27+E28</f>
+        <f>H26+H27+E28</f>
         <v/>
       </c>
       <c r="I28" s="250">
-        <f>I27+G28</f>
+        <f>I26+I27+G28</f>
         <v/>
       </c>
       <c r="J28" s="253">
@@ -4059,18 +5279,18 @@
         <f>0.00275*H28*J28*K28</f>
         <v/>
       </c>
-      <c r="M28" s="251" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="N28" s="254" t="n">
-        <v>300</v>
+      <c r="M28" s="283" t="n">
+        <v>0.0123</v>
+      </c>
+      <c r="N28" s="285" t="n">
+        <v>250</v>
       </c>
       <c r="O28" s="249">
         <f>IF(OR(N28&lt;=0,M28&lt;=0),0,((N28/4000)^(2/3)*SQRT(M28))/$S$11)</f>
         <v/>
       </c>
-      <c r="P28" s="255" t="n">
-        <v>12.4</v>
+      <c r="P28" s="286" t="n">
+        <v>10.9</v>
       </c>
       <c r="Q28" s="249">
         <f>IF(O28=0,0,P28/(O28*60))</f>
@@ -4080,17 +5300,26 @@
         <f>O28*(PI()*(N28/1000)^2/4)</f>
         <v/>
       </c>
-      <c r="S28" s="114" t="n"/>
-      <c r="T28" s="114" t="n"/>
-      <c r="U28" s="253">
-        <f>V28+(M28*P28)</f>
-        <v/>
-      </c>
-      <c r="V28" s="257" t="n">
-        <v>15.305</v>
-      </c>
-      <c r="W28" s="112" t="n"/>
-      <c r="X28" s="112" t="n"/>
+      <c r="S28" s="287" t="n">
+        <v>16.874</v>
+      </c>
+      <c r="T28" s="287" t="n">
+        <v>16.73</v>
+      </c>
+      <c r="U28" s="253" t="n">
+        <v>15.603</v>
+      </c>
+      <c r="V28" s="253" t="n">
+        <v>15.449</v>
+      </c>
+      <c r="W28" s="253">
+        <f>IF(OR(S28="",U28=""),"",S28-U28-N28/1000)</f>
+        <v/>
+      </c>
+      <c r="X28" s="253">
+        <f>IF(OR(T28="",V28=""),"",T28-V28-N28/1000)</f>
+        <v/>
+      </c>
       <c r="Y28" s="253">
         <f>P28*PI()*(N28/1000)^2/4</f>
         <v/>
@@ -4103,48 +5332,121 @@
       </c>
       <c r="AC28" s="117" t="inlineStr">
         <is>
-          <t>L12_P12_PUB</t>
+          <t>L11_P11_P12</t>
         </is>
       </c>
     </row>
     <row r="29" ht="22.5" customHeight="1" s="227">
-      <c r="A29" s="128" t="inlineStr">
-        <is>
-          <t>INSTRUCTIONS / HYPOTHÈSES</t>
-        </is>
-      </c>
-      <c r="B29" s="119" t="n"/>
-      <c r="C29" s="120" t="n"/>
-      <c r="D29" s="258" t="n"/>
-      <c r="E29" s="122" t="n"/>
-      <c r="F29" s="100" t="n"/>
-      <c r="G29" s="122" t="n"/>
-      <c r="H29" s="122" t="n"/>
-      <c r="I29" s="122" t="n"/>
-      <c r="J29" s="100" t="n"/>
-      <c r="K29" s="100" t="n"/>
-      <c r="L29" s="123" t="n"/>
-      <c r="M29" s="124" t="n"/>
-      <c r="N29" s="94" t="n"/>
-      <c r="O29" s="125" t="n"/>
-      <c r="P29" s="258" t="n"/>
-      <c r="Q29" s="100" t="n"/>
-      <c r="R29" s="123" t="n"/>
-      <c r="S29" s="100" t="n"/>
-      <c r="T29" s="100" t="n"/>
-      <c r="U29" s="95" t="n"/>
-      <c r="V29" s="126" t="n"/>
-      <c r="W29" s="105" t="n"/>
-      <c r="X29" s="95" t="n"/>
-      <c r="Y29" s="95" t="n"/>
+      <c r="A29" s="107" t="inlineStr">
+        <is>
+          <t>P12</t>
+        </is>
+      </c>
+      <c r="B29" s="107" t="inlineStr">
+        <is>
+          <t>@</t>
+        </is>
+      </c>
+      <c r="C29" s="107" t="inlineStr">
+        <is>
+          <t>PUB</t>
+        </is>
+      </c>
+      <c r="D29" s="249">
+        <f>D28+Q28</f>
+        <v/>
+      </c>
+      <c r="E29" s="283" t="n">
+        <v>0</v>
+      </c>
+      <c r="F29" s="284" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="G29" s="250">
+        <f>E29*F29</f>
+        <v/>
+      </c>
+      <c r="H29" s="250">
+        <f>H28+E29</f>
+        <v/>
+      </c>
+      <c r="I29" s="250">
+        <f>I28+G29</f>
+        <v/>
+      </c>
+      <c r="J29" s="253">
+        <f>IF(H29=0,0,I29/H29)</f>
+        <v/>
+      </c>
+      <c r="K29" s="249">
+        <f>IF($S$2=0.5,$R$5/((D29+$S$5)^$T$5),IF($S$2=0.2,$R$6/((D29+$S$6)^$T$6),IF($S$2=0.1,$R$7/((D29+$S$7)^$T$7),IF($S$2=0.04,$R$8/((D29+$S$8)^$T$8),IF($S$2=0.02,$R$9/((D29+$S$9)^$T$9),$R$10/((D29+$S$10)^$T$10))))))</f>
+        <v/>
+      </c>
+      <c r="L29" s="253">
+        <f>0.00275*H29*J29*K29</f>
+        <v/>
+      </c>
+      <c r="M29" s="283" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="N29" s="285" t="n">
+        <v>300</v>
+      </c>
+      <c r="O29" s="249">
+        <f>IF(OR(N29&lt;=0,M29&lt;=0),0,((N29/4000)^(2/3)*SQRT(M29))/$S$11)</f>
+        <v/>
+      </c>
+      <c r="P29" s="286" t="n">
+        <v>12.4</v>
+      </c>
+      <c r="Q29" s="249">
+        <f>IF(O29=0,0,P29/(O29*60))</f>
+        <v/>
+      </c>
+      <c r="R29" s="253">
+        <f>O29*(PI()*(N29/1000)^2/4)</f>
+        <v/>
+      </c>
+      <c r="S29" s="287" t="n">
+        <v>16.73</v>
+      </c>
+      <c r="T29" s="287" t="n">
+        <v>16.73</v>
+      </c>
+      <c r="U29" s="253" t="n">
+        <v>15.449</v>
+      </c>
+      <c r="V29" s="253" t="n">
+        <v>15.305</v>
+      </c>
+      <c r="W29" s="253">
+        <f>IF(OR(S29="",U29=""),"",S29-U29-N29/1000)</f>
+        <v/>
+      </c>
+      <c r="X29" s="253">
+        <f>IF(OR(T29="",V29=""),"",T29-V29-N29/1000)</f>
+        <v/>
+      </c>
+      <c r="Y29" s="253">
+        <f>P29*PI()*(N29/1000)^2/4</f>
+        <v/>
+      </c>
       <c r="Z29" s="95" t="n"/>
       <c r="AA29" s="115" t="n"/>
-      <c r="AB29" s="127" t="n"/>
+      <c r="AB29" s="256">
+        <f>IF(R29&gt;L29,"OK","AUGMENTER D")</f>
+        <v/>
+      </c>
+      <c r="AC29" s="117" t="inlineStr">
+        <is>
+          <t>L12_P12_PUB</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="22.5" customHeight="1" s="227">
-      <c r="A30" s="208" t="inlineStr">
-        <is>
-          <t>Jaune = saisie; Vert = calculé automatiquement (Station Saint-Hubert).</t>
+      <c r="A30" s="297" t="inlineStr">
+        <is>
+          <t>INSTRUCTIONS / HYPOTHÈSES</t>
         </is>
       </c>
       <c r="B30" s="259" t="n"/>
@@ -4176,9 +5478,9 @@
       <c r="AB30" s="127" t="n"/>
     </row>
     <row r="31" ht="22.5" customHeight="1" s="227">
-      <c r="A31" s="207" t="inlineStr">
-        <is>
-          <t>Source données: Reseau_pluvial_dimensionnement_v1.xlsx (CB_plan aires, Conduites longueurs/topologie, Noeuds élévations, Inputs IDF/n/pente).</t>
+      <c r="A31" s="208" t="inlineStr">
+        <is>
+          <t>Jaune = saisie; Vert = calculé.</t>
         </is>
       </c>
       <c r="B31" s="259" t="n"/>
@@ -4210,9 +5512,9 @@
       <c r="AB31" s="127" t="n"/>
     </row>
     <row r="32" ht="22.5" customHeight="1" s="227">
-      <c r="A32" s="208" t="inlineStr">
-        <is>
-          <t>Qmax = 0.00275 × A(ha) × R × I   |   I = A/(tc+B)^C selon période S2 (défaut 1/10 ans).</t>
+      <c r="A32" s="207" t="inlineStr">
+        <is>
+          <t>Radiers (U/V): calés depuis exutoire PUB=15.305 m; pente radier = max(s conduite, 1%); chute regard=0.02 m.</t>
         </is>
       </c>
       <c r="B32" s="259" t="n"/>
@@ -4244,9 +5546,9 @@
       <c r="AB32" s="127" t="n"/>
     </row>
     <row r="33" ht="22.5" customHeight="1" s="227">
-      <c r="A33" s="207" t="inlineStr">
-        <is>
-          <t>v et Qp = Manning pleine section; n = S11 (0.013). Diamètre N est une suggestion — ajuster si AB = AUGMENTER D.</t>
+      <c r="A33" s="208" t="inlineStr">
+        <is>
+          <t>Confluences P06, J01, P11: si plusieurs branches imposent un radier, on retient le PLUS BAS (MIN). Voir onglet Radiers.</t>
         </is>
       </c>
       <c r="B33" s="259" t="n"/>
@@ -4260,7 +5562,7 @@
       <c r="J33" s="259" t="n"/>
       <c r="K33" s="259" t="n"/>
       <c r="L33" s="260" t="n"/>
-      <c r="M33" s="129" t="n"/>
+      <c r="M33" s="124" t="n"/>
       <c r="N33" s="94" t="n"/>
       <c r="O33" s="125" t="n"/>
       <c r="P33" s="258" t="n"/>
@@ -4268,85 +5570,121 @@
       <c r="R33" s="123" t="n"/>
       <c r="S33" s="100" t="n"/>
       <c r="T33" s="100" t="n"/>
-      <c r="U33" s="100" t="n"/>
+      <c r="U33" s="95" t="n"/>
       <c r="V33" s="126" t="n"/>
       <c r="W33" s="105" t="n"/>
       <c r="X33" s="95" t="n"/>
       <c r="Y33" s="95" t="n"/>
       <c r="Z33" s="95" t="n"/>
       <c r="AA33" s="115" t="n"/>
-      <c r="AC33" s="127" t="n"/>
+      <c r="AB33" s="127" t="n"/>
     </row>
     <row r="34" ht="22.5" customHeight="1" s="227">
-      <c r="A34" s="209" t="inlineStr">
-        <is>
-          <t>tc: temps d’entrée (Temps de concentration) puis cumul + temps de parcours Q=L/(v*60).</t>
-        </is>
-      </c>
-      <c r="B34" s="244" t="n"/>
-      <c r="C34" s="244" t="n"/>
-      <c r="D34" s="244" t="n"/>
-      <c r="E34" s="244" t="n"/>
-      <c r="F34" s="244" t="n"/>
-      <c r="G34" s="244" t="n"/>
-      <c r="H34" s="244" t="n"/>
-      <c r="I34" s="244" t="n"/>
-      <c r="J34" s="244" t="n"/>
-      <c r="K34" s="244" t="n"/>
-      <c r="L34" s="245" t="n"/>
-      <c r="M34" s="130" t="n"/>
-      <c r="N34" s="80" t="n"/>
-      <c r="O34" s="88" t="n"/>
-      <c r="P34" s="261" t="n"/>
-      <c r="Q34" s="81" t="n"/>
-      <c r="R34" s="132" t="n"/>
-      <c r="S34" s="81" t="n"/>
-      <c r="T34" s="81" t="n"/>
-      <c r="U34" s="81" t="n"/>
-      <c r="V34" s="133" t="n"/>
-      <c r="W34" s="134" t="n"/>
-      <c r="X34" s="135" t="n"/>
-      <c r="Y34" s="135" t="n"/>
-      <c r="Z34" s="135" t="n"/>
-      <c r="AA34" s="136" t="n"/>
+      <c r="A34" s="207" t="inlineStr">
+        <is>
+          <t>T1 = noeud toiture (zone N, 903 m², C=0.95) raccordé à P11. Longueur LT1 jaune (défaut 12 m) — ajuster puis redemander recalcul radiers si changée.</t>
+        </is>
+      </c>
+      <c r="B34" s="259" t="n"/>
+      <c r="C34" s="259" t="n"/>
+      <c r="D34" s="259" t="n"/>
+      <c r="E34" s="259" t="n"/>
+      <c r="F34" s="259" t="n"/>
+      <c r="G34" s="259" t="n"/>
+      <c r="H34" s="259" t="n"/>
+      <c r="I34" s="259" t="n"/>
+      <c r="J34" s="259" t="n"/>
+      <c r="K34" s="259" t="n"/>
+      <c r="L34" s="260" t="n"/>
+      <c r="M34" s="129" t="n"/>
+      <c r="N34" s="94" t="n"/>
+      <c r="O34" s="125" t="n"/>
+      <c r="P34" s="258" t="n"/>
+      <c r="Q34" s="100" t="n"/>
+      <c r="R34" s="123" t="n"/>
+      <c r="S34" s="100" t="n"/>
+      <c r="T34" s="100" t="n"/>
+      <c r="U34" s="100" t="n"/>
+      <c r="V34" s="126" t="n"/>
+      <c r="W34" s="105" t="n"/>
+      <c r="X34" s="95" t="n"/>
+      <c r="Y34" s="95" t="n"/>
+      <c r="Z34" s="95" t="n"/>
+      <c r="AA34" s="115" t="n"/>
       <c r="AC34" s="127" t="n"/>
     </row>
     <row r="35" ht="15" customHeight="1" s="227">
-      <c r="A35" s="206" t="inlineStr">
-        <is>
-          <t>Radiers: calés depuis exutoire invert 15.305 m (Inputs), pente min 1%, chute regard 0.02 m.</t>
-        </is>
-      </c>
+      <c r="A35" s="209" t="inlineStr">
+        <is>
+          <t>H/I: branches L07, L12, LT1 en DA locale; fusion à P06, J01 et P11.</t>
+        </is>
+      </c>
+      <c r="B35" s="244" t="n"/>
+      <c r="C35" s="244" t="n"/>
+      <c r="D35" s="244" t="n"/>
+      <c r="E35" s="244" t="n"/>
+      <c r="F35" s="244" t="n"/>
+      <c r="G35" s="244" t="n"/>
+      <c r="H35" s="244" t="n"/>
+      <c r="I35" s="244" t="n"/>
+      <c r="J35" s="244" t="n"/>
+      <c r="K35" s="244" t="n"/>
+      <c r="L35" s="245" t="n"/>
+      <c r="M35" s="130" t="n"/>
+      <c r="N35" s="80" t="n"/>
+      <c r="O35" s="88" t="n"/>
+      <c r="P35" s="261" t="n"/>
+      <c r="Q35" s="81" t="n"/>
+      <c r="R35" s="132" t="n"/>
+      <c r="S35" s="81" t="n"/>
+      <c r="T35" s="81" t="n"/>
+      <c r="U35" s="81" t="n"/>
+      <c r="V35" s="133" t="n"/>
+      <c r="W35" s="134" t="n"/>
+      <c r="X35" s="135" t="n"/>
+      <c r="Y35" s="135" t="n"/>
+      <c r="Z35" s="135" t="n"/>
+      <c r="AA35" s="136" t="n"/>
+      <c r="AC35" s="127" t="n"/>
     </row>
     <row r="36" ht="15" customHeight="1" s="227">
       <c r="A36" s="206" t="inlineStr">
         <is>
-          <t>Changer la période: modifier S2. H/I à J01 corrigé: branche P02→J01 = DA locale; fusion dans J01→RP03.</t>
-        </is>
-      </c>
-      <c r="P36" s="203" t="n"/>
-      <c r="Q36" s="206" t="inlineStr">
-        <is>
-          <t>Longueurs à compléter/valider par tech.</t>
+          <t>Radiers: calés depuis exutoire invert 15.305 m (Inputs), pente min 1%, chute regard 0.02 m.</t>
         </is>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1" s="227">
       <c r="A37" s="206" t="inlineStr">
         <is>
+          <t>Changer la période: modifier S2. H/I à J01 corrigé: branche P02→J01 = DA locale; fusion dans J01→RP03.</t>
+        </is>
+      </c>
+      <c r="P37" s="203" t="n"/>
+      <c r="Q37" s="206" t="inlineStr">
+        <is>
+          <t>Longueurs à compléter/valider par tech.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="206" t="inlineStr">
+        <is>
           <t>Cette feuille garde la logique simple demandée; le classeur v1 reste la référence détaillée.</t>
         </is>
       </c>
     </row>
-    <row r="81" ht="15" customHeight="1" s="227">
-      <c r="F81" s="206" t="inlineStr">
+    <row r="81" ht="15" customHeight="1" s="227"/>
+    <row r="82">
+      <c r="F82" s="206" t="inlineStr">
         <is>
           <t>*</t>
         </is>
       </c>
     </row>
-    <row r="173" ht="15" customHeight="1" s="227">
-      <c r="F173" s="206" t="inlineStr">
+    <row r="173" ht="15" customHeight="1" s="227"/>
+    <row r="174">
+      <c r="F174" s="206" t="inlineStr">
         <is>
           <t>,0,</t>
         </is>
@@ -4395,7 +5733,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4518,7 +5856,11 @@
         </is>
       </c>
       <c r="J5" s="143" t="n"/>
-      <c r="K5" s="143" t="n"/>
+      <c r="K5" s="143" t="inlineStr">
+        <is>
+          <t>LT1</t>
+        </is>
+      </c>
       <c r="L5" s="143" t="n"/>
       <c r="M5" s="144" t="n"/>
       <c r="N5" s="145" t="n"/>
@@ -4585,7 +5927,9 @@
         <v>0.049761</v>
       </c>
       <c r="J6" s="151" t="n"/>
-      <c r="K6" s="151" t="n"/>
+      <c r="K6" s="288" t="n">
+        <v>0.09030000000000001</v>
+      </c>
       <c r="L6" s="152" t="n"/>
       <c r="M6" s="153" t="n"/>
       <c r="N6" s="139" t="n"/>
@@ -4652,7 +5996,10 @@
         <v/>
       </c>
       <c r="J7" s="263" t="n"/>
-      <c r="K7" s="263" t="n"/>
+      <c r="K7" s="289">
+        <f>((2.187*K10*K11)/(K12)^0.5)^0.467</f>
+        <v/>
+      </c>
       <c r="L7" s="263" t="n"/>
       <c r="M7" s="264" t="n"/>
       <c r="N7" s="265" t="n"/>
@@ -4715,7 +6062,9 @@
         <v>0.335</v>
       </c>
       <c r="J8" s="170" t="n"/>
-      <c r="K8" s="170" t="n"/>
+      <c r="K8" s="290" t="n">
+        <v>0.95</v>
+      </c>
       <c r="L8" s="170" t="n"/>
       <c r="M8" s="171" t="n"/>
       <c r="N8" s="139" t="n"/>
@@ -4813,7 +6162,9 @@
         <v>22.3</v>
       </c>
       <c r="J10" s="270" t="n"/>
-      <c r="K10" s="270" t="n"/>
+      <c r="K10" s="291" t="n">
+        <v>30</v>
+      </c>
       <c r="L10" s="270" t="n"/>
       <c r="M10" s="271" t="n"/>
       <c r="N10" s="265" t="n"/>
@@ -4872,7 +6223,9 @@
         <v>0.02</v>
       </c>
       <c r="J11" s="181" t="n"/>
-      <c r="K11" s="181" t="n"/>
+      <c r="K11" s="292" t="n">
+        <v>0.02</v>
+      </c>
       <c r="L11" s="181" t="n"/>
       <c r="M11" s="182" t="n"/>
       <c r="N11" s="139" t="n"/>
@@ -4931,7 +6284,9 @@
         <v>0.01231</v>
       </c>
       <c r="J12" s="186" t="n"/>
-      <c r="K12" s="187" t="n"/>
+      <c r="K12" s="293" t="n">
+        <v>0.01</v>
+      </c>
       <c r="L12" s="170" t="n"/>
       <c r="M12" s="188" t="n"/>
       <c r="N12" s="189" t="n"/>
@@ -5015,6 +6370,28 @@
         <is>
           <t>Jaune = saisie (depuis Reseau_pluvial_dimensionnement_v1). Vert = calculé.</t>
         </is>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>LT1</t>
+        </is>
+      </c>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>N (toit → P11)</t>
+        </is>
+      </c>
+      <c r="Q15" t="n">
+        <v>903</v>
+      </c>
+      <c r="R15" t="n">
+        <v>857.85</v>
+      </c>
+      <c r="S15" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="T15" t="n">
+        <v>0.09030000000000001</v>
       </c>
     </row>
     <row r="16" ht="15" customHeight="1" s="227">
@@ -7074,14 +8451,14 @@
     <row r="117" ht="15" customHeight="1" s="227">
       <c r="A117" s="225" t="inlineStr">
         <is>
-          <t>Examples</t>
+          <t>LT1_T1_P11 (toiture zone N): A=903 m², C=0.95; se raccorde à P11. Radiers: MIN aux confluences.</t>
         </is>
       </c>
     </row>
     <row r="118" ht="15" customHeight="1" s="227">
       <c r="A118" s="200" t="inlineStr">
         <is>
-          <t>Pipe</t>
+          <t>P10→P11: DA locale=0 (toit déplacé vers T1). Fusion H à P11 = H(P10)+H(T1)+DA(P11).</t>
         </is>
       </c>
       <c r="B118" s="200" t="inlineStr">

</xml_diff>

<commit_message>
Make network radiers fully dynamic from pipe L and slope
Link U/V to Radiers formulas so invert updates when length or slope
changes; apply MIN branch info at confluences; set P09-P06 s=0.01
and P11-P12 / P12-PUB s=0.015.

Co-authored-by: acon560-prog <acon560-prog@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/engineering/drainage-design/Dimensionnement_reseau_pluvial_ADAPTE_methode_simple OLIVIER TECH. MODIF.xlsx
+++ b/engineering/drainage-design/Dimensionnement_reseau_pluvial_ADAPTE_methode_simple OLIVIER TECH. MODIF.xlsx
@@ -29,7 +29,7 @@
     <numFmt numFmtId="168" formatCode="0.0000"/>
     <numFmt numFmtId="169" formatCode="0.00000"/>
   </numFmts>
-  <fonts count="24">
+  <fonts count="26">
     <font>
       <name val="Times New Roman"/>
       <charset val="1"/>
@@ -183,8 +183,18 @@
       <color rgb="00C00000"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001F4E79"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="19">
+  <fills count="20">
     <fill>
       <patternFill/>
     </fill>
@@ -288,6 +298,11 @@
         <fgColor rgb="00FCE4D6"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DDEBF7"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="66">
     <border>
@@ -1110,7 +1125,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="298">
+  <cellXfs count="303">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
@@ -1862,6 +1877,11 @@
     <xf numFmtId="0" fontId="15" fillId="0" borderId="48" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="0" fillId="19" borderId="65" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="0" fillId="18" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2315,999 +2335,1555 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J42"/>
+  <dimension ref="A1:J65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" style="227" min="1" max="1"/>
-    <col width="10" customWidth="1" style="227" min="2" max="2"/>
-    <col width="10" customWidth="1" style="227" min="3" max="3"/>
-    <col width="10" customWidth="1" style="227" min="4" max="4"/>
-    <col width="12" customWidth="1" style="227" min="5" max="5"/>
-    <col width="16" customWidth="1" style="227" min="6" max="6"/>
+    <col width="14" customWidth="1" style="227" min="1" max="1"/>
+    <col width="14" customWidth="1" style="227" min="2" max="2"/>
+    <col width="12" customWidth="1" style="227" min="3" max="3"/>
+    <col width="18" customWidth="1" style="227" min="4" max="4"/>
+    <col width="28" customWidth="1" style="227" min="5" max="5"/>
+    <col width="14" customWidth="1" style="227" min="6" max="6"/>
     <col width="14" customWidth="1" style="227" min="7" max="7"/>
     <col width="12" customWidth="1" style="227" min="8" max="8"/>
     <col width="12" customWidth="1" style="227" min="9" max="9"/>
-    <col width="16" customWidth="1" style="227" min="10" max="10"/>
+    <col width="28" customWidth="1" style="227" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="272" t="inlineStr">
-        <is>
-          <t>RADIERS (invert elevations) — règle MIN aux confluences</t>
+      <c r="A1" s="298" t="inlineStr">
+        <is>
+          <t>RADIERS DYNAMIQUES — changez L ou s dans Calcul_reseau; les inverts se mettent à jour</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Exutoire PUB fixe = 15.305 m. Remontée: Inv_amont = Inv_aval + max(s,1%)*L + chute 0.02 m.</t>
+          <t>Formules Excel (pas de recalcul manuel). Aux confluences: radier du noeud = MIN des propositions des branches.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Si plusieurs branches proposent un radier au même noeud → on garde le PLUS BAS.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="294" t="inlineStr">
-        <is>
-          <t>Règle confluences (P06, J01, P11): toutes les branches amont se calent sur le radier du noeud fixé depuis l’aval; si plusieurs contraintes, retenir le PLUS BAS.</t>
+          <t>Dynamique: Inv amont = Inv aval + MAX(s,smin)·L + chute. Aux confluences le radier du noeud suit l’AVAL (drainable). Colonne D = MIN des arrivées des branches (couverture) pour choisir/contrôler.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="273" t="inlineStr">
         <is>
-          <t>Paramètres</t>
+          <t>PARAMÈTRES (jaune = modifiable)</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Invert PUB (m)</t>
-        </is>
-      </c>
-      <c r="B6" s="274" t="n">
+      <c r="A6" s="276" t="inlineStr">
+        <is>
+          <t>Invert PUB / exutoire (m)</t>
+        </is>
+      </c>
+      <c r="B6" s="279" t="n">
         <v>15.305</v>
       </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Les longueurs L et pentes s sont lues dans Calcul_reseau (colonnes P et M).</t>
+        </is>
+      </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Chute regard (m)</t>
-        </is>
-      </c>
-      <c r="B7" s="274" t="n">
+      <c r="A7" s="276" t="inlineStr">
+        <is>
+          <t>Chute de regard (m)</t>
+        </is>
+      </c>
+      <c r="B7" s="279" t="n">
         <v>0.02</v>
       </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Changez M18=0.01, M28=0.015, M29=0.015 déjà appliqué; vous pouvez les modifier encore.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Pente min radier</t>
-        </is>
-      </c>
-      <c r="B8" s="274" t="n">
+      <c r="A8" s="276" t="inlineStr">
+        <is>
+          <t>Pente min radier smin (m/m)</t>
+        </is>
+      </c>
+      <c r="B8" s="279" t="n">
         <v>0.01</v>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="275" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="276" t="inlineStr">
+        <is>
+          <t>Couverture mini pour proposition amont (m)</t>
+        </is>
+      </c>
+      <c r="B9" s="279" t="n">
+        <v>1.8</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="273" t="inlineStr">
+        <is>
+          <t>TABLE DES CONDUITES (liée à Calcul_reseau)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="275" t="inlineStr">
+        <is>
+          <t>Row</t>
+        </is>
+      </c>
+      <c r="B12" s="275" t="inlineStr">
+        <is>
+          <t>Pipe_ID</t>
+        </is>
+      </c>
+      <c r="C12" s="275" t="inlineStr">
+        <is>
+          <t>De</t>
+        </is>
+      </c>
+      <c r="D12" s="275" t="inlineStr">
+        <is>
+          <t>Vers</t>
+        </is>
+      </c>
+      <c r="E12" s="275" t="inlineStr">
+        <is>
+          <t>L (m)</t>
+        </is>
+      </c>
+      <c r="F12" s="275" t="inlineStr">
+        <is>
+          <t>s design</t>
+        </is>
+      </c>
+      <c r="G12" s="275" t="inlineStr">
+        <is>
+          <t>s utilisée</t>
+        </is>
+      </c>
+      <c r="H12" s="275" t="inlineStr">
+        <is>
+          <t>D (m)</t>
+        </is>
+      </c>
+      <c r="I12" s="275" t="inlineStr">
+        <is>
+          <t>Sol amont</t>
+        </is>
+      </c>
+      <c r="J12" s="275" t="inlineStr">
+        <is>
+          <t>Proposition amont (couverture)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="276" t="n">
+        <v>18</v>
+      </c>
+      <c r="B13" s="276">
+        <f>Calcul_reseau!AC18</f>
+        <v/>
+      </c>
+      <c r="C13" s="276">
+        <f>Calcul_reseau!A18</f>
+        <v/>
+      </c>
+      <c r="D13" s="276">
+        <f>Calcul_reseau!C18</f>
+        <v/>
+      </c>
+      <c r="E13" s="277">
+        <f>Calcul_reseau!P18</f>
+        <v/>
+      </c>
+      <c r="F13" s="281">
+        <f>Calcul_reseau!M18</f>
+        <v/>
+      </c>
+      <c r="G13" s="281">
+        <f>MAX(F13,$B$8)</f>
+        <v/>
+      </c>
+      <c r="H13" s="277">
+        <f>IF(Calcul_reseau!N18="",0,Calcul_reseau!N18/1000)</f>
+        <v/>
+      </c>
+      <c r="I13" s="278">
+        <f>Calcul_reseau!S18</f>
+        <v/>
+      </c>
+      <c r="J13" s="299">
+        <f>IF(OR(I13="",H13=0),"",I13-$B$9-H13)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="276" t="n">
+        <v>19</v>
+      </c>
+      <c r="B14" s="276">
+        <f>Calcul_reseau!AC19</f>
+        <v/>
+      </c>
+      <c r="C14" s="276">
+        <f>Calcul_reseau!A19</f>
+        <v/>
+      </c>
+      <c r="D14" s="276">
+        <f>Calcul_reseau!C19</f>
+        <v/>
+      </c>
+      <c r="E14" s="277">
+        <f>Calcul_reseau!P19</f>
+        <v/>
+      </c>
+      <c r="F14" s="281">
+        <f>Calcul_reseau!M19</f>
+        <v/>
+      </c>
+      <c r="G14" s="281">
+        <f>MAX(F14,$B$8)</f>
+        <v/>
+      </c>
+      <c r="H14" s="277">
+        <f>IF(Calcul_reseau!N19="",0,Calcul_reseau!N19/1000)</f>
+        <v/>
+      </c>
+      <c r="I14" s="278">
+        <f>Calcul_reseau!S19</f>
+        <v/>
+      </c>
+      <c r="J14" s="299">
+        <f>IF(OR(I14="",H14=0),"",I14-$B$9-H14)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="276" t="n">
+        <v>20</v>
+      </c>
+      <c r="B15" s="276">
+        <f>Calcul_reseau!AC20</f>
+        <v/>
+      </c>
+      <c r="C15" s="276">
+        <f>Calcul_reseau!A20</f>
+        <v/>
+      </c>
+      <c r="D15" s="276">
+        <f>Calcul_reseau!C20</f>
+        <v/>
+      </c>
+      <c r="E15" s="277">
+        <f>Calcul_reseau!P20</f>
+        <v/>
+      </c>
+      <c r="F15" s="281">
+        <f>Calcul_reseau!M20</f>
+        <v/>
+      </c>
+      <c r="G15" s="281">
+        <f>MAX(F15,$B$8)</f>
+        <v/>
+      </c>
+      <c r="H15" s="277">
+        <f>IF(Calcul_reseau!N20="",0,Calcul_reseau!N20/1000)</f>
+        <v/>
+      </c>
+      <c r="I15" s="278">
+        <f>Calcul_reseau!S20</f>
+        <v/>
+      </c>
+      <c r="J15" s="299">
+        <f>IF(OR(I15="",H15=0),"",I15-$B$9-H15)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="276" t="n">
+        <v>21</v>
+      </c>
+      <c r="B16" s="276">
+        <f>Calcul_reseau!AC21</f>
+        <v/>
+      </c>
+      <c r="C16" s="276">
+        <f>Calcul_reseau!A21</f>
+        <v/>
+      </c>
+      <c r="D16" s="276">
+        <f>Calcul_reseau!C21</f>
+        <v/>
+      </c>
+      <c r="E16" s="277">
+        <f>Calcul_reseau!P21</f>
+        <v/>
+      </c>
+      <c r="F16" s="281">
+        <f>Calcul_reseau!M21</f>
+        <v/>
+      </c>
+      <c r="G16" s="281">
+        <f>MAX(F16,$B$8)</f>
+        <v/>
+      </c>
+      <c r="H16" s="277">
+        <f>IF(Calcul_reseau!N21="",0,Calcul_reseau!N21/1000)</f>
+        <v/>
+      </c>
+      <c r="I16" s="278">
+        <f>Calcul_reseau!S21</f>
+        <v/>
+      </c>
+      <c r="J16" s="299">
+        <f>IF(OR(I16="",H16=0),"",I16-$B$9-H16)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="276" t="n">
+        <v>22</v>
+      </c>
+      <c r="B17" s="276">
+        <f>Calcul_reseau!AC22</f>
+        <v/>
+      </c>
+      <c r="C17" s="276">
+        <f>Calcul_reseau!A22</f>
+        <v/>
+      </c>
+      <c r="D17" s="276">
+        <f>Calcul_reseau!C22</f>
+        <v/>
+      </c>
+      <c r="E17" s="277">
+        <f>Calcul_reseau!P22</f>
+        <v/>
+      </c>
+      <c r="F17" s="281">
+        <f>Calcul_reseau!M22</f>
+        <v/>
+      </c>
+      <c r="G17" s="281">
+        <f>MAX(F17,$B$8)</f>
+        <v/>
+      </c>
+      <c r="H17" s="277">
+        <f>IF(Calcul_reseau!N22="",0,Calcul_reseau!N22/1000)</f>
+        <v/>
+      </c>
+      <c r="I17" s="278">
+        <f>Calcul_reseau!S22</f>
+        <v/>
+      </c>
+      <c r="J17" s="299">
+        <f>IF(OR(I17="",H17=0),"",I17-$B$9-H17)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="276" t="n">
+        <v>23</v>
+      </c>
+      <c r="B18" s="276">
+        <f>Calcul_reseau!AC23</f>
+        <v/>
+      </c>
+      <c r="C18" s="276">
+        <f>Calcul_reseau!A23</f>
+        <v/>
+      </c>
+      <c r="D18" s="276">
+        <f>Calcul_reseau!C23</f>
+        <v/>
+      </c>
+      <c r="E18" s="277">
+        <f>Calcul_reseau!P23</f>
+        <v/>
+      </c>
+      <c r="F18" s="281">
+        <f>Calcul_reseau!M23</f>
+        <v/>
+      </c>
+      <c r="G18" s="281">
+        <f>MAX(F18,$B$8)</f>
+        <v/>
+      </c>
+      <c r="H18" s="277">
+        <f>IF(Calcul_reseau!N23="",0,Calcul_reseau!N23/1000)</f>
+        <v/>
+      </c>
+      <c r="I18" s="278">
+        <f>Calcul_reseau!S23</f>
+        <v/>
+      </c>
+      <c r="J18" s="299">
+        <f>IF(OR(I18="",H18=0),"",I18-$B$9-H18)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="276" t="n">
+        <v>24</v>
+      </c>
+      <c r="B19" s="276">
+        <f>Calcul_reseau!AC24</f>
+        <v/>
+      </c>
+      <c r="C19" s="276">
+        <f>Calcul_reseau!A24</f>
+        <v/>
+      </c>
+      <c r="D19" s="276">
+        <f>Calcul_reseau!C24</f>
+        <v/>
+      </c>
+      <c r="E19" s="277">
+        <f>Calcul_reseau!P24</f>
+        <v/>
+      </c>
+      <c r="F19" s="281">
+        <f>Calcul_reseau!M24</f>
+        <v/>
+      </c>
+      <c r="G19" s="281">
+        <f>MAX(F19,$B$8)</f>
+        <v/>
+      </c>
+      <c r="H19" s="277">
+        <f>IF(Calcul_reseau!N24="",0,Calcul_reseau!N24/1000)</f>
+        <v/>
+      </c>
+      <c r="I19" s="278">
+        <f>Calcul_reseau!S24</f>
+        <v/>
+      </c>
+      <c r="J19" s="299">
+        <f>IF(OR(I19="",H19=0),"",I19-$B$9-H19)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="276" t="n">
+        <v>25</v>
+      </c>
+      <c r="B20" s="276">
+        <f>Calcul_reseau!AC25</f>
+        <v/>
+      </c>
+      <c r="C20" s="276">
+        <f>Calcul_reseau!A25</f>
+        <v/>
+      </c>
+      <c r="D20" s="276">
+        <f>Calcul_reseau!C25</f>
+        <v/>
+      </c>
+      <c r="E20" s="277">
+        <f>Calcul_reseau!P25</f>
+        <v/>
+      </c>
+      <c r="F20" s="281">
+        <f>Calcul_reseau!M25</f>
+        <v/>
+      </c>
+      <c r="G20" s="281">
+        <f>MAX(F20,$B$8)</f>
+        <v/>
+      </c>
+      <c r="H20" s="277">
+        <f>IF(Calcul_reseau!N25="",0,Calcul_reseau!N25/1000)</f>
+        <v/>
+      </c>
+      <c r="I20" s="278">
+        <f>Calcul_reseau!S25</f>
+        <v/>
+      </c>
+      <c r="J20" s="299">
+        <f>IF(OR(I20="",H20=0),"",I20-$B$9-H20)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="276" t="n">
+        <v>26</v>
+      </c>
+      <c r="B21" s="276">
+        <f>Calcul_reseau!AC26</f>
+        <v/>
+      </c>
+      <c r="C21" s="276">
+        <f>Calcul_reseau!A26</f>
+        <v/>
+      </c>
+      <c r="D21" s="276">
+        <f>Calcul_reseau!C26</f>
+        <v/>
+      </c>
+      <c r="E21" s="277">
+        <f>Calcul_reseau!P26</f>
+        <v/>
+      </c>
+      <c r="F21" s="281">
+        <f>Calcul_reseau!M26</f>
+        <v/>
+      </c>
+      <c r="G21" s="281">
+        <f>MAX(F21,$B$8)</f>
+        <v/>
+      </c>
+      <c r="H21" s="277">
+        <f>IF(Calcul_reseau!N26="",0,Calcul_reseau!N26/1000)</f>
+        <v/>
+      </c>
+      <c r="I21" s="278">
+        <f>Calcul_reseau!S26</f>
+        <v/>
+      </c>
+      <c r="J21" s="299">
+        <f>IF(OR(I21="",H21=0),"",I21-$B$9-H21)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="276" t="n">
+        <v>27</v>
+      </c>
+      <c r="B22" s="276">
+        <f>Calcul_reseau!AC27</f>
+        <v/>
+      </c>
+      <c r="C22" s="276">
+        <f>Calcul_reseau!A27</f>
+        <v/>
+      </c>
+      <c r="D22" s="276">
+        <f>Calcul_reseau!C27</f>
+        <v/>
+      </c>
+      <c r="E22" s="277">
+        <f>Calcul_reseau!P27</f>
+        <v/>
+      </c>
+      <c r="F22" s="281">
+        <f>Calcul_reseau!M27</f>
+        <v/>
+      </c>
+      <c r="G22" s="281">
+        <f>MAX(F22,$B$8)</f>
+        <v/>
+      </c>
+      <c r="H22" s="277">
+        <f>IF(Calcul_reseau!N27="",0,Calcul_reseau!N27/1000)</f>
+        <v/>
+      </c>
+      <c r="I22" s="278">
+        <f>Calcul_reseau!S27</f>
+        <v/>
+      </c>
+      <c r="J22" s="299">
+        <f>IF(OR(I22="",H22=0),"",I22-$B$9-H22)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="276" t="n">
+        <v>28</v>
+      </c>
+      <c r="B23" s="276">
+        <f>Calcul_reseau!AC28</f>
+        <v/>
+      </c>
+      <c r="C23" s="276">
+        <f>Calcul_reseau!A28</f>
+        <v/>
+      </c>
+      <c r="D23" s="276">
+        <f>Calcul_reseau!C28</f>
+        <v/>
+      </c>
+      <c r="E23" s="277">
+        <f>Calcul_reseau!P28</f>
+        <v/>
+      </c>
+      <c r="F23" s="281">
+        <f>Calcul_reseau!M28</f>
+        <v/>
+      </c>
+      <c r="G23" s="281">
+        <f>MAX(F23,$B$8)</f>
+        <v/>
+      </c>
+      <c r="H23" s="277">
+        <f>IF(Calcul_reseau!N28="",0,Calcul_reseau!N28/1000)</f>
+        <v/>
+      </c>
+      <c r="I23" s="278">
+        <f>Calcul_reseau!S28</f>
+        <v/>
+      </c>
+      <c r="J23" s="299">
+        <f>IF(OR(I23="",H23=0),"",I23-$B$9-H23)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="276" t="n">
+        <v>29</v>
+      </c>
+      <c r="B24" s="276">
+        <f>Calcul_reseau!AC29</f>
+        <v/>
+      </c>
+      <c r="C24" s="276">
+        <f>Calcul_reseau!A29</f>
+        <v/>
+      </c>
+      <c r="D24" s="276">
+        <f>Calcul_reseau!C29</f>
+        <v/>
+      </c>
+      <c r="E24" s="277">
+        <f>Calcul_reseau!P29</f>
+        <v/>
+      </c>
+      <c r="F24" s="281">
+        <f>Calcul_reseau!M29</f>
+        <v/>
+      </c>
+      <c r="G24" s="281">
+        <f>MAX(F24,$B$8)</f>
+        <v/>
+      </c>
+      <c r="H24" s="277">
+        <f>IF(Calcul_reseau!N29="",0,Calcul_reseau!N29/1000)</f>
+        <v/>
+      </c>
+      <c r="I24" s="278">
+        <f>Calcul_reseau!S29</f>
+        <v/>
+      </c>
+      <c r="J24" s="299">
+        <f>IF(OR(I24="",H24=0),"",I24-$B$9-H24)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="273" t="inlineStr">
+        <is>
+          <t>INVERTS DES NOEUDS (formules dynamiques)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Noeud.final = proposition AVAL (pour garder l’écoulement vers PUB). Si MIN branches (col D) &lt; aval (col C) → alerte couverture.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="275" t="inlineStr">
         <is>
           <t>Noeud</t>
         </is>
       </c>
-      <c r="B10" s="275" t="inlineStr">
-        <is>
-          <t>Invert (m)</t>
-        </is>
-      </c>
-      <c r="C10" s="275" t="inlineStr">
+      <c r="B28" s="275" t="inlineStr">
+        <is>
+          <t>Invert final (m)</t>
+        </is>
+      </c>
+      <c r="C28" s="275" t="inlineStr">
+        <is>
+          <t>Depuis aval (m)</t>
+        </is>
+      </c>
+      <c r="D28" s="275" t="inlineStr">
+        <is>
+          <t>Arrivée branche(s) (m)</t>
+        </is>
+      </c>
+      <c r="E28" s="275" t="inlineStr">
+        <is>
+          <t>Règle</t>
+        </is>
+      </c>
+      <c r="F28" s="275" t="inlineStr">
         <is>
           <t>Sol (m)</t>
         </is>
       </c>
-      <c r="D10" s="275" t="inlineStr">
-        <is>
-          <t>Couverture approx (m)</t>
-        </is>
-      </c>
-      <c r="E10" s="275" t="inlineStr">
-        <is>
-          <t>Nb propositions</t>
-        </is>
-      </c>
-      <c r="F10" s="275" t="inlineStr">
-        <is>
-          <t>Propositions (m)</t>
-        </is>
-      </c>
-      <c r="G10" s="275" t="inlineStr">
-        <is>
-          <t>Note</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="276" t="inlineStr">
-        <is>
-          <t>P09</t>
-        </is>
-      </c>
-      <c r="B11" s="277" t="n">
-        <v>16.976</v>
-      </c>
-      <c r="C11" s="278" t="n">
-        <v>17.62</v>
-      </c>
-      <c r="D11" s="277" t="n">
-        <v>0.644</v>
-      </c>
-      <c r="E11" s="276" t="n">
-        <v>1</v>
-      </c>
-      <c r="F11" s="276" t="inlineStr">
-        <is>
-          <t>16.976</t>
-        </is>
-      </c>
-      <c r="G11" s="276" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="276" t="inlineStr">
-        <is>
-          <t>P07</t>
-        </is>
-      </c>
-      <c r="B12" s="277" t="n">
-        <v>16.567</v>
-      </c>
-      <c r="C12" s="278" t="n">
-        <v>17.09</v>
-      </c>
-      <c r="D12" s="277" t="n">
-        <v>0.523</v>
-      </c>
-      <c r="E12" s="276" t="n">
-        <v>1</v>
-      </c>
-      <c r="F12" s="276" t="inlineStr">
-        <is>
-          <t>16.567</t>
-        </is>
-      </c>
-      <c r="G12" s="276" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="295" t="inlineStr">
-        <is>
-          <t>P06</t>
-        </is>
-      </c>
-      <c r="B13" s="296" t="n">
-        <v>16.422</v>
-      </c>
-      <c r="C13" s="296" t="n">
-        <v>17.14</v>
-      </c>
-      <c r="D13" s="296" t="n">
-        <v>0.718</v>
-      </c>
-      <c r="E13" s="295" t="n">
-        <v>1</v>
-      </c>
-      <c r="F13" s="295" t="inlineStr">
-        <is>
-          <t>16.422</t>
-        </is>
-      </c>
-      <c r="G13" s="295" t="inlineStr">
-        <is>
-          <t>CONFLUENCE — radier unique (plus bas / calé aval); branches amont: P06</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="276" t="inlineStr">
-        <is>
-          <t>P04</t>
-        </is>
-      </c>
-      <c r="B14" s="277" t="n">
-        <v>16.306</v>
-      </c>
-      <c r="C14" s="278" t="n">
-        <v>17.28</v>
-      </c>
-      <c r="D14" s="277" t="n">
-        <v>0.974</v>
-      </c>
-      <c r="E14" s="276" t="n">
-        <v>1</v>
-      </c>
-      <c r="F14" s="276" t="inlineStr">
-        <is>
-          <t>16.306</t>
-        </is>
-      </c>
-      <c r="G14" s="276" t="inlineStr"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="276" t="inlineStr">
-        <is>
-          <t>P01</t>
-        </is>
-      </c>
-      <c r="B15" s="277" t="n">
-        <v>16.153</v>
-      </c>
-      <c r="C15" s="278" t="n">
-        <v>17.23</v>
-      </c>
-      <c r="D15" s="277" t="n">
-        <v>1.077</v>
-      </c>
-      <c r="E15" s="276" t="n">
-        <v>1</v>
-      </c>
-      <c r="F15" s="276" t="inlineStr">
-        <is>
-          <t>16.153</t>
-        </is>
-      </c>
-      <c r="G15" s="276" t="inlineStr"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="276" t="inlineStr">
-        <is>
-          <t>P02</t>
-        </is>
-      </c>
-      <c r="B16" s="277" t="n">
-        <v>16.025</v>
-      </c>
-      <c r="C16" s="278" t="n">
-        <v>17.131</v>
-      </c>
-      <c r="D16" s="277" t="n">
-        <v>1.106</v>
-      </c>
-      <c r="E16" s="276" t="n">
-        <v>1</v>
-      </c>
-      <c r="F16" s="276" t="inlineStr">
-        <is>
-          <t>16.025</t>
-        </is>
-      </c>
-      <c r="G16" s="276" t="inlineStr"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="295" t="inlineStr">
-        <is>
-          <t>J01</t>
-        </is>
-      </c>
-      <c r="B17" s="296" t="n">
-        <v>15.989</v>
-      </c>
-      <c r="C17" s="296" t="n">
-        <v>17.12</v>
-      </c>
-      <c r="D17" s="296" t="n">
-        <v>1.131</v>
-      </c>
-      <c r="E17" s="295" t="n">
-        <v>1</v>
-      </c>
-      <c r="F17" s="295" t="inlineStr">
-        <is>
-          <t>15.989</t>
-        </is>
-      </c>
-      <c r="G17" s="295" t="inlineStr">
-        <is>
-          <t>CONFLUENCE — radier unique (plus bas / calé aval); branches amont: J01</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="276" t="inlineStr">
-        <is>
-          <t>RP03</t>
-        </is>
-      </c>
-      <c r="B18" s="277" t="n">
-        <v>15.857</v>
-      </c>
-      <c r="C18" s="278" t="n">
-        <v>17.01</v>
-      </c>
-      <c r="D18" s="277" t="n">
-        <v>1.153</v>
-      </c>
-      <c r="E18" s="276" t="n">
-        <v>1</v>
-      </c>
-      <c r="F18" s="276" t="inlineStr">
-        <is>
-          <t>15.857</t>
-        </is>
-      </c>
-      <c r="G18" s="276" t="inlineStr"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="276" t="inlineStr">
-        <is>
-          <t>P10</t>
-        </is>
-      </c>
-      <c r="B19" s="277" t="n">
-        <v>15.766</v>
-      </c>
-      <c r="C19" s="278" t="n">
-        <v>16.965</v>
-      </c>
-      <c r="D19" s="277" t="n">
-        <v>1.199</v>
-      </c>
-      <c r="E19" s="276" t="n">
-        <v>1</v>
-      </c>
-      <c r="F19" s="276" t="inlineStr">
-        <is>
-          <t>15.766</t>
-        </is>
-      </c>
-      <c r="G19" s="276" t="inlineStr"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="276" t="inlineStr">
-        <is>
-          <t>T1</t>
-        </is>
-      </c>
-      <c r="B20" s="277" t="n">
-        <v>15.743</v>
-      </c>
-      <c r="C20" s="278" t="n">
-        <v>17.01</v>
-      </c>
-      <c r="D20" s="277" t="n">
-        <v>1.267</v>
-      </c>
-      <c r="E20" s="276" t="n">
-        <v>1</v>
-      </c>
-      <c r="F20" s="276" t="inlineStr">
-        <is>
-          <t>15.743</t>
-        </is>
-      </c>
-      <c r="G20" s="276" t="inlineStr">
-        <is>
-          <t>Toiture (zone N)</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="295" t="inlineStr">
-        <is>
-          <t>P11</t>
-        </is>
-      </c>
-      <c r="B21" s="296" t="n">
-        <v>15.603</v>
-      </c>
-      <c r="C21" s="296" t="n">
-        <v>16.874</v>
-      </c>
-      <c r="D21" s="296" t="n">
-        <v>1.271</v>
-      </c>
-      <c r="E21" s="295" t="n">
-        <v>1</v>
-      </c>
-      <c r="F21" s="295" t="inlineStr">
-        <is>
-          <t>15.603</t>
-        </is>
-      </c>
-      <c r="G21" s="295" t="inlineStr">
-        <is>
-          <t>CONFLUENCE — radier unique (plus bas / calé aval); branches amont: P11</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="276" t="inlineStr">
-        <is>
-          <t>P12</t>
-        </is>
-      </c>
-      <c r="B22" s="277" t="n">
-        <v>15.449</v>
-      </c>
-      <c r="C22" s="278" t="n">
-        <v>16.73</v>
-      </c>
-      <c r="D22" s="277" t="n">
-        <v>1.281</v>
-      </c>
-      <c r="E22" s="276" t="n">
-        <v>1</v>
-      </c>
-      <c r="F22" s="276" t="inlineStr">
-        <is>
-          <t>15.449</t>
-        </is>
-      </c>
-      <c r="G22" s="276" t="inlineStr"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="276" t="inlineStr">
-        <is>
-          <t>PUB</t>
-        </is>
-      </c>
-      <c r="B23" s="277" t="n">
-        <v>15.305</v>
-      </c>
-      <c r="C23" s="278" t="n">
-        <v>16.73</v>
-      </c>
-      <c r="D23" s="277" t="n">
-        <v>1.425</v>
-      </c>
-      <c r="E23" s="276" t="n">
-        <v>1</v>
-      </c>
-      <c r="F23" s="276" t="inlineStr">
-        <is>
-          <t>15.305</t>
-        </is>
-      </c>
-      <c r="G23" s="276" t="inlineStr">
-        <is>
-          <t>Exutoire fixe</t>
-        </is>
-      </c>
-    </row>
-    <row r="24"/>
-    <row r="25">
-      <c r="A25" s="273" t="inlineStr">
-        <is>
-          <t>Profil par conduite (U amont / V aval)</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="275" t="inlineStr">
-        <is>
-          <t>Pipe_ID</t>
-        </is>
-      </c>
-      <c r="B26" s="275" t="inlineStr">
-        <is>
-          <t>De</t>
-        </is>
-      </c>
-      <c r="C26" s="275" t="inlineStr">
-        <is>
-          <t>Vers</t>
-        </is>
-      </c>
-      <c r="D26" s="275" t="inlineStr">
-        <is>
-          <t>L (m)</t>
-        </is>
-      </c>
-      <c r="E26" s="275" t="inlineStr">
-        <is>
-          <t>s design</t>
-        </is>
-      </c>
-      <c r="F26" s="275" t="inlineStr">
-        <is>
-          <t>s radier utilisée</t>
-        </is>
-      </c>
-      <c r="G26" s="275" t="inlineStr">
-        <is>
-          <t>U amont (m)</t>
-        </is>
-      </c>
-      <c r="H26" s="275" t="inlineStr">
-        <is>
-          <t>V aval (m)</t>
-        </is>
-      </c>
-      <c r="I26" s="275" t="inlineStr">
-        <is>
-          <t>ΔU-V (m)</t>
-        </is>
-      </c>
-      <c r="J26" s="275" t="inlineStr">
-        <is>
-          <t>s réelle (U-V)/L</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="276" t="inlineStr">
-        <is>
-          <t>L06_P09_P06</t>
-        </is>
-      </c>
-      <c r="B27" s="276" t="inlineStr">
-        <is>
-          <t>P09</t>
-        </is>
-      </c>
-      <c r="C27" s="276" t="inlineStr">
-        <is>
-          <t>P06</t>
-        </is>
-      </c>
-      <c r="D27" s="279" t="n">
-        <v>17.458</v>
-      </c>
-      <c r="E27" s="280" t="n">
-        <v>0.0306</v>
-      </c>
-      <c r="F27" s="281" t="n">
-        <v>0.0306</v>
-      </c>
-      <c r="G27" s="277" t="n">
-        <v>16.976</v>
-      </c>
-      <c r="H27" s="277" t="n">
-        <v>16.422</v>
-      </c>
-      <c r="I27" s="277" t="n">
-        <v>0.554</v>
-      </c>
-      <c r="J27" s="281" t="n">
-        <v>0.0317</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="276" t="inlineStr">
-        <is>
-          <t>L07_P07_P06</t>
-        </is>
-      </c>
-      <c r="B28" s="276" t="inlineStr">
-        <is>
-          <t>P07</t>
-        </is>
-      </c>
-      <c r="C28" s="276" t="inlineStr">
-        <is>
-          <t>P06</t>
-        </is>
-      </c>
-      <c r="D28" s="279" t="n">
-        <v>12.477</v>
-      </c>
-      <c r="E28" s="280" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="F28" s="281" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="G28" s="277" t="n">
-        <v>16.567</v>
-      </c>
-      <c r="H28" s="277" t="n">
-        <v>16.422</v>
-      </c>
-      <c r="I28" s="277" t="n">
-        <v>0.145</v>
-      </c>
-      <c r="J28" s="281" t="n">
-        <v>0.0116</v>
+      <c r="G28" s="275" t="inlineStr">
+        <is>
+          <t>Couverture (m)</t>
+        </is>
+      </c>
+      <c r="H28" s="301" t="inlineStr">
+        <is>
+          <t>MIN invert amont des branches</t>
+        </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="276" t="inlineStr">
         <is>
-          <t>L08_P06_P04</t>
-        </is>
-      </c>
-      <c r="B29" s="276" t="inlineStr">
-        <is>
-          <t>P06</t>
-        </is>
-      </c>
-      <c r="C29" s="276" t="inlineStr">
-        <is>
-          <t>P04</t>
-        </is>
-      </c>
-      <c r="D29" s="279" t="n">
-        <v>9.579000000000001</v>
-      </c>
-      <c r="E29" s="280" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="F29" s="281" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="G29" s="277" t="n">
-        <v>16.422</v>
-      </c>
-      <c r="H29" s="277" t="n">
-        <v>16.306</v>
-      </c>
-      <c r="I29" s="277" t="n">
-        <v>0.116</v>
-      </c>
-      <c r="J29" s="281" t="n">
-        <v>0.0121</v>
+          <t>PUB</t>
+        </is>
+      </c>
+      <c r="B29" s="277">
+        <f>C29</f>
+        <v/>
+      </c>
+      <c r="C29" s="278">
+        <f>$B$6</f>
+        <v/>
+      </c>
+      <c r="D29" s="276" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E29" s="276" t="inlineStr">
+        <is>
+          <t>Exutoire fixe</t>
+        </is>
+      </c>
+      <c r="F29" s="278">
+        <f>IFERROR(AVERAGEIF(Calcul_reseau!C:C,A29,Calcul_reseau!T:T),"")</f>
+        <v/>
+      </c>
+      <c r="G29" s="277">
+        <f>IF(OR(F29="",B29=""),"",F29-B29)</f>
+        <v/>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="276" t="inlineStr">
         <is>
-          <t>L09_P04_P01</t>
-        </is>
-      </c>
-      <c r="B30" s="276" t="inlineStr">
-        <is>
-          <t>P04</t>
-        </is>
-      </c>
-      <c r="C30" s="276" t="inlineStr">
-        <is>
-          <t>P01</t>
-        </is>
-      </c>
-      <c r="D30" s="279" t="n">
-        <v>13.317</v>
-      </c>
-      <c r="E30" s="280" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="F30" s="281" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="G30" s="277" t="n">
-        <v>16.306</v>
-      </c>
-      <c r="H30" s="277" t="n">
-        <v>16.153</v>
-      </c>
-      <c r="I30" s="277" t="n">
-        <v>0.153</v>
-      </c>
-      <c r="J30" s="281" t="n">
-        <v>0.0115</v>
+          <t>P12</t>
+        </is>
+      </c>
+      <c r="B30" s="277">
+        <f>C30</f>
+        <v/>
+      </c>
+      <c r="C30" s="278">
+        <f>$B$6+G24*E24+$B$7</f>
+        <v/>
+      </c>
+      <c r="D30" s="276" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E30" s="276" t="inlineStr">
+        <is>
+          <t>Aval</t>
+        </is>
+      </c>
+      <c r="F30" s="278">
+        <f>Calcul_reseau!S29</f>
+        <v/>
+      </c>
+      <c r="G30" s="277">
+        <f>IF(OR(F30="",B30=""),"",F30-B30)</f>
+        <v/>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="276" t="inlineStr">
-        <is>
-          <t>L01_P01_J01</t>
-        </is>
-      </c>
-      <c r="B31" s="276" t="inlineStr">
-        <is>
-          <t>P01</t>
-        </is>
-      </c>
-      <c r="C31" s="276" t="inlineStr">
-        <is>
-          <t>J01</t>
-        </is>
-      </c>
-      <c r="D31" s="279" t="n">
-        <v>14.401</v>
-      </c>
-      <c r="E31" s="280" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="F31" s="281" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="G31" s="277" t="n">
-        <v>16.153</v>
-      </c>
-      <c r="H31" s="277" t="n">
-        <v>15.989</v>
-      </c>
-      <c r="I31" s="277" t="n">
-        <v>0.164</v>
-      </c>
-      <c r="J31" s="281" t="n">
-        <v>0.0114</v>
+      <c r="A31" s="295" t="inlineStr">
+        <is>
+          <t>P11</t>
+        </is>
+      </c>
+      <c r="B31" s="296">
+        <f>C31</f>
+        <v/>
+      </c>
+      <c r="C31" s="296">
+        <f>B30+G23*E23+$B$7</f>
+        <v/>
+      </c>
+      <c r="D31" s="296">
+        <f>MIN(IFERROR(J21-G21*E21,1E99),IFERROR(J22-G22*E22,1E99))</f>
+        <v/>
+      </c>
+      <c r="E31" s="295" t="inlineStr">
+        <is>
+          <t>CONFLUENCE: radier=AVAL; D=MIN arrivées branches (info)</t>
+        </is>
+      </c>
+      <c r="F31" s="296">
+        <f>Calcul_reseau!S28</f>
+        <v/>
+      </c>
+      <c r="G31" s="296">
+        <f>IF(OR(F31="",B31=""),"",F31-B31)</f>
+        <v/>
+      </c>
+      <c r="H31" s="302">
+        <f>MIN(B32,B33)</f>
+        <v/>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>← branche la plus basse entre P10 et T1</t>
+        </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="276" t="inlineStr">
         <is>
-          <t>L12_P02_J01</t>
-        </is>
-      </c>
-      <c r="B32" s="276" t="inlineStr">
-        <is>
-          <t>P02</t>
-        </is>
-      </c>
-      <c r="C32" s="276" t="inlineStr">
-        <is>
-          <t>J01</t>
-        </is>
-      </c>
-      <c r="D32" s="279" t="n">
-        <v>1.4</v>
-      </c>
-      <c r="E32" s="280" t="n">
-        <v>0.0114</v>
-      </c>
-      <c r="F32" s="281" t="n">
-        <v>0.0114</v>
-      </c>
-      <c r="G32" s="277" t="n">
-        <v>16.025</v>
-      </c>
-      <c r="H32" s="277" t="n">
-        <v>15.989</v>
-      </c>
-      <c r="I32" s="277" t="n">
-        <v>0.036</v>
-      </c>
-      <c r="J32" s="281" t="n">
-        <v>0.0257</v>
+          <t>P10</t>
+        </is>
+      </c>
+      <c r="B32" s="277">
+        <f>C32</f>
+        <v/>
+      </c>
+      <c r="C32" s="278">
+        <f>B31+G21*E21+$B$7</f>
+        <v/>
+      </c>
+      <c r="D32" s="278">
+        <f>IF(J21="","",J21)</f>
+        <v/>
+      </c>
+      <c r="E32" s="276" t="inlineStr">
+        <is>
+          <t>MIN(aval, couverture P10)</t>
+        </is>
+      </c>
+      <c r="F32" s="278">
+        <f>Calcul_reseau!S26</f>
+        <v/>
+      </c>
+      <c r="G32" s="277">
+        <f>IF(OR(F32="",B32=""),"",F32-B32)</f>
+        <v/>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="276" t="inlineStr">
         <is>
-          <t>L02_J01_RP03</t>
-        </is>
-      </c>
-      <c r="B33" s="276" t="inlineStr">
-        <is>
-          <t>J01</t>
-        </is>
-      </c>
-      <c r="C33" s="276" t="inlineStr">
-        <is>
-          <t>RP03</t>
-        </is>
-      </c>
-      <c r="D33" s="279" t="n">
-        <v>11.2</v>
-      </c>
-      <c r="E33" s="280" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="F33" s="281" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="G33" s="277" t="n">
-        <v>15.989</v>
-      </c>
-      <c r="H33" s="277" t="n">
-        <v>15.857</v>
-      </c>
-      <c r="I33" s="277" t="n">
-        <v>0.132</v>
-      </c>
-      <c r="J33" s="281" t="n">
-        <v>0.0118</v>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="B33" s="277">
+        <f>C33</f>
+        <v/>
+      </c>
+      <c r="C33" s="278">
+        <f>B31+G22*E22+$B$7</f>
+        <v/>
+      </c>
+      <c r="D33" s="278">
+        <f>IF(J22="","",J22)</f>
+        <v/>
+      </c>
+      <c r="E33" s="276" t="inlineStr">
+        <is>
+          <t>MIN(aval, couverture T1)</t>
+        </is>
+      </c>
+      <c r="F33" s="278">
+        <f>Calcul_reseau!S27</f>
+        <v/>
+      </c>
+      <c r="G33" s="277">
+        <f>IF(OR(F33="",B33=""),"",F33-B33)</f>
+        <v/>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="276" t="inlineStr">
         <is>
-          <t>L03_RP03_P10</t>
-        </is>
-      </c>
-      <c r="B34" s="276" t="inlineStr">
-        <is>
           <t>RP03</t>
         </is>
       </c>
-      <c r="C34" s="276" t="inlineStr">
-        <is>
-          <t>P10</t>
-        </is>
-      </c>
-      <c r="D34" s="279" t="n">
-        <v>7.1</v>
-      </c>
-      <c r="E34" s="280" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="F34" s="281" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="G34" s="277" t="n">
-        <v>15.857</v>
-      </c>
-      <c r="H34" s="277" t="n">
-        <v>15.766</v>
-      </c>
-      <c r="I34" s="277" t="n">
-        <v>0.091</v>
-      </c>
-      <c r="J34" s="281" t="n">
-        <v>0.0128</v>
+      <c r="B34" s="277">
+        <f>C34</f>
+        <v/>
+      </c>
+      <c r="C34" s="278">
+        <f>B32+G20*E20+$B$7</f>
+        <v/>
+      </c>
+      <c r="D34" s="276" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E34" s="276" t="inlineStr">
+        <is>
+          <t>Aval</t>
+        </is>
+      </c>
+      <c r="F34" s="278">
+        <f>Calcul_reseau!S25</f>
+        <v/>
+      </c>
+      <c r="G34" s="277">
+        <f>IF(OR(F34="",B34=""),"",F34-B34)</f>
+        <v/>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="276" t="inlineStr">
-        <is>
-          <t>L10_P10_P11</t>
-        </is>
-      </c>
-      <c r="B35" s="276" t="inlineStr">
-        <is>
-          <t>P10</t>
-        </is>
-      </c>
-      <c r="C35" s="276" t="inlineStr">
-        <is>
-          <t>P11</t>
-        </is>
-      </c>
-      <c r="D35" s="279" t="n">
-        <v>14.3</v>
-      </c>
-      <c r="E35" s="280" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="F35" s="281" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="G35" s="277" t="n">
-        <v>15.766</v>
-      </c>
-      <c r="H35" s="277" t="n">
-        <v>15.603</v>
-      </c>
-      <c r="I35" s="277" t="n">
-        <v>0.163</v>
-      </c>
-      <c r="J35" s="281" t="n">
-        <v>0.0114</v>
+      <c r="A35" s="295" t="inlineStr">
+        <is>
+          <t>J01</t>
+        </is>
+      </c>
+      <c r="B35" s="296">
+        <f>C35</f>
+        <v/>
+      </c>
+      <c r="C35" s="296">
+        <f>B34+G19*E19+$B$7</f>
+        <v/>
+      </c>
+      <c r="D35" s="296">
+        <f>MIN(IFERROR(J17-G17*E17,1E99),IFERROR(J18-G18*E18,1E99))</f>
+        <v/>
+      </c>
+      <c r="E35" s="295" t="inlineStr">
+        <is>
+          <t>CONFLUENCE: radier=AVAL; D=MIN arrivées branches (info)</t>
+        </is>
+      </c>
+      <c r="F35" s="296">
+        <f>Calcul_reseau!S24</f>
+        <v/>
+      </c>
+      <c r="G35" s="296">
+        <f>IF(OR(F35="",B35=""),"",F35-B35)</f>
+        <v/>
+      </c>
+      <c r="H35" s="302">
+        <f>MIN(B36,B37)</f>
+        <v/>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>← branche la plus basse entre P01 et P02</t>
+        </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="276" t="inlineStr">
         <is>
-          <t>LT1_T1_P11</t>
-        </is>
-      </c>
-      <c r="B36" s="276" t="inlineStr">
-        <is>
-          <t>T1</t>
-        </is>
-      </c>
-      <c r="C36" s="276" t="inlineStr">
-        <is>
-          <t>P11</t>
-        </is>
-      </c>
-      <c r="D36" s="279" t="n">
-        <v>12</v>
-      </c>
-      <c r="E36" s="280" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="F36" s="281" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="G36" s="277" t="n">
-        <v>15.743</v>
-      </c>
-      <c r="H36" s="277" t="n">
-        <v>15.603</v>
-      </c>
-      <c r="I36" s="277" t="n">
-        <v>0.14</v>
-      </c>
-      <c r="J36" s="281" t="n">
-        <v>0.0117</v>
+          <t>P01</t>
+        </is>
+      </c>
+      <c r="B36" s="277">
+        <f>C36</f>
+        <v/>
+      </c>
+      <c r="C36" s="278">
+        <f>B35+G17*E17+$B$7</f>
+        <v/>
+      </c>
+      <c r="D36" s="278">
+        <f>IF(J17="","",J17)</f>
+        <v/>
+      </c>
+      <c r="E36" s="276" t="inlineStr">
+        <is>
+          <t>MIN(aval, couverture)</t>
+        </is>
+      </c>
+      <c r="F36" s="278">
+        <f>Calcul_reseau!S22</f>
+        <v/>
+      </c>
+      <c r="G36" s="277">
+        <f>IF(OR(F36="",B36=""),"",F36-B36)</f>
+        <v/>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="276" t="inlineStr">
         <is>
-          <t>L11_P11_P12</t>
-        </is>
-      </c>
-      <c r="B37" s="276" t="inlineStr">
-        <is>
-          <t>P11</t>
-        </is>
-      </c>
-      <c r="C37" s="276" t="inlineStr">
-        <is>
-          <t>P12</t>
-        </is>
-      </c>
-      <c r="D37" s="279" t="n">
-        <v>10.9</v>
-      </c>
-      <c r="E37" s="280" t="n">
-        <v>0.0123</v>
-      </c>
-      <c r="F37" s="281" t="n">
-        <v>0.0123</v>
-      </c>
-      <c r="G37" s="277" t="n">
-        <v>15.603</v>
-      </c>
-      <c r="H37" s="277" t="n">
-        <v>15.449</v>
-      </c>
-      <c r="I37" s="277" t="n">
-        <v>0.154</v>
-      </c>
-      <c r="J37" s="281" t="n">
-        <v>0.0141</v>
+          <t>P02</t>
+        </is>
+      </c>
+      <c r="B37" s="277">
+        <f>C37</f>
+        <v/>
+      </c>
+      <c r="C37" s="278">
+        <f>B35+G18*E18+$B$7</f>
+        <v/>
+      </c>
+      <c r="D37" s="278">
+        <f>IF(J18="","",J18)</f>
+        <v/>
+      </c>
+      <c r="E37" s="276" t="inlineStr">
+        <is>
+          <t>MIN(aval, couverture)</t>
+        </is>
+      </c>
+      <c r="F37" s="278">
+        <f>Calcul_reseau!S23</f>
+        <v/>
+      </c>
+      <c r="G37" s="277">
+        <f>IF(OR(F37="",B37=""),"",F37-B37)</f>
+        <v/>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="276" t="inlineStr">
         <is>
-          <t>L12_P12_PUB</t>
-        </is>
-      </c>
-      <c r="B38" s="276" t="inlineStr">
-        <is>
-          <t>P12</t>
-        </is>
-      </c>
-      <c r="C38" s="276" t="inlineStr">
-        <is>
-          <t>PUB</t>
-        </is>
-      </c>
-      <c r="D38" s="279" t="n">
-        <v>12.4</v>
-      </c>
-      <c r="E38" s="280" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="F38" s="281" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="G38" s="277" t="n">
-        <v>15.449</v>
-      </c>
-      <c r="H38" s="277" t="n">
-        <v>15.305</v>
-      </c>
-      <c r="I38" s="277" t="n">
-        <v>0.144</v>
-      </c>
-      <c r="J38" s="281" t="n">
-        <v>0.0116</v>
+          <t>P04</t>
+        </is>
+      </c>
+      <c r="B38" s="277">
+        <f>C38</f>
+        <v/>
+      </c>
+      <c r="C38" s="278">
+        <f>B36+G16*E16+$B$7</f>
+        <v/>
+      </c>
+      <c r="D38" s="278">
+        <f>IF(J16="","",J16)</f>
+        <v/>
+      </c>
+      <c r="E38" s="276" t="inlineStr">
+        <is>
+          <t>MIN(aval, couverture)</t>
+        </is>
+      </c>
+      <c r="F38" s="278">
+        <f>Calcul_reseau!S21</f>
+        <v/>
+      </c>
+      <c r="G38" s="277">
+        <f>IF(OR(F38="",B38=""),"",F38-B38)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="295" t="inlineStr">
+        <is>
+          <t>P06</t>
+        </is>
+      </c>
+      <c r="B39" s="296">
+        <f>C39</f>
+        <v/>
+      </c>
+      <c r="C39" s="296">
+        <f>B38+G15*E15+$B$7</f>
+        <v/>
+      </c>
+      <c r="D39" s="296">
+        <f>MIN(IFERROR(J13-G13*E13,1E99),IFERROR(J14-G14*E14,1E99))</f>
+        <v/>
+      </c>
+      <c r="E39" s="295" t="inlineStr">
+        <is>
+          <t>CONFLUENCE: radier=AVAL; D=MIN arrivées branches (info)</t>
+        </is>
+      </c>
+      <c r="F39" s="296">
+        <f>Calcul_reseau!S20</f>
+        <v/>
+      </c>
+      <c r="G39" s="296">
+        <f>IF(OR(F39="",B39=""),"",F39-B39)</f>
+        <v/>
+      </c>
+      <c r="H39" s="302">
+        <f>MIN(B40,B41)</f>
+        <v/>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>← branche la plus basse entre P09 et P07</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="276" t="inlineStr">
+        <is>
+          <t>P09</t>
+        </is>
+      </c>
+      <c r="B40" s="277">
+        <f>C40</f>
+        <v/>
+      </c>
+      <c r="C40" s="278">
+        <f>B39+G13*E13+$B$7</f>
+        <v/>
+      </c>
+      <c r="D40" s="278">
+        <f>IF(J13="","",J13)</f>
+        <v/>
+      </c>
+      <c r="E40" s="276" t="inlineStr">
+        <is>
+          <t>MIN(aval, couverture)</t>
+        </is>
+      </c>
+      <c r="F40" s="278">
+        <f>Calcul_reseau!S18</f>
+        <v/>
+      </c>
+      <c r="G40" s="277">
+        <f>IF(OR(F40="",B40=""),"",F40-B40)</f>
+        <v/>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="282" t="inlineStr">
-        <is>
-          <t>Lecture: aux confluences, la cellule Invert orange = MIN des propositions des branches.</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>Les U/V de Calcul_reseau sont alignés sur cette table. Si vous changez une longueur (ex. T1), il faut recalculer les radiers.</t>
+      <c r="A41" s="276" t="inlineStr">
+        <is>
+          <t>P07</t>
+        </is>
+      </c>
+      <c r="B41" s="277">
+        <f>C41</f>
+        <v/>
+      </c>
+      <c r="C41" s="278">
+        <f>B39+G14*E14+$B$7</f>
+        <v/>
+      </c>
+      <c r="D41" s="278">
+        <f>IF(J14="","",J14)</f>
+        <v/>
+      </c>
+      <c r="E41" s="276" t="inlineStr">
+        <is>
+          <t>MIN(aval, couverture)</t>
+        </is>
+      </c>
+      <c r="F41" s="278">
+        <f>Calcul_reseau!S19</f>
+        <v/>
+      </c>
+      <c r="G41" s="277">
+        <f>IF(OR(F41="",B41=""),"",F41-B41)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="273" t="inlineStr">
+        <is>
+          <t>Alerte drainage</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="300">
+        <f>IF(OR(AND(ISNUMBER(D31),D31&lt;C31),AND(ISNUMBER(D35),D35&lt;C35),AND(ISNUMBER(D39),D39&lt;C39)),"ALERTE: couverture d'une branche impose un radier plus bas que l'aval — approfondir ou revoir s/L","OK: confluences cohérentes avec l'exutoire")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="273" t="inlineStr">
+        <is>
+          <t>U/V PAR CONDUITE (dynamique) — Calcul_reseau lit ces valeurs</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="275" t="inlineStr">
+        <is>
+          <t>Pipe_ID</t>
+        </is>
+      </c>
+      <c r="B47" s="275" t="inlineStr">
+        <is>
+          <t>De</t>
+        </is>
+      </c>
+      <c r="C47" s="275" t="inlineStr">
+        <is>
+          <t>Vers</t>
+        </is>
+      </c>
+      <c r="D47" s="275" t="inlineStr">
+        <is>
+          <t>V aval = Inv(vers)</t>
+        </is>
+      </c>
+      <c r="E47" s="275" t="inlineStr">
+        <is>
+          <t>U amont = V + s_util·L + chute</t>
+        </is>
+      </c>
+      <c r="F47" s="275" t="inlineStr">
+        <is>
+          <t>s réelle (U−V)/L</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="276">
+        <f>B13</f>
+        <v/>
+      </c>
+      <c r="B48" s="276">
+        <f>C13</f>
+        <v/>
+      </c>
+      <c r="C48" s="276">
+        <f>D13</f>
+        <v/>
+      </c>
+      <c r="D48" s="277">
+        <f>VLOOKUP(D13,$A$29:$B$41,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="E48" s="277">
+        <f>VLOOKUP(C13,$A$29:$B$41,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="F48" s="281">
+        <f>IF(E13=0,"",(E48-D48)/E13)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="276">
+        <f>B14</f>
+        <v/>
+      </c>
+      <c r="B49" s="276">
+        <f>C14</f>
+        <v/>
+      </c>
+      <c r="C49" s="276">
+        <f>D14</f>
+        <v/>
+      </c>
+      <c r="D49" s="277">
+        <f>VLOOKUP(D14,$A$29:$B$41,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="E49" s="277">
+        <f>VLOOKUP(C14,$A$29:$B$41,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="F49" s="281">
+        <f>IF(E14=0,"",(E49-D49)/E14)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="276">
+        <f>B15</f>
+        <v/>
+      </c>
+      <c r="B50" s="276">
+        <f>C15</f>
+        <v/>
+      </c>
+      <c r="C50" s="276">
+        <f>D15</f>
+        <v/>
+      </c>
+      <c r="D50" s="277">
+        <f>VLOOKUP(D15,$A$29:$B$41,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="E50" s="277">
+        <f>VLOOKUP(C15,$A$29:$B$41,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="F50" s="281">
+        <f>IF(E15=0,"",(E50-D50)/E15)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="276">
+        <f>B16</f>
+        <v/>
+      </c>
+      <c r="B51" s="276">
+        <f>C16</f>
+        <v/>
+      </c>
+      <c r="C51" s="276">
+        <f>D16</f>
+        <v/>
+      </c>
+      <c r="D51" s="277">
+        <f>VLOOKUP(D16,$A$29:$B$41,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="E51" s="277">
+        <f>VLOOKUP(C16,$A$29:$B$41,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="F51" s="281">
+        <f>IF(E16=0,"",(E51-D51)/E16)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="276">
+        <f>B17</f>
+        <v/>
+      </c>
+      <c r="B52" s="276">
+        <f>C17</f>
+        <v/>
+      </c>
+      <c r="C52" s="276">
+        <f>D17</f>
+        <v/>
+      </c>
+      <c r="D52" s="277">
+        <f>VLOOKUP(D17,$A$29:$B$41,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="E52" s="277">
+        <f>VLOOKUP(C17,$A$29:$B$41,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="F52" s="281">
+        <f>IF(E17=0,"",(E52-D52)/E17)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="276">
+        <f>B18</f>
+        <v/>
+      </c>
+      <c r="B53" s="276">
+        <f>C18</f>
+        <v/>
+      </c>
+      <c r="C53" s="276">
+        <f>D18</f>
+        <v/>
+      </c>
+      <c r="D53" s="277">
+        <f>VLOOKUP(D18,$A$29:$B$41,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="E53" s="277">
+        <f>VLOOKUP(C18,$A$29:$B$41,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="F53" s="281">
+        <f>IF(E18=0,"",(E53-D53)/E18)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="276">
+        <f>B19</f>
+        <v/>
+      </c>
+      <c r="B54" s="276">
+        <f>C19</f>
+        <v/>
+      </c>
+      <c r="C54" s="276">
+        <f>D19</f>
+        <v/>
+      </c>
+      <c r="D54" s="277">
+        <f>VLOOKUP(D19,$A$29:$B$41,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="E54" s="277">
+        <f>VLOOKUP(C19,$A$29:$B$41,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="F54" s="281">
+        <f>IF(E19=0,"",(E54-D54)/E19)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="276">
+        <f>B20</f>
+        <v/>
+      </c>
+      <c r="B55" s="276">
+        <f>C20</f>
+        <v/>
+      </c>
+      <c r="C55" s="276">
+        <f>D20</f>
+        <v/>
+      </c>
+      <c r="D55" s="277">
+        <f>VLOOKUP(D20,$A$29:$B$41,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="E55" s="277">
+        <f>VLOOKUP(C20,$A$29:$B$41,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="F55" s="281">
+        <f>IF(E20=0,"",(E55-D55)/E20)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="276">
+        <f>B21</f>
+        <v/>
+      </c>
+      <c r="B56" s="276">
+        <f>C21</f>
+        <v/>
+      </c>
+      <c r="C56" s="276">
+        <f>D21</f>
+        <v/>
+      </c>
+      <c r="D56" s="277">
+        <f>VLOOKUP(D21,$A$29:$B$41,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="E56" s="277">
+        <f>VLOOKUP(C21,$A$29:$B$41,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="F56" s="281">
+        <f>IF(E21=0,"",(E56-D56)/E21)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="276">
+        <f>B22</f>
+        <v/>
+      </c>
+      <c r="B57" s="276">
+        <f>C22</f>
+        <v/>
+      </c>
+      <c r="C57" s="276">
+        <f>D22</f>
+        <v/>
+      </c>
+      <c r="D57" s="277">
+        <f>VLOOKUP(D22,$A$29:$B$41,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="E57" s="277">
+        <f>VLOOKUP(C22,$A$29:$B$41,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="F57" s="281">
+        <f>IF(E22=0,"",(E57-D57)/E22)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="276">
+        <f>B23</f>
+        <v/>
+      </c>
+      <c r="B58" s="276">
+        <f>C23</f>
+        <v/>
+      </c>
+      <c r="C58" s="276">
+        <f>D23</f>
+        <v/>
+      </c>
+      <c r="D58" s="277">
+        <f>VLOOKUP(D23,$A$29:$B$41,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="E58" s="277">
+        <f>VLOOKUP(C23,$A$29:$B$41,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="F58" s="281">
+        <f>IF(E23=0,"",(E58-D58)/E23)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="276">
+        <f>B24</f>
+        <v/>
+      </c>
+      <c r="B59" s="276">
+        <f>C24</f>
+        <v/>
+      </c>
+      <c r="C59" s="276">
+        <f>D24</f>
+        <v/>
+      </c>
+      <c r="D59" s="277">
+        <f>VLOOKUP(D24,$A$29:$B$41,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="E59" s="277">
+        <f>VLOOKUP(C24,$A$29:$B$41,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="F59" s="281">
+        <f>IF(E24=0,"",(E59-D59)/E24)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Note: U et V = inverts des noeuds (formules). Si vous changez L (col P) ou s (col M) dans Calcul_reseau, tout se recalcule.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Pentes mises à jour: P09→P06 s=0.01; P11→P12 s=0.015; P12→PUB s=0.015 (modifiables en jaune dans Calcul_reseau).</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Changez librement: Calcul_reseau col M (pente) et col P (longueur). Radiers + U/V se recalculent seuls.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Pentes actuelles demandées: P09→P06=0.01; P11→P12=0.015; P12→PUB=0.015.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>À une confluence, le radier du regard = chaîne AVAL. La branche « appropriée » la plus basse est en colonne H (MIN des inverts amont).</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:H1"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4129,7 +4705,7 @@
     <row r="17" ht="22.5" customHeight="1" s="227">
       <c r="A17" s="104" t="inlineStr">
         <is>
-          <t>Tronçons (amont → aval) — J01 + T1(toit)→P11; radiers: plus bas aux confluences</t>
+          <t>Tronçons — radiers dynamiques (formules). T1→P11 inclus. Confluences: MIN.</t>
         </is>
       </c>
       <c r="B17" s="92" t="n"/>
@@ -4210,7 +4786,7 @@
         <v/>
       </c>
       <c r="M18" s="283" t="n">
-        <v>0.0306</v>
+        <v>0.01</v>
       </c>
       <c r="N18" s="285" t="n">
         <v>200</v>
@@ -4236,11 +4812,13 @@
       <c r="T18" s="287" t="n">
         <v>17.14</v>
       </c>
-      <c r="U18" s="253" t="n">
-        <v>16.976</v>
-      </c>
-      <c r="V18" s="253" t="n">
-        <v>16.422</v>
+      <c r="U18" s="253">
+        <f>Radiers!E48</f>
+        <v/>
+      </c>
+      <c r="V18" s="253">
+        <f>Radiers!D48</f>
+        <v/>
       </c>
       <c r="W18" s="253">
         <f>IF(OR(S18="",U18=""),"",S18-U18-N18/1000)</f>
@@ -4343,11 +4921,13 @@
       <c r="T19" s="287" t="n">
         <v>17.14</v>
       </c>
-      <c r="U19" s="253" t="n">
-        <v>16.567</v>
-      </c>
-      <c r="V19" s="253" t="n">
-        <v>16.422</v>
+      <c r="U19" s="253">
+        <f>Radiers!E49</f>
+        <v/>
+      </c>
+      <c r="V19" s="253">
+        <f>Radiers!D49</f>
+        <v/>
       </c>
       <c r="W19" s="253">
         <f>IF(OR(S19="",U19=""),"",S19-U19-N19/1000)</f>
@@ -4450,11 +5030,13 @@
       <c r="T20" s="287" t="n">
         <v>17.28</v>
       </c>
-      <c r="U20" s="253" t="n">
-        <v>16.422</v>
-      </c>
-      <c r="V20" s="253" t="n">
-        <v>16.306</v>
+      <c r="U20" s="253">
+        <f>Radiers!E50</f>
+        <v/>
+      </c>
+      <c r="V20" s="253">
+        <f>Radiers!D50</f>
+        <v/>
       </c>
       <c r="W20" s="253">
         <f>IF(OR(S20="",U20=""),"",S20-U20-N20/1000)</f>
@@ -4557,11 +5139,13 @@
       <c r="T21" s="287" t="n">
         <v>17.23</v>
       </c>
-      <c r="U21" s="253" t="n">
-        <v>16.306</v>
-      </c>
-      <c r="V21" s="253" t="n">
-        <v>16.153</v>
+      <c r="U21" s="253">
+        <f>Radiers!E51</f>
+        <v/>
+      </c>
+      <c r="V21" s="253">
+        <f>Radiers!D51</f>
+        <v/>
       </c>
       <c r="W21" s="253">
         <f>IF(OR(S21="",U21=""),"",S21-U21-N21/1000)</f>
@@ -4664,11 +5248,13 @@
       <c r="T22" s="287" t="n">
         <v>17.12</v>
       </c>
-      <c r="U22" s="253" t="n">
-        <v>16.153</v>
-      </c>
-      <c r="V22" s="253" t="n">
-        <v>15.989</v>
+      <c r="U22" s="253">
+        <f>Radiers!E52</f>
+        <v/>
+      </c>
+      <c r="V22" s="253">
+        <f>Radiers!D52</f>
+        <v/>
       </c>
       <c r="W22" s="253">
         <f>IF(OR(S22="",U22=""),"",S22-U22-N22/1000)</f>
@@ -4771,11 +5357,13 @@
       <c r="T23" s="287" t="n">
         <v>17.12</v>
       </c>
-      <c r="U23" s="253" t="n">
-        <v>16.025</v>
-      </c>
-      <c r="V23" s="253" t="n">
-        <v>15.989</v>
+      <c r="U23" s="253">
+        <f>Radiers!E53</f>
+        <v/>
+      </c>
+      <c r="V23" s="253">
+        <f>Radiers!D53</f>
+        <v/>
       </c>
       <c r="W23" s="253">
         <f>IF(OR(S23="",U23=""),"",S23-U23-N23/1000)</f>
@@ -4878,11 +5466,13 @@
       <c r="T24" s="287" t="n">
         <v>17.01</v>
       </c>
-      <c r="U24" s="253" t="n">
-        <v>15.989</v>
-      </c>
-      <c r="V24" s="253" t="n">
-        <v>15.857</v>
+      <c r="U24" s="253">
+        <f>Radiers!E54</f>
+        <v/>
+      </c>
+      <c r="V24" s="253">
+        <f>Radiers!D54</f>
+        <v/>
       </c>
       <c r="W24" s="253">
         <f>IF(OR(S24="",U24=""),"",S24-U24-N24/1000)</f>
@@ -4985,11 +5575,13 @@
       <c r="T25" s="287" t="n">
         <v>16.965</v>
       </c>
-      <c r="U25" s="253" t="n">
-        <v>15.857</v>
-      </c>
-      <c r="V25" s="253" t="n">
-        <v>15.766</v>
+      <c r="U25" s="253">
+        <f>Radiers!E55</f>
+        <v/>
+      </c>
+      <c r="V25" s="253">
+        <f>Radiers!D55</f>
+        <v/>
       </c>
       <c r="W25" s="253">
         <f>IF(OR(S25="",U25=""),"",S25-U25-N25/1000)</f>
@@ -5092,11 +5684,13 @@
       <c r="T26" s="287" t="n">
         <v>16.874</v>
       </c>
-      <c r="U26" s="253" t="n">
-        <v>15.766</v>
-      </c>
-      <c r="V26" s="253" t="n">
-        <v>15.603</v>
+      <c r="U26" s="253">
+        <f>Radiers!E56</f>
+        <v/>
+      </c>
+      <c r="V26" s="253">
+        <f>Radiers!D56</f>
+        <v/>
       </c>
       <c r="W26" s="253">
         <f>IF(OR(S26="",U26=""),"",S26-U26-N26/1000)</f>
@@ -5199,11 +5793,13 @@
       <c r="T27" s="287" t="n">
         <v>16.874</v>
       </c>
-      <c r="U27" s="253" t="n">
-        <v>15.743</v>
-      </c>
-      <c r="V27" s="253" t="n">
-        <v>15.603</v>
+      <c r="U27" s="253">
+        <f>Radiers!E57</f>
+        <v/>
+      </c>
+      <c r="V27" s="253">
+        <f>Radiers!D57</f>
+        <v/>
       </c>
       <c r="W27" s="253">
         <f>IF(OR(S27="",U27=""),"",S27-U27-N27/1000)</f>
@@ -5280,7 +5876,7 @@
         <v/>
       </c>
       <c r="M28" s="283" t="n">
-        <v>0.0123</v>
+        <v>0.015</v>
       </c>
       <c r="N28" s="285" t="n">
         <v>250</v>
@@ -5306,11 +5902,13 @@
       <c r="T28" s="287" t="n">
         <v>16.73</v>
       </c>
-      <c r="U28" s="253" t="n">
-        <v>15.603</v>
-      </c>
-      <c r="V28" s="253" t="n">
-        <v>15.449</v>
+      <c r="U28" s="253">
+        <f>Radiers!E58</f>
+        <v/>
+      </c>
+      <c r="V28" s="253">
+        <f>Radiers!D58</f>
+        <v/>
       </c>
       <c r="W28" s="253">
         <f>IF(OR(S28="",U28=""),"",S28-U28-N28/1000)</f>
@@ -5387,7 +5985,7 @@
         <v/>
       </c>
       <c r="M29" s="283" t="n">
-        <v>0.01</v>
+        <v>0.015</v>
       </c>
       <c r="N29" s="285" t="n">
         <v>300</v>
@@ -5413,11 +6011,13 @@
       <c r="T29" s="287" t="n">
         <v>16.73</v>
       </c>
-      <c r="U29" s="253" t="n">
-        <v>15.449</v>
-      </c>
-      <c r="V29" s="253" t="n">
-        <v>15.305</v>
+      <c r="U29" s="253">
+        <f>Radiers!E59</f>
+        <v/>
+      </c>
+      <c r="V29" s="253">
+        <f>Radiers!D59</f>
+        <v/>
       </c>
       <c r="W29" s="253">
         <f>IF(OR(S29="",U29=""),"",S29-U29-N29/1000)</f>
@@ -5514,7 +6114,7 @@
     <row r="32" ht="22.5" customHeight="1" s="227">
       <c r="A32" s="207" t="inlineStr">
         <is>
-          <t>Radiers (U/V): calés depuis exutoire PUB=15.305 m; pente radier = max(s conduite, 1%); chute regard=0.02 m.</t>
+          <t>Radiers DYNAMIQUES (onglet Radiers): changez L (col P) ou s (col M) — U/V se recalculent. Confluences = MIN(aval, branches).</t>
         </is>
       </c>
       <c r="B32" s="259" t="n"/>

</xml_diff>

<commit_message>
Fix duplicate zone N (903 m²) on L10 vs LT1 across all tabs
RESUME and Temps still attributed roof zone N to L10 while LT1 also
had it. Zero L10 area/te everywhere; keep N only on LT1. Align Guide
and notes; document Q repercussions at P11; radiers unaffected.

Co-authored-by: acon560-prog <acon560-prog@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/engineering/drainage-design/Dimensionnement_reseau_pluvial_ADAPTE_methode_simple OLIVIER TECH. MODIF.xlsx
+++ b/engineering/drainage-design/Dimensionnement_reseau_pluvial_ADAPTE_methode_simple OLIVIER TECH. MODIF.xlsx
@@ -29,7 +29,7 @@
     <numFmt numFmtId="168" formatCode="0.0000"/>
     <numFmt numFmtId="169" formatCode="0.00000"/>
   </numFmts>
-  <fonts count="26">
+  <fonts count="30">
     <font>
       <name val="Times New Roman"/>
       <charset val="1"/>
@@ -193,8 +193,27 @@
       <b val="1"/>
       <sz val="10"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00922B21"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00922B21"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="001B4F72"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="001B4F72"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="20">
+  <fills count="24">
     <fill>
       <patternFill/>
     </fill>
@@ -303,6 +322,26 @@
         <fgColor rgb="00DDEBF7"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FDEBD0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D5F5E3"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FADBD8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCF3CF"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="66">
     <border>
@@ -1125,7 +1164,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="303">
+  <cellXfs count="322">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
@@ -1882,6 +1921,41 @@
     <xf numFmtId="0" fontId="0" fillId="19" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="0" fillId="18" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="20" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="21" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="26" fillId="22" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="23" borderId="48" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="168" fontId="2" fillId="20" borderId="41" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="2" fillId="21" borderId="41" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="2" fillId="20" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="21" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="20" borderId="47" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="0" fillId="20" borderId="47" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="0" fillId="20" borderId="47" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="0" fillId="20" borderId="47" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="26" fillId="22" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="4" fillId="20" borderId="47" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="27" fillId="20" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="18" fillId="21" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="20" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2149,7 +2223,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A28"/>
+  <dimension ref="A1:Y200"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.5" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="110" customWidth="1" style="227" min="1" max="1"/>
@@ -2162,6 +2236,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="15" customHeight="1" s="227">
       <c r="A3" s="4" t="inlineStr">
         <is>
@@ -2183,6 +2258,7 @@
         </is>
       </c>
     </row>
+    <row r="6"/>
     <row r="7" ht="15" customHeight="1" s="227">
       <c r="A7" s="4" t="inlineStr">
         <is>
@@ -2204,6 +2280,7 @@
         </is>
       </c>
     </row>
+    <row r="10"/>
     <row r="11" ht="15" customHeight="1" s="227">
       <c r="A11" s="4" t="inlineStr">
         <is>
@@ -2268,61 +2345,246 @@
       </c>
     </row>
     <row r="20" ht="15" customHeight="1" s="227">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>L10: P10 → P11 | L=14.3 m | zone N</t>
+      <c r="A20" s="303" t="inlineStr">
+        <is>
+          <t>L10: P10 → P11 | L=14.3 m | TRANSFERT DA=0 (zone N retirée)</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>L11: P11 → P12 | L=10.9 m | zone O</t>
+      <c r="A21" s="304" t="inlineStr">
+        <is>
+          <t>LT1: T1 → P11 | L=12 m | zone N = 903 m², C=0.95 (SEUL)</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>L12_out: P12 → PUB | L=12.4 m</t>
+          <t>L11: P11 → P12 | L=10.9 m | zone O seulement (PAS de N)</t>
         </is>
       </c>
     </row>
     <row r="23" ht="15" customHeight="1" s="227">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>H/I: à J01, P02→J01 ne cumule pas le réseau amont; J01→RP03 = H(P01→J01)+H(P02→J01)+DA.</t>
+          <t>L12_out: P12 → PUB | L=12.4 m</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>H/I: à J01, P02→J01 = DA locale; J01→RP03 fusionne. À P11: P10(DA=0)+T1(N)+L11(O).</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>MAJ radiers + T1:</t>
+      <c r="A25" s="305" t="inlineStr">
+        <is>
+          <t>⚠ RÉPERCUSSIONS: Remettre N sur L10 alors qu'elle est sur LT1 → A cumulée à P11 +903 m² en trop, Qmax surdimensionné, C et I faussés. Radiers (onglet Radiers) NON affectés (L et s seulement).</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>- Onglet Radiers: inverts depuis PUB=15.305, chute 0.02, pente min 1%, MIN aux confluences P06/J01/P11</t>
+          <t>MAJ radiers + T1:</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>- Nouveau T1 (toit zone N) → P11; DA 903 m² retirée de P10→P11</t>
+          <t>- Onglet Radiers: inverts depuis PUB=15.305, chute 0.02, pente min 1%, MIN aux confluences P06/J01/P11</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>- Calcul_reseau U/V = radiers calculés (vert)</t>
-        </is>
-      </c>
-    </row>
+          <t>- T1 (toit zone N) → P11; 903 m² retirée de L10 partout (Calcul E26=0, Temps H6=0, RESUME L10=0)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>- Calcul_reseau U/V = radiers dynamiques; te L10 (Temps!H7)=0 → tc P10→P11 = trajet amont seulement</t>
+        </is>
+      </c>
+    </row>
+    <row r="30"/>
+    <row r="31"/>
+    <row r="32"/>
+    <row r="33"/>
+    <row r="34"/>
+    <row r="35"/>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39"/>
+    <row r="40"/>
+    <row r="41"/>
+    <row r="42"/>
+    <row r="43"/>
+    <row r="44"/>
+    <row r="45"/>
+    <row r="46"/>
+    <row r="47"/>
+    <row r="48"/>
+    <row r="49"/>
+    <row r="50"/>
+    <row r="51"/>
+    <row r="52"/>
+    <row r="53"/>
+    <row r="54"/>
+    <row r="55"/>
+    <row r="56"/>
+    <row r="57"/>
+    <row r="58"/>
+    <row r="59"/>
+    <row r="60"/>
+    <row r="61"/>
+    <row r="62"/>
+    <row r="63"/>
+    <row r="64"/>
+    <row r="65"/>
+    <row r="66"/>
+    <row r="67"/>
+    <row r="68"/>
+    <row r="69"/>
+    <row r="70"/>
+    <row r="71"/>
+    <row r="72"/>
+    <row r="73"/>
+    <row r="74"/>
+    <row r="75"/>
+    <row r="76"/>
+    <row r="77"/>
+    <row r="78"/>
+    <row r="79"/>
+    <row r="80"/>
+    <row r="81"/>
+    <row r="82"/>
+    <row r="83"/>
+    <row r="84"/>
+    <row r="85"/>
+    <row r="86"/>
+    <row r="87"/>
+    <row r="88"/>
+    <row r="89"/>
+    <row r="90"/>
+    <row r="91"/>
+    <row r="92"/>
+    <row r="93"/>
+    <row r="94"/>
+    <row r="95"/>
+    <row r="96"/>
+    <row r="97"/>
+    <row r="98"/>
+    <row r="99"/>
+    <row r="100"/>
+    <row r="101"/>
+    <row r="102"/>
+    <row r="103"/>
+    <row r="104"/>
+    <row r="105"/>
+    <row r="106"/>
+    <row r="107"/>
+    <row r="108"/>
+    <row r="109"/>
+    <row r="110"/>
+    <row r="111"/>
+    <row r="112"/>
+    <row r="113"/>
+    <row r="114"/>
+    <row r="115"/>
+    <row r="116"/>
+    <row r="117"/>
+    <row r="118"/>
+    <row r="119"/>
+    <row r="120"/>
+    <row r="121"/>
+    <row r="122"/>
+    <row r="123"/>
+    <row r="124"/>
+    <row r="125"/>
+    <row r="126"/>
+    <row r="127"/>
+    <row r="128"/>
+    <row r="129"/>
+    <row r="130"/>
+    <row r="131"/>
+    <row r="132"/>
+    <row r="133"/>
+    <row r="134"/>
+    <row r="135"/>
+    <row r="136"/>
+    <row r="137"/>
+    <row r="138"/>
+    <row r="139"/>
+    <row r="140"/>
+    <row r="141"/>
+    <row r="142"/>
+    <row r="143"/>
+    <row r="144"/>
+    <row r="145"/>
+    <row r="146"/>
+    <row r="147"/>
+    <row r="148"/>
+    <row r="149"/>
+    <row r="150"/>
+    <row r="151"/>
+    <row r="152"/>
+    <row r="153"/>
+    <row r="154"/>
+    <row r="155"/>
+    <row r="156"/>
+    <row r="157"/>
+    <row r="158"/>
+    <row r="159"/>
+    <row r="160"/>
+    <row r="161"/>
+    <row r="162"/>
+    <row r="163"/>
+    <row r="164"/>
+    <row r="165"/>
+    <row r="166"/>
+    <row r="167"/>
+    <row r="168"/>
+    <row r="169"/>
+    <row r="170"/>
+    <row r="171"/>
+    <row r="172"/>
+    <row r="173"/>
+    <row r="174"/>
+    <row r="175"/>
+    <row r="176"/>
+    <row r="177"/>
+    <row r="178"/>
+    <row r="179"/>
+    <row r="180"/>
+    <row r="181"/>
+    <row r="182"/>
+    <row r="183"/>
+    <row r="184"/>
+    <row r="185"/>
+    <row r="186"/>
+    <row r="187"/>
+    <row r="188"/>
+    <row r="189"/>
+    <row r="190"/>
+    <row r="191"/>
+    <row r="192"/>
+    <row r="193"/>
+    <row r="194"/>
+    <row r="195"/>
+    <row r="196"/>
+    <row r="197"/>
+    <row r="198"/>
+    <row r="199"/>
+    <row r="200"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -2335,7 +2597,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J65"/>
+  <dimension ref="A1:Y200"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="227" min="1" max="1"/>
@@ -2356,6 +2618,11 @@
           <t>RADIERS DYNAMIQUES — changez L ou s dans Calcul_reseau; les inverts se mettent à jour</t>
         </is>
       </c>
+      <c r="J1" s="306" t="inlineStr">
+        <is>
+          <t>Note: correction zone N (L10→LT1) sans effet sur radiers.</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -2371,6 +2638,13 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" s="321" t="inlineStr">
+        <is>
+          <t>Note aires: la correction zone N (retirée de L10, seule sur LT1) n'affecte PAS les radiers — ceux-ci dépendent uniquement de L (Calcul!P) et s (Calcul!M).</t>
+        </is>
+      </c>
+    </row>
     <row r="5">
       <c r="A5" s="273" t="inlineStr">
         <is>
@@ -2428,6 +2702,7 @@
         <v>1.8</v>
       </c>
     </row>
+    <row r="10"/>
     <row r="11">
       <c r="A11" s="273" t="inlineStr">
         <is>
@@ -2979,6 +3254,7 @@
         <v/>
       </c>
     </row>
+    <row r="25"/>
     <row r="26">
       <c r="A26" s="273" t="inlineStr">
         <is>
@@ -3481,6 +3757,7 @@
         <v/>
       </c>
     </row>
+    <row r="42"/>
     <row r="43">
       <c r="A43" s="273" t="inlineStr">
         <is>
@@ -3494,6 +3771,7 @@
         <v/>
       </c>
     </row>
+    <row r="45"/>
     <row r="46">
       <c r="A46" s="273" t="inlineStr">
         <is>
@@ -3845,6 +4123,7 @@
         <v/>
       </c>
     </row>
+    <row r="60"/>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
@@ -3880,6 +4159,141 @@
         </is>
       </c>
     </row>
+    <row r="66"/>
+    <row r="67"/>
+    <row r="68"/>
+    <row r="69"/>
+    <row r="70"/>
+    <row r="71"/>
+    <row r="72"/>
+    <row r="73"/>
+    <row r="74"/>
+    <row r="75"/>
+    <row r="76"/>
+    <row r="77"/>
+    <row r="78"/>
+    <row r="79"/>
+    <row r="80"/>
+    <row r="81"/>
+    <row r="82"/>
+    <row r="83"/>
+    <row r="84"/>
+    <row r="85"/>
+    <row r="86"/>
+    <row r="87"/>
+    <row r="88"/>
+    <row r="89"/>
+    <row r="90"/>
+    <row r="91"/>
+    <row r="92"/>
+    <row r="93"/>
+    <row r="94"/>
+    <row r="95"/>
+    <row r="96"/>
+    <row r="97"/>
+    <row r="98"/>
+    <row r="99"/>
+    <row r="100"/>
+    <row r="101"/>
+    <row r="102"/>
+    <row r="103"/>
+    <row r="104"/>
+    <row r="105"/>
+    <row r="106"/>
+    <row r="107"/>
+    <row r="108"/>
+    <row r="109"/>
+    <row r="110"/>
+    <row r="111"/>
+    <row r="112"/>
+    <row r="113"/>
+    <row r="114"/>
+    <row r="115"/>
+    <row r="116"/>
+    <row r="117"/>
+    <row r="118"/>
+    <row r="119"/>
+    <row r="120"/>
+    <row r="121"/>
+    <row r="122"/>
+    <row r="123"/>
+    <row r="124"/>
+    <row r="125"/>
+    <row r="126"/>
+    <row r="127"/>
+    <row r="128"/>
+    <row r="129"/>
+    <row r="130"/>
+    <row r="131"/>
+    <row r="132"/>
+    <row r="133"/>
+    <row r="134"/>
+    <row r="135"/>
+    <row r="136"/>
+    <row r="137"/>
+    <row r="138"/>
+    <row r="139"/>
+    <row r="140"/>
+    <row r="141"/>
+    <row r="142"/>
+    <row r="143"/>
+    <row r="144"/>
+    <row r="145"/>
+    <row r="146"/>
+    <row r="147"/>
+    <row r="148"/>
+    <row r="149"/>
+    <row r="150"/>
+    <row r="151"/>
+    <row r="152"/>
+    <row r="153"/>
+    <row r="154"/>
+    <row r="155"/>
+    <row r="156"/>
+    <row r="157"/>
+    <row r="158"/>
+    <row r="159"/>
+    <row r="160"/>
+    <row r="161"/>
+    <row r="162"/>
+    <row r="163"/>
+    <row r="164"/>
+    <row r="165"/>
+    <row r="166"/>
+    <row r="167"/>
+    <row r="168"/>
+    <row r="169"/>
+    <row r="170"/>
+    <row r="171"/>
+    <row r="172"/>
+    <row r="173"/>
+    <row r="174"/>
+    <row r="175"/>
+    <row r="176"/>
+    <row r="177"/>
+    <row r="178"/>
+    <row r="179"/>
+    <row r="180"/>
+    <row r="181"/>
+    <row r="182"/>
+    <row r="183"/>
+    <row r="184"/>
+    <row r="185"/>
+    <row r="186"/>
+    <row r="187"/>
+    <row r="188"/>
+    <row r="189"/>
+    <row r="190"/>
+    <row r="191"/>
+    <row r="192"/>
+    <row r="193"/>
+    <row r="194"/>
+    <row r="195"/>
+    <row r="196"/>
+    <row r="197"/>
+    <row r="198"/>
+    <row r="199"/>
+    <row r="200"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:H1"/>
@@ -3894,7 +4308,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AC174"/>
+  <dimension ref="A1:AC200"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="12" customWidth="1" style="206" min="1" max="1"/>
@@ -6180,9 +6594,9 @@
       <c r="AB33" s="127" t="n"/>
     </row>
     <row r="34" ht="22.5" customHeight="1" s="227">
-      <c r="A34" s="207" t="inlineStr">
-        <is>
-          <t>T1 = noeud toiture (zone N, 903 m², C=0.95) raccordé à P11. Longueur LT1 jaune (défaut 12 m) — ajuster puis redemander recalcul radiers si changée.</t>
+      <c r="A34" s="307" t="inlineStr">
+        <is>
+          <t>T1 = noeud toiture (zone N, 903 m², C=0.95) → P11. P10→P11: E26=0 (transfert). Ne PAS remettre 0.0903 sur E26 (doublerait avec E27).</t>
         </is>
       </c>
       <c r="B34" s="259" t="n"/>
@@ -6216,7 +6630,7 @@
     <row r="35" ht="15" customHeight="1" s="227">
       <c r="A35" s="209" t="inlineStr">
         <is>
-          <t>H/I: branches L07, L12, LT1 en DA locale; fusion à P06, J01 et P11.</t>
+          <t>H/I: branches L07, L12, LT1 en DA locale; fusion à P06, J01 et P11. Temps!H6 doit rester 0 (aligné sur E26).</t>
         </is>
       </c>
       <c r="B35" s="244" t="n"/>
@@ -6274,6 +6688,48 @@
         </is>
       </c>
     </row>
+    <row r="39"/>
+    <row r="40"/>
+    <row r="41"/>
+    <row r="42"/>
+    <row r="43"/>
+    <row r="44"/>
+    <row r="45"/>
+    <row r="46"/>
+    <row r="47"/>
+    <row r="48"/>
+    <row r="49"/>
+    <row r="50"/>
+    <row r="51"/>
+    <row r="52"/>
+    <row r="53"/>
+    <row r="54"/>
+    <row r="55"/>
+    <row r="56"/>
+    <row r="57"/>
+    <row r="58"/>
+    <row r="59"/>
+    <row r="60"/>
+    <row r="61"/>
+    <row r="62"/>
+    <row r="63"/>
+    <row r="64"/>
+    <row r="65"/>
+    <row r="66"/>
+    <row r="67"/>
+    <row r="68"/>
+    <row r="69"/>
+    <row r="70"/>
+    <row r="71"/>
+    <row r="72"/>
+    <row r="73"/>
+    <row r="74"/>
+    <row r="75"/>
+    <row r="76"/>
+    <row r="77"/>
+    <row r="78"/>
+    <row r="79"/>
+    <row r="80"/>
     <row r="81" ht="15" customHeight="1" s="227"/>
     <row r="82">
       <c r="F82" s="206" t="inlineStr">
@@ -6282,6 +6738,96 @@
         </is>
       </c>
     </row>
+    <row r="83"/>
+    <row r="84"/>
+    <row r="85"/>
+    <row r="86"/>
+    <row r="87"/>
+    <row r="88"/>
+    <row r="89"/>
+    <row r="90"/>
+    <row r="91"/>
+    <row r="92"/>
+    <row r="93"/>
+    <row r="94"/>
+    <row r="95"/>
+    <row r="96"/>
+    <row r="97"/>
+    <row r="98"/>
+    <row r="99"/>
+    <row r="100"/>
+    <row r="101"/>
+    <row r="102"/>
+    <row r="103"/>
+    <row r="104"/>
+    <row r="105"/>
+    <row r="106"/>
+    <row r="107"/>
+    <row r="108"/>
+    <row r="109"/>
+    <row r="110"/>
+    <row r="111"/>
+    <row r="112"/>
+    <row r="113"/>
+    <row r="114"/>
+    <row r="115"/>
+    <row r="116"/>
+    <row r="117"/>
+    <row r="118"/>
+    <row r="119"/>
+    <row r="120"/>
+    <row r="121"/>
+    <row r="122"/>
+    <row r="123"/>
+    <row r="124"/>
+    <row r="125"/>
+    <row r="126"/>
+    <row r="127"/>
+    <row r="128"/>
+    <row r="129"/>
+    <row r="130"/>
+    <row r="131"/>
+    <row r="132"/>
+    <row r="133"/>
+    <row r="134"/>
+    <row r="135"/>
+    <row r="136"/>
+    <row r="137"/>
+    <row r="138"/>
+    <row r="139"/>
+    <row r="140"/>
+    <row r="141"/>
+    <row r="142"/>
+    <row r="143"/>
+    <row r="144"/>
+    <row r="145"/>
+    <row r="146"/>
+    <row r="147"/>
+    <row r="148"/>
+    <row r="149"/>
+    <row r="150"/>
+    <row r="151"/>
+    <row r="152"/>
+    <row r="153"/>
+    <row r="154"/>
+    <row r="155"/>
+    <row r="156"/>
+    <row r="157"/>
+    <row r="158"/>
+    <row r="159"/>
+    <row r="160"/>
+    <row r="161"/>
+    <row r="162"/>
+    <row r="163"/>
+    <row r="164"/>
+    <row r="165"/>
+    <row r="166"/>
+    <row r="167"/>
+    <row r="168"/>
+    <row r="169"/>
+    <row r="170"/>
+    <row r="171"/>
+    <row r="172"/>
     <row r="173" ht="15" customHeight="1" s="227"/>
     <row r="174">
       <c r="F174" s="206" t="inlineStr">
@@ -6290,6 +6836,32 @@
         </is>
       </c>
     </row>
+    <row r="175"/>
+    <row r="176"/>
+    <row r="177"/>
+    <row r="178"/>
+    <row r="179"/>
+    <row r="180"/>
+    <row r="181"/>
+    <row r="182"/>
+    <row r="183"/>
+    <row r="184"/>
+    <row r="185"/>
+    <row r="186"/>
+    <row r="187"/>
+    <row r="188"/>
+    <row r="189"/>
+    <row r="190"/>
+    <row r="191"/>
+    <row r="192"/>
+    <row r="193"/>
+    <row r="194"/>
+    <row r="195"/>
+    <row r="196"/>
+    <row r="197"/>
+    <row r="198"/>
+    <row r="199"/>
+    <row r="200"/>
   </sheetData>
   <mergeCells count="22">
     <mergeCell ref="S12:T12"/>
@@ -6339,7 +6911,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y134"/>
+  <dimension ref="A1:Y200"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="19.625" customWidth="1" style="227" min="1" max="1"/>
@@ -6447,7 +7019,8 @@
       </c>
       <c r="H5" s="142" t="inlineStr">
         <is>
-          <t>L10</t>
+          <t>L10
+(DA=0)</t>
         </is>
       </c>
       <c r="I5" s="142" t="inlineStr">
@@ -6458,7 +7031,8 @@
       <c r="J5" s="143" t="n"/>
       <c r="K5" s="143" t="inlineStr">
         <is>
-          <t>LT1</t>
+          <t>LT1
+(N=903)</t>
         </is>
       </c>
       <c r="L5" s="143" t="n"/>
@@ -6520,14 +7094,14 @@
       <c r="G6" s="150" t="n">
         <v>0.046789</v>
       </c>
-      <c r="H6" s="150" t="n">
-        <v>0.09030000000000001</v>
+      <c r="H6" s="308" t="n">
+        <v>0</v>
       </c>
       <c r="I6" s="150" t="n">
         <v>0.049761</v>
       </c>
       <c r="J6" s="151" t="n"/>
-      <c r="K6" s="288" t="n">
+      <c r="K6" s="309" t="n">
         <v>0.09030000000000001</v>
       </c>
       <c r="L6" s="152" t="n"/>
@@ -6587,9 +7161,8 @@
         <f>((2.187*G10*G11)/(G12)^0.5)^0.467</f>
         <v/>
       </c>
-      <c r="H7" s="160">
-        <f>((2.187*H10*H11)/(H12)^0.5)^0.467</f>
-        <v/>
+      <c r="H7" s="310" t="n">
+        <v>0</v>
       </c>
       <c r="I7" s="160">
         <f>((2.187*I10*I11)/(I12)^0.5)^0.467</f>
@@ -6656,13 +7229,13 @@
         <v>0.642</v>
       </c>
       <c r="H8" s="169" t="n">
-        <v>0.95</v>
+        <v>0.9</v>
       </c>
       <c r="I8" s="169" t="n">
         <v>0.335</v>
       </c>
       <c r="J8" s="170" t="n"/>
-      <c r="K8" s="290" t="n">
+      <c r="K8" s="311" t="n">
         <v>0.95</v>
       </c>
       <c r="L8" s="170" t="n"/>
@@ -6756,7 +7329,7 @@
         <v>21.6</v>
       </c>
       <c r="H10" s="269" t="n">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="I10" s="269" t="n">
         <v>22.3</v>
@@ -6913,27 +7486,25 @@
       <c r="U12" s="139" t="n"/>
     </row>
     <row r="13" ht="15.75" customHeight="1" s="227">
-      <c r="O13" s="191" t="inlineStr">
+      <c r="O13" s="312" t="inlineStr">
         <is>
           <t>L10</t>
         </is>
       </c>
-      <c r="P13" s="192" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="Q13" s="193" t="n">
-        <v>903</v>
-      </c>
-      <c r="R13" s="193" t="n">
-        <v>857.85</v>
-      </c>
-      <c r="S13" s="194" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="T13" s="195" t="n">
-        <v>0.09030000000000001</v>
+      <c r="P13" s="312" t="inlineStr">
+        <is>
+          <t>(aucune – transfert; N déplacée → LT1)</t>
+        </is>
+      </c>
+      <c r="Q13" s="313" t="n">
+        <v>0</v>
+      </c>
+      <c r="R13" s="313" t="n">
+        <v>0</v>
+      </c>
+      <c r="S13" s="314" t="n"/>
+      <c r="T13" s="315" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="14" ht="15" customHeight="1" s="227">
@@ -6949,7 +7520,7 @@
       </c>
       <c r="P14" s="192" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>O (PAS de zone N)</t>
         </is>
       </c>
       <c r="Q14" s="193" t="n">
@@ -6971,26 +7542,26 @@
           <t>Jaune = saisie (depuis Reseau_pluvial_dimensionnement_v1). Vert = calculé.</t>
         </is>
       </c>
-      <c r="O15" t="inlineStr">
+      <c r="O15" s="304" t="inlineStr">
         <is>
           <t>LT1</t>
         </is>
       </c>
-      <c r="P15" t="inlineStr">
-        <is>
-          <t>N (toit → P11)</t>
-        </is>
-      </c>
-      <c r="Q15" t="n">
+      <c r="P15" s="304" t="inlineStr">
+        <is>
+          <t>N (toit → P11) — SEUL propriétaire</t>
+        </is>
+      </c>
+      <c r="Q15" s="304" t="n">
         <v>903</v>
       </c>
-      <c r="R15" t="n">
+      <c r="R15" s="304" t="n">
         <v>857.85</v>
       </c>
-      <c r="S15" t="n">
+      <c r="S15" s="304" t="n">
         <v>0.95</v>
       </c>
-      <c r="T15" t="n">
+      <c r="T15" s="304" t="n">
         <v>0.09030000000000001</v>
       </c>
     </row>
@@ -7059,6 +7630,11 @@
       </c>
     </row>
     <row r="18" ht="15.75" customHeight="1" s="227">
+      <c r="A18" s="316" t="inlineStr">
+        <is>
+          <t>CORRECTION: Zone N (903 m²) UNIQUEMENT sur LT1 (col K). L10 (col H) = transfert DA=0, te=0. Ne pas remettre 0.0903 sur H6 — double comptage avec K6 / Calcul E27.</t>
+        </is>
+      </c>
       <c r="O18" s="191" t="inlineStr">
         <is>
           <t>L06</t>
@@ -7906,30 +8482,30 @@
           <t>C zone</t>
         </is>
       </c>
-      <c r="O44" s="191" t="inlineStr">
+      <c r="O44" s="312" t="inlineStr">
         <is>
           <t>L10</t>
         </is>
       </c>
-      <c r="P44" s="191" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="Q44" s="193" t="n">
-        <v>903</v>
-      </c>
-      <c r="R44" s="193" t="n">
+      <c r="P44" s="312" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q44" s="313" t="n">
         <v>0</v>
       </c>
-      <c r="S44" s="193" t="n">
+      <c r="R44" s="313" t="n">
         <v>0</v>
       </c>
-      <c r="T44" s="193" t="n">
+      <c r="S44" s="313" t="n">
         <v>0</v>
       </c>
-      <c r="U44" s="193" t="n">
-        <v>903</v>
+      <c r="T44" s="313" t="n">
+        <v>0</v>
+      </c>
+      <c r="U44" s="313" t="n">
+        <v>0</v>
       </c>
       <c r="V44" s="193" t="n">
         <v>857.85</v>
@@ -7981,8 +8557,8 @@
       <c r="R45" s="197" t="n"/>
       <c r="S45" s="197" t="n"/>
       <c r="T45" s="197" t="n"/>
-      <c r="U45" s="198" t="n">
-        <v>903</v>
+      <c r="U45" s="317" t="n">
+        <v>0</v>
       </c>
       <c r="V45" s="198" t="n">
         <v>857.85</v>
@@ -8151,6 +8727,31 @@
       <c r="G49" s="224" t="n">
         <v>338.185</v>
       </c>
+      <c r="O49" s="304" t="inlineStr">
+        <is>
+          <t>LT1</t>
+        </is>
+      </c>
+      <c r="P49" s="304" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="Q49" s="304" t="n">
+        <v>903</v>
+      </c>
+      <c r="R49" s="304" t="n">
+        <v>0</v>
+      </c>
+      <c r="S49" s="304" t="n">
+        <v>0</v>
+      </c>
+      <c r="T49" s="304" t="n">
+        <v>0</v>
+      </c>
+      <c r="U49" s="304" t="n">
+        <v>903</v>
+      </c>
     </row>
     <row r="50" ht="15" customHeight="1" s="227">
       <c r="A50" s="224" t="inlineStr">
@@ -8158,11 +8759,24 @@
           <t>C = 338.185 / 442.35 = 0.7645 ≈ 0.765</t>
         </is>
       </c>
+      <c r="O50" t="inlineStr">
+        <is>
+          <t>LT1</t>
+        </is>
+      </c>
+      <c r="P50" t="inlineStr">
+        <is>
+          <t>SUM</t>
+        </is>
+      </c>
+      <c r="U50" s="304" t="n">
+        <v>903</v>
+      </c>
     </row>
     <row r="51" ht="15.75" customHeight="1" s="227">
-      <c r="O51" s="226" t="inlineStr">
-        <is>
-          <t>A = roof+pave+grass+other; A_eff = 0.95·roof + 0.90·pave + 0.25·grass + 0.60·other; C = ΣA_eff/ΣA</t>
+      <c r="O51" s="305" t="inlineStr">
+        <is>
+          <t>TOTAL zones: chaque m² une fois. Zone N=903 uniquement LT1. L10=0. L11=O seulement. Si N sur L10 ET LT1 → débit à P11 doublé.</t>
         </is>
       </c>
     </row>
@@ -8249,6 +8863,7 @@
         </is>
       </c>
     </row>
+    <row r="61"/>
     <row r="62" ht="15.75" customHeight="1" s="227">
       <c r="A62" s="228" t="inlineStr">
         <is>
@@ -8256,6 +8871,7 @@
         </is>
       </c>
     </row>
+    <row r="63"/>
     <row r="64" ht="15.75" customHeight="1" s="227">
       <c r="A64" s="4" t="inlineStr">
         <is>
@@ -8367,6 +8983,7 @@
         </is>
       </c>
     </row>
+    <row r="70"/>
     <row r="71" ht="15.75" customHeight="1" s="227">
       <c r="A71" s="4" t="inlineStr">
         <is>
@@ -8478,6 +9095,7 @@
         </is>
       </c>
     </row>
+    <row r="77"/>
     <row r="78" ht="15.75" customHeight="1" s="227">
       <c r="A78" s="4" t="inlineStr">
         <is>
@@ -8617,6 +9235,7 @@
         </is>
       </c>
     </row>
+    <row r="85"/>
     <row r="86" ht="15.75" customHeight="1" s="227">
       <c r="A86" s="4" t="inlineStr">
         <is>
@@ -8784,6 +9403,7 @@
         </is>
       </c>
     </row>
+    <row r="94"/>
     <row r="95" ht="15.75" customHeight="1" s="227">
       <c r="A95" s="4" t="inlineStr">
         <is>
@@ -8791,17 +9411,18 @@
         </is>
       </c>
     </row>
+    <row r="96"/>
     <row r="97" ht="15.75" customHeight="1" s="227">
-      <c r="A97" s="4" t="inlineStr">
-        <is>
-          <t>L10_P10_P11 → A = 903.00 m², C ≈ 0.950</t>
+      <c r="A97" s="318" t="inlineStr">
+        <is>
+          <t>L10_P10_P11 → A = 0 m² (transfert — zone N RETIRÉE, déplacée vers LT1/T1→P11)</t>
         </is>
       </c>
     </row>
     <row r="98" ht="15.75" customHeight="1" s="227">
       <c r="A98" t="inlineStr">
         <is>
-          <t>Zones N:</t>
+          <t>Zones: aucune (N n'est PLUS sur L10)</t>
         </is>
       </c>
     </row>
@@ -8850,11 +9471,11 @@
     <row r="100" ht="15.75" customHeight="1" s="227">
       <c r="A100" s="192" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>—</t>
         </is>
       </c>
       <c r="B100" s="193" t="n">
-        <v>903</v>
+        <v>0</v>
       </c>
       <c r="C100" s="193" t="n">
         <v>0</v>
@@ -8866,14 +9487,12 @@
         <v>0</v>
       </c>
       <c r="F100" s="193" t="n">
-        <v>903</v>
+        <v>0</v>
       </c>
       <c r="G100" s="193" t="n">
-        <v>857.85</v>
-      </c>
-      <c r="H100" s="194" t="n">
-        <v>0.95</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="H100" s="194" t="n"/>
     </row>
     <row r="101" ht="15.75" customHeight="1" s="227">
       <c r="A101" s="197" t="inlineStr">
@@ -8886,22 +9505,21 @@
       <c r="D101" s="197" t="n"/>
       <c r="E101" s="197" t="n"/>
       <c r="F101" s="197" t="n">
-        <v>903</v>
+        <v>0</v>
       </c>
       <c r="G101" s="197" t="n">
-        <v>857.85</v>
-      </c>
-      <c r="H101" s="197" t="n">
-        <v>0.95</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="H101" s="197" t="n"/>
     </row>
     <row r="102" ht="15.75" customHeight="1" s="227">
       <c r="A102" t="inlineStr">
         <is>
-          <t>C = 857.8500 / 903.00 = 0.9500</t>
-        </is>
-      </c>
-    </row>
+          <t>C = n/a (DA=0). Voir bloc LT1 ci-dessous pour zone N.</t>
+        </is>
+      </c>
+    </row>
+    <row r="103"/>
     <row r="104" ht="15.75" customHeight="1" s="227">
       <c r="A104" s="4" t="inlineStr">
         <is>
@@ -9013,6 +9631,8 @@
         </is>
       </c>
     </row>
+    <row r="110"/>
+    <row r="111"/>
     <row r="112" ht="15" customHeight="1" s="227">
       <c r="A112" s="224" t="inlineStr">
         <is>
@@ -9049,16 +9669,16 @@
       </c>
     </row>
     <row r="117" ht="15" customHeight="1" s="227">
-      <c r="A117" s="225" t="inlineStr">
-        <is>
-          <t>LT1_T1_P11 (toiture zone N): A=903 m², C=0.95; se raccorde à P11. Radiers: MIN aux confluences.</t>
+      <c r="A117" s="319" t="inlineStr">
+        <is>
+          <t>LT1_T1_P11 (toiture zone N): A=903 m², C=0.95 — SEUL propriétaire de N. Colonne K du tableau (K6=0.0903). Ne jamais recopier N sur L10/H6.</t>
         </is>
       </c>
     </row>
     <row r="118" ht="15" customHeight="1" s="227">
       <c r="A118" s="200" t="inlineStr">
         <is>
-          <t>P10→P11: DA locale=0 (toit déplacé vers T1). Fusion H à P11 = H(P10)+H(T1)+DA(P11).</t>
+          <t>P10→P11: DA locale=0 dans Calcul_reseau E26 ET dans Temps H6/RESUME. Fusion à P11 = H(P10)+H(T1)+DA(P11). Radiers inchangés (dépendent de L,s).</t>
         </is>
       </c>
       <c r="B118" s="200" t="inlineStr">
@@ -9188,18 +9808,31 @@
     <row r="125" ht="15" customHeight="1" s="227">
       <c r="A125" s="224" t="inlineStr">
         <is>
-          <t>L10</t>
-        </is>
-      </c>
-      <c r="B125" s="224" t="n">
+          <t>L10 (DA=0)</t>
+        </is>
+      </c>
+      <c r="B125" s="320" t="n">
+        <v>0</v>
+      </c>
+      <c r="C125" s="224" t="n">
+        <v>0</v>
+      </c>
+      <c r="D125" s="224" t="inlineStr">
+        <is>
+          <t>0 m (transfert)</t>
+        </is>
+      </c>
+      <c r="F125" s="304" t="inlineStr">
+        <is>
+          <t>LT1</t>
+        </is>
+      </c>
+      <c r="G125" s="304" t="n">
         <v>903</v>
       </c>
-      <c r="C125" s="224" t="n">
-        <v>30.05</v>
-      </c>
-      <c r="D125" s="224" t="inlineStr">
-        <is>
-          <t>30.0 m</t>
+      <c r="H125" t="inlineStr">
+        <is>
+          <t>√A≈30 → K10=30 m (toit)</t>
         </is>
       </c>
     </row>
@@ -9277,6 +9910,72 @@
         </is>
       </c>
     </row>
+    <row r="135"/>
+    <row r="136"/>
+    <row r="137"/>
+    <row r="138"/>
+    <row r="139"/>
+    <row r="140"/>
+    <row r="141"/>
+    <row r="142"/>
+    <row r="143"/>
+    <row r="144"/>
+    <row r="145"/>
+    <row r="146"/>
+    <row r="147"/>
+    <row r="148"/>
+    <row r="149"/>
+    <row r="150"/>
+    <row r="151"/>
+    <row r="152"/>
+    <row r="153"/>
+    <row r="154"/>
+    <row r="155"/>
+    <row r="156"/>
+    <row r="157"/>
+    <row r="158"/>
+    <row r="159"/>
+    <row r="160"/>
+    <row r="161"/>
+    <row r="162"/>
+    <row r="163"/>
+    <row r="164"/>
+    <row r="165"/>
+    <row r="166"/>
+    <row r="167"/>
+    <row r="168"/>
+    <row r="169"/>
+    <row r="170"/>
+    <row r="171"/>
+    <row r="172"/>
+    <row r="173"/>
+    <row r="174"/>
+    <row r="175"/>
+    <row r="176"/>
+    <row r="177"/>
+    <row r="178"/>
+    <row r="179"/>
+    <row r="180"/>
+    <row r="181"/>
+    <row r="182"/>
+    <row r="183"/>
+    <row r="184"/>
+    <row r="185"/>
+    <row r="186"/>
+    <row r="187"/>
+    <row r="188"/>
+    <row r="189"/>
+    <row r="190"/>
+    <row r="191"/>
+    <row r="192"/>
+    <row r="193"/>
+    <row r="194"/>
+    <row r="195"/>
+    <row r="196"/>
+    <row r="197"/>
+    <row r="198"/>
+    <row r="199"/>
+    <row r="200"/>
   </sheetData>
   <mergeCells count="38">
     <mergeCell ref="A116:D116"/>

</xml_diff>